<commit_message>
T108: làm mới báo cáo hệ thống Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,17 +80,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00854D0E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -147,12 +141,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-        <bgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
@@ -184,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -243,9 +231,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -844,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>110 việc (T01 - T108)</t>
+          <t>112 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>91 việc (82.7%)</t>
+          <t>92 việc (82.1%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -878,7 +863,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>1 việc</t>
+          <t>0 việc</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -895,7 +880,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>18 việc</t>
+          <t>20 việc</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -21026,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21087,29 +21072,25 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T109</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, báo cáo tài chính riêng TT58 (doanh nghiệp siêu nhỏ) theo bộ biểu mẫu `D:\IACC-CLOUD\TT58`: chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); cột, dòng in sẵn đúng từng mẫu S1–S4d; thêm S2a, S3a; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu TT58</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr"/>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Sửa file chung `ReportScreen.tsx` (tiêu đề cột 2 tầng), `app.css`; thêm `mau-in.ts`, `so-bo-sung.ts`, `danh-sach.ts`, `BaoCaoTaiChinh.tsx`, `session.tsx`, `HeThong.tsx`, `registry.ts`, `plan.ts`</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21119,20 +21100,16 @@
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E3" s="26" t="inlineStr">
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr"/>
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21141,7 +21118,7 @@
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
         </is>
       </c>
     </row>
@@ -21151,12 +21128,12 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T101</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
@@ -21164,7 +21141,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21173,7 +21150,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T25</t>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
         </is>
       </c>
     </row>
@@ -21183,27 +21160,31 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E5" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Tách từ T25</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n">
@@ -21211,27 +21192,27 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="26" t="inlineStr">
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr"/>
       <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr">
-        <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
-        </is>
-      </c>
+      <c r="H6" s="13" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
@@ -21239,16 +21220,16 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21257,7 +21238,7 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Chỉ máy Trum chạy được script</t>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
         </is>
       </c>
     </row>
@@ -21267,16 +21248,16 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21285,7 +21266,7 @@
       <c r="G8" s="13" t="inlineStr"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có</t>
+          <t>Chỉ máy Trum chạy được script</t>
         </is>
       </c>
     </row>
@@ -21295,16 +21276,16 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21313,7 +21294,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
         </is>
       </c>
     </row>
@@ -21323,23 +21304,27 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
@@ -21347,27 +21332,23 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr"/>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
-        </is>
-      </c>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -21375,16 +21356,16 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21393,7 +21374,7 @@
       <c r="G12" s="13" t="inlineStr"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
         </is>
       </c>
     </row>
@@ -21403,16 +21384,16 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21421,7 +21402,7 @@
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
         </is>
       </c>
     </row>
@@ -21431,16 +21412,16 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21449,7 +21430,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -21459,16 +21440,16 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="26" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21477,7 +21458,7 @@
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -21487,16 +21468,16 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="26" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21505,7 +21486,7 @@
       <c r="G16" s="13" t="inlineStr"/>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -21515,16 +21496,16 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="26" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21533,7 +21514,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -21543,16 +21524,16 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="26" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21561,7 +21542,7 @@
       <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -21571,16 +21552,16 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21589,7 +21570,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+          <t>Chưa có file logo iPOS</t>
         </is>
       </c>
     </row>
@@ -21599,16 +21580,16 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21617,7 +21598,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
         </is>
       </c>
     </row>
@@ -21627,35 +21608,27 @@
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>dinhlanphuongipacc</t>
-        </is>
-      </c>
-      <c r="E21" s="27" t="inlineStr">
-        <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr"/>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr"/>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n">
@@ -21663,20 +21636,20 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21688,7 +21661,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr"/>
@@ -21699,20 +21672,20 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E23" s="27" t="inlineStr">
+          <t>dinhlanphuongipacc</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21724,7 +21697,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
@@ -21735,12 +21708,12 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -21748,7 +21721,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21771,12 +21744,12 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -21784,7 +21757,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E25" s="27" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21807,12 +21780,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21820,7 +21793,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E26" s="27" t="inlineStr">
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21843,12 +21816,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21856,7 +21829,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E27" s="27" t="inlineStr">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21868,7 +21841,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21879,12 +21852,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21892,7 +21865,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21904,7 +21877,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21915,12 +21888,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21928,7 +21901,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21951,20 +21924,20 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E30" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21976,7 +21949,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21987,12 +21960,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -22000,7 +21973,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E31" s="27" t="inlineStr">
+      <c r="E31" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22012,7 +21985,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -22023,20 +21996,20 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22048,7 +22021,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22059,12 +22032,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22072,7 +22045,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E33" s="27" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22095,12 +22068,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22108,7 +22081,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E34" s="27" t="inlineStr">
+      <c r="E34" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22120,7 +22093,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22131,12 +22104,12 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22144,7 +22117,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E35" s="27" t="inlineStr">
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22156,7 +22129,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22167,12 +22140,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22180,7 +22153,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E36" s="27" t="inlineStr">
+      <c r="E36" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22203,12 +22176,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22216,7 +22189,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E37" s="27" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22228,7 +22201,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22239,12 +22212,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22252,7 +22225,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E38" s="27" t="inlineStr">
+      <c r="E38" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22264,7 +22237,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22275,20 +22248,20 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E39" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22300,7 +22273,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22311,20 +22284,20 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E40" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22336,7 +22309,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22347,12 +22320,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22360,7 +22333,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E41" s="27" t="inlineStr">
+      <c r="E41" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22372,7 +22345,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22383,12 +22356,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22396,7 +22369,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E42" s="27" t="inlineStr">
+      <c r="E42" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22419,20 +22392,20 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E43" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22444,7 +22417,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22455,20 +22428,20 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E44" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22480,7 +22453,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22491,12 +22464,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22504,7 +22477,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E45" s="27" t="inlineStr">
+      <c r="E45" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22516,7 +22489,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22527,12 +22500,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22540,7 +22513,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E46" s="27" t="inlineStr">
+      <c r="E46" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22552,7 +22525,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22563,12 +22536,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22576,7 +22549,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E47" s="27" t="inlineStr">
+      <c r="E47" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22588,7 +22561,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22599,12 +22572,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22612,7 +22585,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E48" s="27" t="inlineStr">
+      <c r="E48" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22635,20 +22608,20 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E49" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22660,7 +22633,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22671,20 +22644,20 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E50" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E50" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22696,7 +22669,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22707,12 +22680,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22720,7 +22693,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E51" s="27" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22743,12 +22716,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22756,7 +22729,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E52" s="27" t="inlineStr">
+      <c r="E52" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22779,32 +22752,32 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E53" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22815,32 +22788,32 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E54" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F54" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22851,12 +22824,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22864,7 +22837,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E55" s="27" t="inlineStr">
+      <c r="E55" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22876,7 +22849,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22887,12 +22860,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22900,7 +22873,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E56" s="27" t="inlineStr">
+      <c r="E56" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22912,7 +22885,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22923,20 +22896,20 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E57" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22948,7 +22921,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22959,20 +22932,20 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E58" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22984,7 +22957,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22995,12 +22968,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -23008,7 +22981,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E59" s="27" t="inlineStr">
+      <c r="E59" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23031,12 +23004,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23044,7 +23017,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E60" s="27" t="inlineStr">
+      <c r="E60" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23067,12 +23040,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23080,7 +23053,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E61" s="27" t="inlineStr">
+      <c r="E61" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23103,12 +23076,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23116,7 +23089,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E62" s="27" t="inlineStr">
+      <c r="E62" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23139,12 +23112,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23152,7 +23125,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E63" s="27" t="inlineStr">
+      <c r="E63" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23175,12 +23148,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23188,7 +23161,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E64" s="27" t="inlineStr">
+      <c r="E64" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23211,20 +23184,20 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E65" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23236,7 +23209,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23247,20 +23220,20 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E66" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E66" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23272,7 +23245,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23283,12 +23256,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23296,7 +23269,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E67" s="27" t="inlineStr">
+      <c r="E67" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23319,12 +23292,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23332,7 +23305,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E68" s="27" t="inlineStr">
+      <c r="E68" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23355,12 +23328,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23368,7 +23341,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E69" s="27" t="inlineStr">
+      <c r="E69" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23391,20 +23364,20 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E70" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E70" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23416,7 +23389,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23427,20 +23400,20 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E71" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E71" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23452,7 +23425,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23463,20 +23436,20 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E72" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E72" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23488,7 +23461,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23499,20 +23472,20 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E73" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23524,7 +23497,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23535,12 +23508,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23548,7 +23521,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E74" s="27" t="inlineStr">
+      <c r="E74" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23560,7 +23533,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23571,12 +23544,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23584,7 +23557,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E75" s="27" t="inlineStr">
+      <c r="E75" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23607,12 +23580,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23620,7 +23593,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E76" s="27" t="inlineStr">
+      <c r="E76" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23632,7 +23605,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23643,12 +23616,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23656,7 +23629,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E77" s="27" t="inlineStr">
+      <c r="E77" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23668,7 +23641,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23679,20 +23652,20 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E78" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E78" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23704,7 +23677,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23715,20 +23688,20 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E79" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E79" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23740,7 +23713,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23751,20 +23724,20 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E80" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E80" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23776,7 +23749,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23787,20 +23760,20 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E81" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23812,7 +23785,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23823,20 +23796,20 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E82" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E82" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23848,7 +23821,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23859,20 +23832,20 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E83" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E83" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23884,7 +23857,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23895,12 +23868,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23908,7 +23881,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E84" s="27" t="inlineStr">
+      <c r="E84" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23920,7 +23893,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23931,12 +23904,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23944,7 +23917,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E85" s="27" t="inlineStr">
+      <c r="E85" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23956,7 +23929,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23967,12 +23940,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23980,19 +23953,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E86" s="27" t="inlineStr">
+      <c r="E86" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -24003,12 +23976,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -24016,19 +23989,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E87" s="27" t="inlineStr">
+      <c r="E87" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24039,12 +24012,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24052,7 +24025,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E88" s="27" t="inlineStr">
+      <c r="E88" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24064,7 +24037,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24075,20 +24048,20 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E89" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E89" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24100,7 +24073,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24111,12 +24084,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24124,7 +24097,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E90" s="27" t="inlineStr">
+      <c r="E90" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24136,7 +24109,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24147,20 +24120,20 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E91" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E91" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24172,7 +24145,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24183,20 +24156,20 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E92" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E92" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24208,7 +24181,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24219,20 +24192,20 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E93" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E93" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24244,7 +24217,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24255,20 +24228,20 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E94" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E94" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24280,7 +24253,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24291,20 +24264,20 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E95" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E95" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24316,7 +24289,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24327,12 +24300,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24340,7 +24313,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E96" s="27" t="inlineStr">
+      <c r="E96" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24352,7 +24325,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24363,12 +24336,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24376,7 +24349,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E97" s="27" t="inlineStr">
+      <c r="E97" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24388,7 +24361,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24399,12 +24372,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24412,7 +24385,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E98" s="27" t="inlineStr">
+      <c r="E98" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24424,7 +24397,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24435,12 +24408,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24448,7 +24421,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E99" s="27" t="inlineStr">
+      <c r="E99" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24460,7 +24433,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24471,12 +24444,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24484,7 +24457,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E100" s="27" t="inlineStr">
+      <c r="E100" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24496,7 +24469,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24507,12 +24480,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24520,7 +24493,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E101" s="27" t="inlineStr">
+      <c r="E101" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24532,7 +24505,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24543,12 +24516,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24556,7 +24529,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E102" s="27" t="inlineStr">
+      <c r="E102" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24568,7 +24541,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24579,12 +24552,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24592,7 +24565,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E103" s="27" t="inlineStr">
+      <c r="E103" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24604,7 +24577,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24615,12 +24588,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24628,19 +24601,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E104" s="27" t="inlineStr">
+      <c r="E104" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24651,12 +24624,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24664,19 +24637,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E105" s="27" t="inlineStr">
+      <c r="E105" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24687,12 +24660,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24700,7 +24673,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E106" s="27" t="inlineStr">
+      <c r="E106" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24712,7 +24685,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24723,12 +24696,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24736,7 +24709,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E107" s="27" t="inlineStr">
+      <c r="E107" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24748,7 +24721,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24759,12 +24732,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24772,19 +24745,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E108" s="27" t="inlineStr">
+      <c r="E108" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24795,12 +24768,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24808,19 +24781,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E109" s="27" t="inlineStr">
+      <c r="E109" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24831,12 +24804,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24844,7 +24817,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E110" s="27" t="inlineStr">
+      <c r="E110" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24867,38 +24840,110 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D111" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E111" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F111" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="23" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C112" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D112" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E112" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G112" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H112" s="13" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="16" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C111" s="5" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E111" s="27" t="inlineStr">
+      <c r="E113" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F111" s="16" t="inlineStr">
+      <c r="F113" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G111" s="5" t="inlineStr">
+      <c r="G113" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H111" s="5" t="inlineStr"/>
+      <c r="H113" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H111"/>
+  <autoFilter ref="A1:H113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T113: thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,11 +80,17 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00854D0E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -141,6 +147,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+        <bgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
@@ -172,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -231,6 +243,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -829,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>112 việc (T01 - T108)</t>
+          <t>115 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>92 việc (82.1%)</t>
+          <t>93 việc (80.9%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -863,7 +878,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>0 việc</t>
+          <t>2 việc</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -21011,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21072,25 +21087,29 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T109</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr"/>
+          <t>Báo cáo: đưa ô chọn khoảng ngày và nút Xem báo cáo sang cột Bộ lọc bên trái; sửa cột hẹp làm vỡ tiêu đề (cột Tỷ lệ (%) khấu hao ở Sổ TSCĐ S4b-DNSN), rà mọi báo cáo</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
+          <t>Sửa `src/ui/generic/ReportScreen.tsx`, `src/ui/bao-cao/chiaCot.ts`, `ToGiay.tsx`, `app.css`</t>
         </is>
       </c>
     </row>
@@ -21100,25 +21119,29 @@
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>T110</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr"/>
+          <t>Thiết kế lại màn Thiết kế mẫu in và toàn bộ mẫu in phiếu chứng từ: đủ thông tin theo thông tư, bố cục gọn, đẹp</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+          <t>Sửa `src/modules/tien-ich/ThietKeMauIn.tsx`, `src/ui/bao-cao/InChungTu.tsx`, `mau-in.ts`, `duLieuIn.ts`, `app.css`</t>
         </is>
       </c>
     </row>
@@ -21128,20 +21151,16 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T109</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E4" s="24" t="inlineStr">
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr"/>
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21150,7 +21169,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21160,20 +21179,16 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr"/>
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21182,7 +21197,7 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T25</t>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
         </is>
       </c>
     </row>
@@ -21192,27 +21207,31 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T101</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr"/>
       <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
@@ -21220,16 +21239,20 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="24" t="inlineStr">
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21238,7 +21261,7 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+          <t>Tách từ T25</t>
         </is>
       </c>
     </row>
@@ -21248,27 +21271,27 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="24" t="inlineStr">
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr"/>
       <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="13" t="inlineStr">
-        <is>
-          <t>Chỉ máy Trum chạy được script</t>
-        </is>
-      </c>
+      <c r="H8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
@@ -21276,16 +21299,16 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21294,7 +21317,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
         </is>
       </c>
     </row>
@@ -21304,16 +21327,16 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21322,7 +21345,7 @@
       <c r="G10" s="13" t="inlineStr"/>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
+          <t>Chỉ máy Trum chạy được script</t>
         </is>
       </c>
     </row>
@@ -21332,23 +21355,27 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr"/>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -21356,16 +21383,16 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21374,7 +21401,7 @@
       <c r="G12" s="13" t="inlineStr"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
         </is>
       </c>
     </row>
@@ -21384,27 +21411,23 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
-        </is>
-      </c>
+      <c r="H13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
@@ -21412,16 +21435,16 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21430,7 +21453,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
         </is>
       </c>
     </row>
@@ -21440,16 +21463,16 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21458,7 +21481,7 @@
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
         </is>
       </c>
     </row>
@@ -21468,16 +21491,16 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21486,7 +21509,7 @@
       <c r="G16" s="13" t="inlineStr"/>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -21496,16 +21519,16 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21514,7 +21537,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -21524,16 +21547,16 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21542,7 +21565,7 @@
       <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -21552,16 +21575,16 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21570,7 +21593,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -21580,16 +21603,16 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21598,7 +21621,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -21608,16 +21631,16 @@
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21626,7 +21649,7 @@
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+          <t>Chưa có file logo iPOS</t>
         </is>
       </c>
     </row>
@@ -21636,35 +21659,27 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr"/>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
-        </is>
-      </c>
-      <c r="H22" s="13" t="inlineStr"/>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr"/>
+      <c r="G22" s="13" t="inlineStr"/>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n">
@@ -21672,35 +21687,27 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>dinhlanphuongipacc</t>
-        </is>
-      </c>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr"/>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr"/>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="n">
@@ -21708,20 +21715,20 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E24" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21733,7 +21740,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -21744,20 +21751,20 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E25" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21769,7 +21776,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21780,20 +21787,20 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E26" s="26" t="inlineStr">
+          <t>dinhlanphuongipacc</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21805,7 +21812,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21816,12 +21823,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21829,7 +21836,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E27" s="26" t="inlineStr">
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21852,12 +21859,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21865,7 +21872,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E28" s="26" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21888,12 +21895,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21901,7 +21908,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E29" s="26" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21913,7 +21920,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21924,12 +21931,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21937,7 +21944,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E30" s="26" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21949,7 +21956,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21960,12 +21967,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21973,7 +21980,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E31" s="26" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21985,7 +21992,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21996,20 +22003,20 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E32" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22021,7 +22028,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22032,12 +22039,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22045,7 +22052,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E33" s="26" t="inlineStr">
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22057,7 +22064,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22068,12 +22075,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22081,7 +22088,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E34" s="26" t="inlineStr">
+      <c r="E34" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22093,7 +22100,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22104,20 +22111,20 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E35" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22129,7 +22136,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22140,12 +22147,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22153,7 +22160,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E36" s="26" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22165,7 +22172,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22176,12 +22183,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22189,7 +22196,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E37" s="26" t="inlineStr">
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22201,7 +22208,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22212,12 +22219,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22225,7 +22232,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E38" s="26" t="inlineStr">
+      <c r="E38" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22237,7 +22244,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22248,12 +22255,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22261,7 +22268,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E39" s="26" t="inlineStr">
+      <c r="E39" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22273,7 +22280,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22284,12 +22291,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22297,7 +22304,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E40" s="26" t="inlineStr">
+      <c r="E40" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22309,7 +22316,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22320,20 +22327,20 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E41" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22345,7 +22352,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22356,20 +22363,20 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E42" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E42" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22381,7 +22388,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22392,20 +22399,20 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E43" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22417,7 +22424,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22428,12 +22435,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22441,7 +22448,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E44" s="26" t="inlineStr">
+      <c r="E44" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22453,7 +22460,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22464,20 +22471,20 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E45" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22489,7 +22496,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22500,20 +22507,20 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E46" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22525,7 +22532,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22536,20 +22543,20 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E47" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E47" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22561,7 +22568,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22572,12 +22579,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22585,7 +22592,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E48" s="26" t="inlineStr">
+      <c r="E48" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22597,7 +22604,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22608,12 +22615,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22621,7 +22628,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E49" s="26" t="inlineStr">
+      <c r="E49" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22633,7 +22640,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22644,12 +22651,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22657,7 +22664,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E50" s="26" t="inlineStr">
+      <c r="E50" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22669,7 +22676,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22680,20 +22687,20 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22705,7 +22712,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22716,20 +22723,20 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E52" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22741,7 +22748,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22752,20 +22759,20 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E53" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22777,7 +22784,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22788,12 +22795,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22801,7 +22808,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E54" s="26" t="inlineStr">
+      <c r="E54" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22824,32 +22831,32 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E55" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22860,32 +22867,32 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E56" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22896,32 +22903,32 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E57" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22932,12 +22939,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22945,7 +22952,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E58" s="26" t="inlineStr">
+      <c r="E58" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22957,7 +22964,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22968,20 +22975,20 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E59" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E59" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22993,7 +23000,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -23004,20 +23011,20 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E60" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E60" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23029,7 +23036,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23040,20 +23047,20 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E61" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23065,7 +23072,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23076,12 +23083,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23089,7 +23096,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E62" s="26" t="inlineStr">
+      <c r="E62" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23112,12 +23119,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23125,7 +23132,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E63" s="26" t="inlineStr">
+      <c r="E63" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23148,12 +23155,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23161,7 +23168,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E64" s="26" t="inlineStr">
+      <c r="E64" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23184,12 +23191,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23197,7 +23204,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E65" s="26" t="inlineStr">
+      <c r="E65" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23220,12 +23227,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23233,7 +23240,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E66" s="26" t="inlineStr">
+      <c r="E66" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23256,20 +23263,20 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E67" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E67" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23281,7 +23288,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23292,20 +23299,20 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E68" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23317,7 +23324,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23328,20 +23335,20 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E69" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23353,7 +23360,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23364,12 +23371,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23377,7 +23384,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E70" s="26" t="inlineStr">
+      <c r="E70" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23400,12 +23407,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23413,7 +23420,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E71" s="26" t="inlineStr">
+      <c r="E71" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23436,20 +23443,20 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E72" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E72" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23461,7 +23468,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23472,20 +23479,20 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E73" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E73" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23497,7 +23504,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23508,12 +23515,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23521,7 +23528,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E74" s="26" t="inlineStr">
+      <c r="E74" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23533,7 +23540,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23544,20 +23551,20 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E75" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E75" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23569,7 +23576,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23580,20 +23587,20 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E76" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E76" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23605,7 +23612,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23616,12 +23623,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23629,7 +23636,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E77" s="26" t="inlineStr">
+      <c r="E77" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23641,7 +23648,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23652,12 +23659,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23665,7 +23672,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E78" s="26" t="inlineStr">
+      <c r="E78" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23677,7 +23684,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23688,12 +23695,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23701,7 +23708,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E79" s="26" t="inlineStr">
+      <c r="E79" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23713,7 +23720,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23724,20 +23731,20 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E80" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E80" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23749,7 +23756,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23760,20 +23767,20 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E81" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E81" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23785,7 +23792,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23796,12 +23803,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23809,7 +23816,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E82" s="26" t="inlineStr">
+      <c r="E82" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23821,7 +23828,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23832,20 +23839,20 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E83" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E83" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23857,7 +23864,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23868,12 +23875,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23881,7 +23888,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E84" s="26" t="inlineStr">
+      <c r="E84" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23893,7 +23900,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23904,20 +23911,20 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E85" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E85" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23929,7 +23936,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23940,20 +23947,20 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E86" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E86" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23965,7 +23972,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23976,12 +23983,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23989,7 +23996,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E87" s="26" t="inlineStr">
+      <c r="E87" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24001,7 +24008,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24012,12 +24019,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24025,19 +24032,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E88" s="26" t="inlineStr">
+      <c r="E88" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24048,12 +24055,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24061,19 +24068,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E89" s="26" t="inlineStr">
+      <c r="E89" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24084,12 +24091,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24097,19 +24104,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E90" s="26" t="inlineStr">
+      <c r="E90" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24120,20 +24127,20 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E91" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E91" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24145,7 +24152,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24156,12 +24163,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24169,7 +24176,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E92" s="26" t="inlineStr">
+      <c r="E92" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24181,7 +24188,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24192,12 +24199,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24205,7 +24212,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E93" s="26" t="inlineStr">
+      <c r="E93" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24217,7 +24224,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24228,12 +24235,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24241,7 +24248,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E94" s="26" t="inlineStr">
+      <c r="E94" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24253,7 +24260,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24264,20 +24271,20 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E95" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E95" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24289,7 +24296,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24300,12 +24307,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24313,7 +24320,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E96" s="26" t="inlineStr">
+      <c r="E96" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24325,7 +24332,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24336,20 +24343,20 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E97" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E97" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24361,7 +24368,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24372,20 +24379,20 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E98" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E98" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24397,7 +24404,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24408,12 +24415,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24421,7 +24428,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E99" s="26" t="inlineStr">
+      <c r="E99" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24433,7 +24440,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24444,12 +24451,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24457,7 +24464,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E100" s="26" t="inlineStr">
+      <c r="E100" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24469,7 +24476,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24480,12 +24487,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24493,7 +24500,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E101" s="26" t="inlineStr">
+      <c r="E101" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24505,7 +24512,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24516,12 +24523,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24529,7 +24536,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E102" s="26" t="inlineStr">
+      <c r="E102" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24541,7 +24548,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24552,12 +24559,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24565,7 +24572,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E103" s="26" t="inlineStr">
+      <c r="E103" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24577,7 +24584,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24588,12 +24595,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24601,7 +24608,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E104" s="26" t="inlineStr">
+      <c r="E104" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24613,7 +24620,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24624,12 +24631,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24637,7 +24644,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E105" s="26" t="inlineStr">
+      <c r="E105" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24649,7 +24656,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24660,12 +24667,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24673,19 +24680,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E106" s="26" t="inlineStr">
+      <c r="E106" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24696,12 +24703,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24709,19 +24716,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E107" s="26" t="inlineStr">
+      <c r="E107" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24732,12 +24739,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24745,19 +24752,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E108" s="26" t="inlineStr">
+      <c r="E108" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24768,12 +24775,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24781,7 +24788,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E109" s="26" t="inlineStr">
+      <c r="E109" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24793,7 +24800,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24804,12 +24811,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24817,19 +24824,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E110" s="26" t="inlineStr">
+      <c r="E110" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24840,12 +24847,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24853,19 +24860,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E111" s="26" t="inlineStr">
+      <c r="E111" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24876,12 +24883,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24889,19 +24896,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E112" s="26" t="inlineStr">
+      <c r="E112" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24912,38 +24919,146 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+        </is>
+      </c>
+      <c r="D113" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E113" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F113" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="23" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C114" s="13" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D114" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E114" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G114" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H114" s="13" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="16" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="25" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D115" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E115" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F115" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H115" s="5" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="23" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
+      <c r="C116" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D116" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E113" s="26" t="inlineStr">
+      <c r="E116" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F113" s="16" t="inlineStr">
+      <c r="F116" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G113" s="5" t="inlineStr">
+      <c r="G116" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H113" s="5" t="inlineStr"/>
+      <c r="H116" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H113"/>
+  <autoFilter ref="A1:H116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T111, T112: bộ lọc báo cáo bên trái, cột không vỡ tiêu đề, thiết kế lại mẫu in
- T111: ô Khoảng ngày và nút Xem báo cáo vào cột Bộ lọc; chiaCot thêm loại cột tỷ lệ, độ rộng tối thiểu theo từ dài nhất tiêu đề.
- T112: màn Thiết kế mẫu in ba vùng; khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu.
- CSS của hai việc đã nằm trong commit T113 (phiên khác chung thư mục).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$117</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,17 +80,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00854D0E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -147,12 +141,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-        <bgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
@@ -184,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -243,9 +231,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -844,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>115 việc (T01 - T108)</t>
+          <t>116 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>93 việc (80.9%)</t>
+          <t>95 việc (81.9%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -878,7 +863,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>2 việc</t>
+          <t>0 việc</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -895,7 +880,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>20 việc</t>
+          <t>21 việc</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -21026,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21087,29 +21072,25 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: đưa ô chọn khoảng ngày và nút Xem báo cáo sang cột Bộ lọc bên trái; sửa cột hẹp làm vỡ tiêu đề (cột Tỷ lệ (%) khấu hao ở Sổ TSCĐ S4b-DNSN), rà mọi báo cáo</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr"/>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Sửa `src/ui/generic/ReportScreen.tsx`, `src/ui/bao-cao/chiaCot.ts`, `ToGiay.tsx`, `app.css`</t>
+          <t>Phát hiện khi làm T112</t>
         </is>
       </c>
     </row>
@@ -21119,29 +21100,25 @@
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T109</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn Thiết kế mẫu in và toàn bộ mẫu in phiếu chứng từ: đủ thông tin theo thông tư, bố cục gọn, đẹp</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr"/>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Sửa `src/modules/tien-ich/ThietKeMauIn.tsx`, `src/ui/bao-cao/InChungTu.tsx`, `mau-in.ts`, `duLieuIn.ts`, `app.css`</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21151,16 +21128,16 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>T109</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21169,7 +21146,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
         </is>
       </c>
     </row>
@@ -21179,16 +21156,20 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>T110</t>
+          <t>T101</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="26" t="inlineStr">
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21197,7 +21178,7 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
         </is>
       </c>
     </row>
@@ -21207,12 +21188,12 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -21220,7 +21201,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21229,7 +21210,7 @@
       <c r="G6" s="13" t="inlineStr"/>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+          <t>Tách từ T25</t>
         </is>
       </c>
     </row>
@@ -21239,31 +21220,27 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E7" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Tách từ T25</t>
-        </is>
-      </c>
+      <c r="H7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -21271,27 +21248,27 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E8" s="26" t="inlineStr">
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr"/>
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr"/>
       <c r="G8" s="13" t="inlineStr"/>
-      <c r="H8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
@@ -21299,16 +21276,16 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr"/>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21317,7 +21294,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+          <t>Chỉ máy Trum chạy được script</t>
         </is>
       </c>
     </row>
@@ -21327,16 +21304,16 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21345,7 +21322,7 @@
       <c r="G10" s="13" t="inlineStr"/>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Chỉ máy Trum chạy được script</t>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
         </is>
       </c>
     </row>
@@ -21355,16 +21332,16 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr"/>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21373,7 +21350,7 @@
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
         </is>
       </c>
     </row>
@@ -21383,27 +21360,23 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="13" t="inlineStr"/>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
-        </is>
-      </c>
+      <c r="H12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
@@ -21411,23 +21384,27 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
@@ -21435,16 +21412,16 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21453,7 +21430,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
         </is>
       </c>
     </row>
@@ -21463,16 +21440,16 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="26" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21481,7 +21458,7 @@
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -21491,16 +21468,16 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="26" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21509,7 +21486,7 @@
       <c r="G16" s="13" t="inlineStr"/>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -21519,16 +21496,16 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="26" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21537,7 +21514,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -21547,16 +21524,16 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="26" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21565,7 +21542,7 @@
       <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -21575,16 +21552,16 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="26" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21593,7 +21570,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -21603,16 +21580,16 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="26" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21621,7 +21598,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>Chưa có file logo iPOS</t>
         </is>
       </c>
     </row>
@@ -21631,16 +21608,16 @@
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="26" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21649,7 +21626,7 @@
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
         </is>
       </c>
     </row>
@@ -21659,16 +21636,16 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="26" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21677,7 +21654,7 @@
       <c r="G22" s="13" t="inlineStr"/>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
         </is>
       </c>
     </row>
@@ -21687,27 +21664,35 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr"/>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>Chờ</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr"/>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
-        </is>
-      </c>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="n">
@@ -21715,12 +21700,12 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -21728,7 +21713,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21740,7 +21725,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -21751,12 +21736,12 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -21764,7 +21749,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E25" s="27" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21776,7 +21761,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21787,20 +21772,20 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
-        </is>
-      </c>
-      <c r="E26" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21812,7 +21797,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21823,20 +21808,20 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E27" s="27" t="inlineStr">
+          <t>dinhlanphuongipacc</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21848,7 +21833,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21859,12 +21844,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21872,7 +21857,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21895,12 +21880,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21908,7 +21893,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21931,12 +21916,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21944,7 +21929,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E30" s="27" t="inlineStr">
+      <c r="E30" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21967,12 +21952,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21980,7 +21965,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E31" s="27" t="inlineStr">
+      <c r="E31" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22003,12 +21988,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22016,7 +22001,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E32" s="27" t="inlineStr">
+      <c r="E32" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22028,7 +22013,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22039,12 +22024,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22052,7 +22037,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E33" s="27" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22075,12 +22060,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22088,7 +22073,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E34" s="27" t="inlineStr">
+      <c r="E34" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22111,20 +22096,20 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E35" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22136,7 +22121,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22147,20 +22132,20 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E36" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22172,7 +22157,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22183,12 +22168,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22196,7 +22181,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E37" s="27" t="inlineStr">
+      <c r="E37" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22219,12 +22204,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22232,7 +22217,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E38" s="27" t="inlineStr">
+      <c r="E38" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22255,12 +22240,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22268,7 +22253,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E39" s="27" t="inlineStr">
+      <c r="E39" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22280,7 +22265,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22291,12 +22276,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22304,7 +22289,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E40" s="27" t="inlineStr">
+      <c r="E40" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22327,12 +22312,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22340,7 +22325,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E41" s="27" t="inlineStr">
+      <c r="E41" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22363,12 +22348,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22376,7 +22361,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E42" s="27" t="inlineStr">
+      <c r="E42" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22388,7 +22373,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22399,12 +22384,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22412,7 +22397,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E43" s="27" t="inlineStr">
+      <c r="E43" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22435,20 +22420,20 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E44" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22460,7 +22445,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22471,12 +22456,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22484,7 +22469,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E45" s="27" t="inlineStr">
+      <c r="E45" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22496,7 +22481,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22507,12 +22492,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22520,7 +22505,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E46" s="27" t="inlineStr">
+      <c r="E46" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22543,12 +22528,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22556,7 +22541,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E47" s="27" t="inlineStr">
+      <c r="E47" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22579,20 +22564,20 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22604,7 +22589,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22615,12 +22600,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22628,7 +22613,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E49" s="27" t="inlineStr">
+      <c r="E49" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22651,12 +22636,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22664,7 +22649,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E50" s="27" t="inlineStr">
+      <c r="E50" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22676,7 +22661,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22687,12 +22672,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22700,7 +22685,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E51" s="27" t="inlineStr">
+      <c r="E51" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22712,7 +22697,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22723,12 +22708,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22736,7 +22721,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E52" s="27" t="inlineStr">
+      <c r="E52" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22759,12 +22744,12 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -22772,7 +22757,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E53" s="27" t="inlineStr">
+      <c r="E53" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22795,20 +22780,20 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E54" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22820,7 +22805,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22831,12 +22816,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22844,7 +22829,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E55" s="27" t="inlineStr">
+      <c r="E55" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22867,12 +22852,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22880,7 +22865,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E56" s="27" t="inlineStr">
+      <c r="E56" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22903,12 +22888,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22916,7 +22901,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E57" s="27" t="inlineStr">
+      <c r="E57" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22939,32 +22924,32 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E58" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F58" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22975,12 +22960,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22988,7 +22973,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E59" s="27" t="inlineStr">
+      <c r="E59" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23000,7 +22985,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -23011,12 +22996,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23024,7 +23009,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E60" s="27" t="inlineStr">
+      <c r="E60" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23036,7 +23021,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23047,12 +23032,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23060,7 +23045,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E61" s="27" t="inlineStr">
+      <c r="E61" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23083,20 +23068,20 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E62" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23108,7 +23093,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23119,12 +23104,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23132,7 +23117,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E63" s="27" t="inlineStr">
+      <c r="E63" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23155,12 +23140,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23168,7 +23153,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E64" s="27" t="inlineStr">
+      <c r="E64" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23191,12 +23176,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23204,7 +23189,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E65" s="27" t="inlineStr">
+      <c r="E65" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23227,12 +23212,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23240,7 +23225,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E66" s="27" t="inlineStr">
+      <c r="E66" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23263,12 +23248,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23276,7 +23261,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E67" s="27" t="inlineStr">
+      <c r="E67" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23299,12 +23284,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23312,7 +23297,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E68" s="27" t="inlineStr">
+      <c r="E68" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23335,12 +23320,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23348,7 +23333,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E69" s="27" t="inlineStr">
+      <c r="E69" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23371,20 +23356,20 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E70" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E70" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23396,7 +23381,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23407,12 +23392,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23420,7 +23405,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E71" s="27" t="inlineStr">
+      <c r="E71" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23443,12 +23428,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23456,7 +23441,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E72" s="27" t="inlineStr">
+      <c r="E72" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23479,12 +23464,12 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -23492,7 +23477,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E73" s="27" t="inlineStr">
+      <c r="E73" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23515,12 +23500,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23528,7 +23513,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E74" s="27" t="inlineStr">
+      <c r="E74" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23551,20 +23536,20 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E75" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23576,7 +23561,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23587,12 +23572,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23600,7 +23585,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E76" s="27" t="inlineStr">
+      <c r="E76" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23612,7 +23597,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23623,20 +23608,20 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E77" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E77" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23648,7 +23633,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23659,12 +23644,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23672,7 +23657,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E78" s="27" t="inlineStr">
+      <c r="E78" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23684,7 +23669,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23695,12 +23680,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23708,7 +23693,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E79" s="27" t="inlineStr">
+      <c r="E79" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23731,12 +23716,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23744,7 +23729,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E80" s="27" t="inlineStr">
+      <c r="E80" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23767,12 +23752,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23780,7 +23765,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E81" s="27" t="inlineStr">
+      <c r="E81" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23792,7 +23777,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23803,12 +23788,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23816,7 +23801,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E82" s="27" t="inlineStr">
+      <c r="E82" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23828,7 +23813,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23839,20 +23824,20 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E83" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E83" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23864,7 +23849,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23875,12 +23860,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23888,7 +23873,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E84" s="27" t="inlineStr">
+      <c r="E84" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23900,7 +23885,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23911,20 +23896,20 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E85" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E85" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23936,7 +23921,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23947,12 +23932,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23960,7 +23945,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E86" s="27" t="inlineStr">
+      <c r="E86" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23972,7 +23957,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23983,20 +23968,20 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E87" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E87" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24008,7 +23993,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24019,12 +24004,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24032,7 +24017,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E88" s="27" t="inlineStr">
+      <c r="E88" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24044,7 +24029,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24055,12 +24040,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24068,7 +24053,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E89" s="27" t="inlineStr">
+      <c r="E89" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24080,7 +24065,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24091,12 +24076,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24104,7 +24089,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E90" s="27" t="inlineStr">
+      <c r="E90" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24116,7 +24101,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24127,12 +24112,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24140,19 +24125,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E91" s="27" t="inlineStr">
+      <c r="E91" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24163,12 +24148,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24176,7 +24161,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E92" s="27" t="inlineStr">
+      <c r="E92" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24188,7 +24173,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24199,12 +24184,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24212,7 +24197,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E93" s="27" t="inlineStr">
+      <c r="E93" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24224,7 +24209,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24235,20 +24220,20 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E94" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E94" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24260,7 +24245,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24271,20 +24256,20 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E95" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E95" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24296,7 +24281,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24307,12 +24292,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24320,7 +24305,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E96" s="27" t="inlineStr">
+      <c r="E96" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24332,7 +24317,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24343,20 +24328,20 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E97" s="27" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E97" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24368,7 +24353,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24379,12 +24364,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24392,7 +24377,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E98" s="27" t="inlineStr">
+      <c r="E98" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24404,7 +24389,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24415,20 +24400,20 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E99" s="27" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E99" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24440,7 +24425,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24451,12 +24436,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24464,7 +24449,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E100" s="27" t="inlineStr">
+      <c r="E100" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24476,7 +24461,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24487,12 +24472,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24500,7 +24485,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E101" s="27" t="inlineStr">
+      <c r="E101" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24523,12 +24508,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24536,7 +24521,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E102" s="27" t="inlineStr">
+      <c r="E102" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24548,7 +24533,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24559,12 +24544,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24572,7 +24557,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E103" s="27" t="inlineStr">
+      <c r="E103" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24584,7 +24569,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24595,12 +24580,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24608,7 +24593,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E104" s="27" t="inlineStr">
+      <c r="E104" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24620,7 +24605,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24631,12 +24616,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24644,7 +24629,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E105" s="27" t="inlineStr">
+      <c r="E105" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24656,7 +24641,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24667,12 +24652,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24680,7 +24665,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E106" s="27" t="inlineStr">
+      <c r="E106" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24692,7 +24677,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24703,12 +24688,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24716,7 +24701,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E107" s="27" t="inlineStr">
+      <c r="E107" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24728,7 +24713,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24739,12 +24724,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24752,7 +24737,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E108" s="27" t="inlineStr">
+      <c r="E108" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24764,7 +24749,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24775,12 +24760,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24788,19 +24773,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E109" s="27" t="inlineStr">
+      <c r="E109" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24811,12 +24796,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24824,7 +24809,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E110" s="27" t="inlineStr">
+      <c r="E110" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24836,7 +24821,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24847,12 +24832,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24860,7 +24845,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E111" s="27" t="inlineStr">
+      <c r="E111" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24872,7 +24857,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24883,12 +24868,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24896,7 +24881,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E112" s="27" t="inlineStr">
+      <c r="E112" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24908,7 +24893,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24919,12 +24904,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24932,19 +24917,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E113" s="27" t="inlineStr">
+      <c r="E113" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24955,12 +24940,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24968,7 +24953,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E114" s="27" t="inlineStr">
+      <c r="E114" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24991,12 +24976,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25004,7 +24989,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E115" s="27" t="inlineStr">
+      <c r="E115" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25027,38 +25012,74 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C116" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E116" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G116" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H116" s="13" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C116" s="13" t="inlineStr">
+      <c r="C117" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D116" s="12" t="inlineStr">
+      <c r="D117" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E116" s="27" t="inlineStr">
+      <c r="E117" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F116" s="12" t="inlineStr">
+      <c r="F117" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G116" s="13" t="inlineStr">
+      <c r="G117" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H116" s="13" t="inlineStr"/>
+      <c r="H117" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H116"/>
+  <autoFilter ref="A1:H117"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T119, T120: đổi mã việc sau khi gộp bản PhuongXT (Gói thuê bao T113 thành T119, in phiếu từ form T114 thành T120); làm mới báo cáo hệ thống Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -829,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>116 việc (T01 - T108)</t>
+          <t>122 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>95 việc (81.9%)</t>
+          <t>101 việc (82.8%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21011,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21072,7 +21072,7 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T120</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
@@ -21736,17 +21736,17 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E25" s="26" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21772,17 +21772,17 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E26" s="26" t="inlineStr">
@@ -21797,7 +21797,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21808,17 +21808,17 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E27" s="26" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21844,12 +21844,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21880,12 +21880,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21905,7 +21905,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21916,12 +21916,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21941,7 +21941,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21952,17 +21952,17 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E31" s="26" t="inlineStr">
@@ -21977,7 +21977,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21988,17 +21988,17 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E32" s="26" t="inlineStr">
@@ -22013,7 +22013,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22024,17 +22024,17 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E33" s="26" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22060,12 +22060,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22085,7 +22085,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22096,12 +22096,12 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22132,17 +22132,17 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
@@ -22157,7 +22157,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22168,12 +22168,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22193,7 +22193,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22204,12 +22204,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22240,12 +22240,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22276,12 +22276,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22301,7 +22301,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22312,12 +22312,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22337,7 +22337,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22348,17 +22348,17 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E42" s="26" t="inlineStr">
@@ -22373,7 +22373,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22384,12 +22384,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22409,7 +22409,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22420,12 +22420,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22456,17 +22456,17 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E45" s="26" t="inlineStr">
@@ -22481,7 +22481,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22492,17 +22492,17 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E46" s="26" t="inlineStr">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22528,17 +22528,17 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E47" s="26" t="inlineStr">
@@ -22553,7 +22553,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22564,17 +22564,17 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E48" s="26" t="inlineStr">
@@ -22589,7 +22589,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22600,12 +22600,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22625,7 +22625,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22636,12 +22636,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22661,7 +22661,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22672,17 +22672,17 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E51" s="26" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22708,17 +22708,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E52" s="26" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22744,17 +22744,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E53" s="26" t="inlineStr">
@@ -22769,7 +22769,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22780,17 +22780,17 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E54" s="26" t="inlineStr">
@@ -22805,7 +22805,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22816,17 +22816,17 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E55" s="26" t="inlineStr">
@@ -22841,7 +22841,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22852,17 +22852,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E56" s="26" t="inlineStr">
@@ -22877,7 +22877,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22888,17 +22888,17 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E57" s="26" t="inlineStr">
@@ -22913,7 +22913,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22924,17 +22924,17 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E58" s="26" t="inlineStr">
@@ -22949,7 +22949,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22960,12 +22960,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22980,12 +22980,12 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22996,12 +22996,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23016,12 +23016,12 @@
       </c>
       <c r="F60" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23032,17 +23032,17 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E61" s="26" t="inlineStr">
@@ -23052,12 +23052,12 @@
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23068,17 +23068,17 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E62" s="26" t="inlineStr">
@@ -23088,12 +23088,12 @@
       </c>
       <c r="F62" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23104,12 +23104,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23124,12 +23124,12 @@
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23140,12 +23140,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23160,12 +23160,12 @@
       </c>
       <c r="F64" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23176,17 +23176,17 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E65" s="26" t="inlineStr">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23212,17 +23212,17 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E66" s="26" t="inlineStr">
@@ -23237,7 +23237,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23248,17 +23248,17 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E67" s="26" t="inlineStr">
@@ -23273,7 +23273,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23284,17 +23284,17 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E68" s="26" t="inlineStr">
@@ -23309,7 +23309,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23320,12 +23320,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23356,12 +23356,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23392,17 +23392,17 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E71" s="26" t="inlineStr">
@@ -23417,7 +23417,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23428,17 +23428,17 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E72" s="26" t="inlineStr">
@@ -23453,7 +23453,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23464,17 +23464,17 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E73" s="26" t="inlineStr">
@@ -23489,7 +23489,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23500,17 +23500,17 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E74" s="26" t="inlineStr">
@@ -23525,7 +23525,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23536,17 +23536,17 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E75" s="26" t="inlineStr">
@@ -23561,7 +23561,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23572,12 +23572,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23597,7 +23597,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23608,17 +23608,17 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E77" s="26" t="inlineStr">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23644,12 +23644,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23669,7 +23669,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23680,12 +23680,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23705,7 +23705,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23716,12 +23716,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23741,7 +23741,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23752,12 +23752,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23777,7 +23777,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23788,17 +23788,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E82" s="26" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23824,17 +23824,17 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E83" s="26" t="inlineStr">
@@ -23849,7 +23849,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23860,17 +23860,17 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E84" s="26" t="inlineStr">
@@ -23885,7 +23885,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23896,17 +23896,17 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E85" s="26" t="inlineStr">
@@ -23921,7 +23921,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23932,12 +23932,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23957,7 +23957,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23968,12 +23968,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23993,7 +23993,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24004,17 +24004,17 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E88" s="26" t="inlineStr">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24040,17 +24040,17 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E89" s="26" t="inlineStr">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24076,12 +24076,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24112,12 +24112,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24137,7 +24137,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24148,17 +24148,17 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E92" s="26" t="inlineStr">
@@ -24168,12 +24168,12 @@
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24184,17 +24184,17 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E93" s="26" t="inlineStr">
@@ -24204,12 +24204,12 @@
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24220,12 +24220,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24240,12 +24240,12 @@
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24256,17 +24256,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E95" s="26" t="inlineStr">
@@ -24276,12 +24276,12 @@
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24292,12 +24292,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24312,12 +24312,12 @@
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24328,12 +24328,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24348,12 +24348,12 @@
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24364,17 +24364,17 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E98" s="26" t="inlineStr">
@@ -24389,7 +24389,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24400,17 +24400,17 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E99" s="26" t="inlineStr">
@@ -24425,7 +24425,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24436,12 +24436,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24461,7 +24461,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24472,17 +24472,17 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E101" s="26" t="inlineStr">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24508,12 +24508,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24544,12 +24544,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24580,17 +24580,17 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E104" s="26" t="inlineStr">
@@ -24605,7 +24605,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24616,17 +24616,17 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E105" s="26" t="inlineStr">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24652,12 +24652,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24677,7 +24677,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24688,12 +24688,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24713,7 +24713,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24724,12 +24724,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24749,7 +24749,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24760,12 +24760,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24785,7 +24785,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24796,12 +24796,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24816,12 +24816,12 @@
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24832,12 +24832,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24852,12 +24852,12 @@
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24868,12 +24868,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24888,12 +24888,12 @@
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24904,12 +24904,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24924,12 +24924,12 @@
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24940,12 +24940,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24965,7 +24965,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24976,12 +24976,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25001,7 +25001,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25012,12 +25012,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25032,12 +25032,12 @@
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25048,38 +25048,254 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+        </is>
+      </c>
+      <c r="D117" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E117" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F117" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="23" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C118" s="13" t="inlineStr">
+        <is>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E118" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G118" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+        </is>
+      </c>
+      <c r="H118" s="13" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="16" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="25" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+        </is>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E119" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F119" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+        </is>
+      </c>
+      <c r="H119" s="5" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="12" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="23" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="C120" s="13" t="inlineStr">
+        <is>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E120" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G120" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H120" s="13" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="16" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="25" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D121" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E121" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F121" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H121" s="5" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="23" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C122" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D122" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E122" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G122" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H122" s="13" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="16" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D117" s="16" t="inlineStr">
+      <c r="D123" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E117" s="26" t="inlineStr">
+      <c r="E123" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F117" s="16" t="inlineStr">
+      <c r="F123" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G117" s="5" t="inlineStr">
+      <c r="G123" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H117" s="5" t="inlineStr"/>
+      <c r="H123" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H117"/>
+  <autoFilter ref="A1:H123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T122: ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45)
Giữ TT58 theo file, TT152 theo iFaster. Trường anTam trong CAU_HINH_BC, apDung đọc; link cũ hiện Báo cáo chưa có mẫu. kiem_tra.py hạ ngưỡng 140 xuống 125.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -829,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>122 việc (T01 - T108)</t>
+          <t>124 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>101 việc (82.8%)</t>
+          <t>103 việc (83.1%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21011,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21664,12 +21664,12 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -21689,7 +21689,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
@@ -21700,17 +21700,17 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E24" s="26" t="inlineStr">
@@ -21725,7 +21725,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -21736,17 +21736,17 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E25" s="26" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21772,17 +21772,17 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E26" s="26" t="inlineStr">
@@ -21797,7 +21797,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21808,12 +21808,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21844,12 +21844,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21880,12 +21880,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21916,12 +21916,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21952,17 +21952,17 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E31" s="26" t="inlineStr">
@@ -21977,7 +21977,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21988,17 +21988,17 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E32" s="26" t="inlineStr">
@@ -22013,7 +22013,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22024,17 +22024,17 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E33" s="26" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22060,17 +22060,17 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E34" s="26" t="inlineStr">
@@ -22085,7 +22085,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22096,17 +22096,17 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E35" s="26" t="inlineStr">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22132,12 +22132,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22168,12 +22168,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22204,12 +22204,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22240,12 +22240,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22276,12 +22276,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22301,7 +22301,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22312,12 +22312,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22348,17 +22348,17 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E42" s="26" t="inlineStr">
@@ -22373,7 +22373,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22384,12 +22384,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22409,7 +22409,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22420,17 +22420,17 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E44" s="26" t="inlineStr">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22456,12 +22456,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22492,12 +22492,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22528,12 +22528,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22553,7 +22553,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22564,12 +22564,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22600,12 +22600,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22625,7 +22625,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22636,12 +22636,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22661,7 +22661,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22672,17 +22672,17 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E51" s="26" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22708,17 +22708,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E52" s="26" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22744,12 +22744,12 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -22769,7 +22769,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22780,12 +22780,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22816,17 +22816,17 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E55" s="26" t="inlineStr">
@@ -22841,7 +22841,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22852,17 +22852,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E56" s="26" t="inlineStr">
@@ -22877,7 +22877,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22888,12 +22888,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22913,7 +22913,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22924,12 +22924,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22949,7 +22949,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22960,12 +22960,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22996,12 +22996,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23032,17 +23032,17 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E61" s="26" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23068,17 +23068,17 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E62" s="26" t="inlineStr">
@@ -23093,7 +23093,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23104,12 +23104,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23140,12 +23140,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23176,17 +23176,17 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E65" s="26" t="inlineStr">
@@ -23196,12 +23196,12 @@
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23212,17 +23212,17 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E66" s="26" t="inlineStr">
@@ -23232,12 +23232,12 @@
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23248,12 +23248,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23273,7 +23273,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23284,12 +23284,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23309,7 +23309,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23320,17 +23320,17 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E69" s="26" t="inlineStr">
@@ -23345,7 +23345,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23356,17 +23356,17 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E70" s="26" t="inlineStr">
@@ -23381,7 +23381,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23392,12 +23392,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23428,12 +23428,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23464,12 +23464,12 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -23500,12 +23500,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23536,12 +23536,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23572,12 +23572,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23608,17 +23608,17 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E77" s="26" t="inlineStr">
@@ -23633,7 +23633,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23644,17 +23644,17 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E78" s="26" t="inlineStr">
@@ -23669,7 +23669,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23680,12 +23680,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23716,12 +23716,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23752,12 +23752,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23788,17 +23788,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E82" s="26" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23824,17 +23824,17 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E83" s="26" t="inlineStr">
@@ -23849,7 +23849,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23860,17 +23860,17 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E84" s="26" t="inlineStr">
@@ -23885,7 +23885,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23896,17 +23896,17 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E85" s="26" t="inlineStr">
@@ -23921,7 +23921,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23932,12 +23932,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23957,7 +23957,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23968,12 +23968,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -24004,12 +24004,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24040,12 +24040,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24076,17 +24076,17 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E90" s="26" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24112,17 +24112,17 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E91" s="26" t="inlineStr">
@@ -24137,7 +24137,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24148,17 +24148,17 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E92" s="26" t="inlineStr">
@@ -24173,7 +24173,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24184,17 +24184,17 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E93" s="26" t="inlineStr">
@@ -24209,7 +24209,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24220,17 +24220,17 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E94" s="26" t="inlineStr">
@@ -24245,7 +24245,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24256,17 +24256,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E95" s="26" t="inlineStr">
@@ -24281,7 +24281,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24292,12 +24292,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24317,7 +24317,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24328,12 +24328,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24353,7 +24353,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24364,12 +24364,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24384,12 +24384,12 @@
       </c>
       <c r="F98" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24400,12 +24400,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24420,12 +24420,12 @@
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24436,12 +24436,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24461,7 +24461,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24472,17 +24472,17 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E101" s="26" t="inlineStr">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24508,12 +24508,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24544,17 +24544,17 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E103" s="26" t="inlineStr">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24580,17 +24580,17 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E104" s="26" t="inlineStr">
@@ -24605,7 +24605,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24616,17 +24616,17 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E105" s="26" t="inlineStr">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24652,17 +24652,17 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E106" s="26" t="inlineStr">
@@ -24677,7 +24677,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24688,17 +24688,17 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E107" s="26" t="inlineStr">
@@ -24713,7 +24713,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24724,12 +24724,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24749,7 +24749,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24760,12 +24760,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24785,7 +24785,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24796,12 +24796,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24821,7 +24821,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24832,12 +24832,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24868,12 +24868,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24893,7 +24893,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24904,12 +24904,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24929,7 +24929,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24940,12 +24940,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24965,7 +24965,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24976,12 +24976,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25001,7 +25001,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25012,12 +25012,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25032,12 +25032,12 @@
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25048,12 +25048,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25068,12 +25068,12 @@
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25084,12 +25084,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25109,7 +25109,7 @@
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25120,12 +25120,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25145,7 +25145,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25156,12 +25156,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25176,12 +25176,12 @@
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25192,12 +25192,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25212,12 +25212,12 @@
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25228,12 +25228,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25264,38 +25264,110 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D123" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E123" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F123" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="12" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="23" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C124" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E124" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G124" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H124" s="13" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C125" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D123" s="16" t="inlineStr">
+      <c r="D125" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E123" s="26" t="inlineStr">
+      <c r="E125" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F123" s="16" t="inlineStr">
+      <c r="F125" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G123" s="5" t="inlineStr">
+      <c r="G125" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H123" s="5" t="inlineStr"/>
+      <c r="H125" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H123"/>
+  <autoFilter ref="A1:H125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T133: thiết kế lại màn Tổng quan: chỉ số sức khoẻ tài chính, thác nước lợi nhuận, dòng tiền, lọc kỳ, chi nhánh, tuỳ chỉnh khối (QD46)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -829,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>124 việc (T01 - T108)</t>
+          <t>135 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>103 việc (83.1%)</t>
+          <t>114 việc (84.4%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21011,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21664,12 +21664,12 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -21689,7 +21689,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
@@ -21700,12 +21700,12 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -21725,7 +21725,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -21736,17 +21736,17 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E25" s="26" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21772,17 +21772,17 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E26" s="26" t="inlineStr">
@@ -21797,7 +21797,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21808,12 +21808,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21844,12 +21844,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21880,12 +21880,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21905,7 +21905,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21916,12 +21916,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21941,7 +21941,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21952,12 +21952,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21977,7 +21977,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21988,12 +21988,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22013,7 +22013,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22024,17 +22024,17 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E33" s="26" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22060,12 +22060,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22085,7 +22085,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22096,17 +22096,17 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E35" s="26" t="inlineStr">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22132,17 +22132,17 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
@@ -22157,7 +22157,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22168,17 +22168,17 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E37" s="26" t="inlineStr">
@@ -22193,7 +22193,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22204,12 +22204,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22240,12 +22240,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22276,12 +22276,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22301,7 +22301,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22312,12 +22312,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22337,7 +22337,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22348,12 +22348,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22373,7 +22373,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22384,12 +22384,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22409,7 +22409,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22420,12 +22420,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22456,17 +22456,17 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E45" s="26" t="inlineStr">
@@ -22481,7 +22481,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22492,17 +22492,17 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E46" s="26" t="inlineStr">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22528,12 +22528,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22553,7 +22553,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22564,12 +22564,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22589,7 +22589,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22600,12 +22600,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22625,7 +22625,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22636,12 +22636,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22661,7 +22661,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22672,12 +22672,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22708,12 +22708,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22744,17 +22744,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E53" s="26" t="inlineStr">
@@ -22769,7 +22769,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22780,17 +22780,17 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E54" s="26" t="inlineStr">
@@ -22805,7 +22805,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22816,12 +22816,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22841,7 +22841,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22852,17 +22852,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E56" s="26" t="inlineStr">
@@ -22877,7 +22877,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22888,12 +22888,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22913,7 +22913,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22924,12 +22924,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22949,7 +22949,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22960,12 +22960,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22996,12 +22996,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23021,7 +23021,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23032,12 +23032,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23068,12 +23068,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23093,7 +23093,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23104,17 +23104,17 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E63" s="26" t="inlineStr">
@@ -23129,7 +23129,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23140,12 +23140,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23176,12 +23176,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23212,12 +23212,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23237,7 +23237,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23248,17 +23248,17 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E67" s="26" t="inlineStr">
@@ -23268,12 +23268,12 @@
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23284,12 +23284,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23304,12 +23304,12 @@
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23320,12 +23320,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23340,12 +23340,12 @@
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23356,12 +23356,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23376,12 +23376,12 @@
       </c>
       <c r="F70" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23392,17 +23392,17 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E71" s="26" t="inlineStr">
@@ -23412,12 +23412,12 @@
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23428,17 +23428,17 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E72" s="26" t="inlineStr">
@@ -23448,12 +23448,12 @@
       </c>
       <c r="F72" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23464,17 +23464,17 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E73" s="26" t="inlineStr">
@@ -23484,12 +23484,12 @@
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23500,12 +23500,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23520,12 +23520,12 @@
       </c>
       <c r="F74" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23536,12 +23536,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23556,12 +23556,12 @@
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23572,12 +23572,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23592,12 +23592,12 @@
       </c>
       <c r="F76" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23608,12 +23608,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23628,12 +23628,12 @@
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23644,17 +23644,17 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E78" s="26" t="inlineStr">
@@ -23669,7 +23669,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23680,12 +23680,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23705,7 +23705,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23716,12 +23716,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23741,7 +23741,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23752,12 +23752,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23777,7 +23777,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23788,17 +23788,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E82" s="26" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23824,17 +23824,17 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E83" s="26" t="inlineStr">
@@ -23849,7 +23849,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23860,12 +23860,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23885,7 +23885,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23896,12 +23896,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23921,7 +23921,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23932,17 +23932,17 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E86" s="26" t="inlineStr">
@@ -23957,7 +23957,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23968,17 +23968,17 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E87" s="26" t="inlineStr">
@@ -23993,7 +23993,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24004,17 +24004,17 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E88" s="26" t="inlineStr">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24040,17 +24040,17 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E89" s="26" t="inlineStr">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24076,12 +24076,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24112,12 +24112,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24137,7 +24137,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24148,17 +24148,17 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E92" s="26" t="inlineStr">
@@ -24173,7 +24173,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24184,17 +24184,17 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E93" s="26" t="inlineStr">
@@ -24209,7 +24209,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24220,12 +24220,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24245,7 +24245,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24256,17 +24256,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E95" s="26" t="inlineStr">
@@ -24281,7 +24281,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24292,12 +24292,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24317,7 +24317,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24328,17 +24328,17 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E97" s="26" t="inlineStr">
@@ -24353,7 +24353,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24364,17 +24364,17 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E98" s="26" t="inlineStr">
@@ -24389,7 +24389,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24400,17 +24400,17 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E99" s="26" t="inlineStr">
@@ -24425,7 +24425,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24436,17 +24436,17 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E100" s="26" t="inlineStr">
@@ -24456,12 +24456,12 @@
       </c>
       <c r="F100" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24472,17 +24472,17 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E101" s="26" t="inlineStr">
@@ -24492,12 +24492,12 @@
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24508,17 +24508,17 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E102" s="26" t="inlineStr">
@@ -24528,12 +24528,12 @@
       </c>
       <c r="F102" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24544,17 +24544,17 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E103" s="26" t="inlineStr">
@@ -24564,12 +24564,12 @@
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24580,12 +24580,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24600,12 +24600,12 @@
       </c>
       <c r="F104" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24616,17 +24616,17 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E105" s="26" t="inlineStr">
@@ -24636,12 +24636,12 @@
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24652,12 +24652,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24672,12 +24672,12 @@
       </c>
       <c r="F106" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24688,17 +24688,17 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E107" s="26" t="inlineStr">
@@ -24708,12 +24708,12 @@
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24724,12 +24724,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24744,12 +24744,12 @@
       </c>
       <c r="F108" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24760,12 +24760,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24780,12 +24780,12 @@
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24796,12 +24796,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24816,12 +24816,12 @@
       </c>
       <c r="F110" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24832,12 +24832,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24868,12 +24868,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24893,7 +24893,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24904,12 +24904,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24929,7 +24929,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24940,17 +24940,17 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E114" s="26" t="inlineStr">
@@ -24965,7 +24965,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24976,12 +24976,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25001,7 +25001,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25012,12 +25012,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25037,7 +25037,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25048,17 +25048,17 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E117" s="26" t="inlineStr">
@@ -25073,7 +25073,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25084,17 +25084,17 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E118" s="26" t="inlineStr">
@@ -25104,12 +25104,12 @@
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25120,12 +25120,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25140,12 +25140,12 @@
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25156,12 +25156,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25176,12 +25176,12 @@
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25192,12 +25192,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25212,12 +25212,12 @@
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25228,12 +25228,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25253,7 +25253,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25264,12 +25264,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25289,7 +25289,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25300,12 +25300,12 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -25325,7 +25325,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25336,38 +25336,434 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
+          <t>T28</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+        </is>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E125" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F125" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+        </is>
+      </c>
+      <c r="H125" s="5" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="12" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="23" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E126" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G126" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+        </is>
+      </c>
+      <c r="H126" s="13" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="25" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+        </is>
+      </c>
+      <c r="D127" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E127" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F127" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+        </is>
+      </c>
+      <c r="H127" s="5" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="23" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E128" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G128" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+        </is>
+      </c>
+      <c r="H128" s="13" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="25" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+        </is>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E129" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F129" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-khung-web.md`</t>
+        </is>
+      </c>
+      <c r="H129" s="5" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="12" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="23" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E130" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G130" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+        </is>
+      </c>
+      <c r="H130" s="13" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="25" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+        </is>
+      </c>
+      <c r="D131" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E131" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F131" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+        </is>
+      </c>
+      <c r="H131" s="5" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="12" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="23" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="inlineStr">
+        <is>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E132" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G132" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+        </is>
+      </c>
+      <c r="H132" s="13" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="25" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+        </is>
+      </c>
+      <c r="D133" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E133" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F133" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H133" s="5" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="12" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="23" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D134" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E134" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G134" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H134" s="13" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="25" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D135" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E135" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F135" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H135" s="5" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="23" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C125" s="5" t="inlineStr">
+      <c r="C136" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D136" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E125" s="26" t="inlineStr">
+      <c r="E136" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F125" s="16" t="inlineStr">
+      <c r="F136" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G125" s="5" t="inlineStr">
+      <c r="G136" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H125" s="5" t="inlineStr"/>
+      <c r="H136" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H125"/>
+  <autoFilter ref="A1:H136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T134: mẫu in tự cân đối khi đổi khổ dọc, ngang, A4, A5
Cột bảng chia theo tỷ lệ thay mm cố định; đổi khổ co giãn độ rộng cột theo vùng in;
khổ hẹp thì chữ bảng co (tối thiểu 75%), thông tin một cột dưới 150 mm, số xuống dòng ở dấu chấm.
Chưa in giấy thật, chưa đo ở TT99, TT58.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -622,7 +622,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ngày xuất: 10/10/2026 | Bản mẫu iaccdemo (React 19 + TypeScript + Vite) | Deploy: https://iaccdemo.pages.dev</t>
+          <t>Ngày xuất: 11/10/2026 | Bản mẫu iaccdemo (React 19 + TypeScript + Vite) | Deploy: https://iaccdemo.pages.dev</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>135 việc (T01 - T108)</t>
+          <t>136 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>114 việc (84.4%)</t>
+          <t>115 việc (84.6%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21011,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21664,12 +21664,12 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -21684,12 +21684,12 @@
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr"/>
@@ -21700,17 +21700,17 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E24" s="26" t="inlineStr">
@@ -21725,7 +21725,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr"/>
@@ -21736,12 +21736,12 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -21761,7 +21761,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -21772,12 +21772,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21797,7 +21797,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21808,12 +21808,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21844,12 +21844,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21880,12 +21880,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21905,7 +21905,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21916,12 +21916,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21941,7 +21941,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21952,12 +21952,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21977,7 +21977,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21988,12 +21988,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22013,7 +22013,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22024,12 +22024,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22060,17 +22060,17 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E34" s="26" t="inlineStr">
@@ -22085,7 +22085,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22096,17 +22096,17 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E35" s="26" t="inlineStr">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22132,17 +22132,17 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
@@ -22157,7 +22157,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22168,12 +22168,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22204,17 +22204,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E38" s="26" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22240,12 +22240,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22276,12 +22276,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22312,12 +22312,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22348,12 +22348,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22384,12 +22384,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22420,17 +22420,17 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E44" s="26" t="inlineStr">
@@ -22445,7 +22445,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22456,12 +22456,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22481,7 +22481,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22492,17 +22492,17 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E46" s="26" t="inlineStr">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22528,17 +22528,17 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E47" s="26" t="inlineStr">
@@ -22553,7 +22553,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22564,12 +22564,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22600,12 +22600,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22636,12 +22636,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22672,12 +22672,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22708,12 +22708,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22744,12 +22744,12 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -22780,12 +22780,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22816,17 +22816,17 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E55" s="26" t="inlineStr">
@@ -22841,7 +22841,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22852,17 +22852,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E56" s="26" t="inlineStr">
@@ -22877,7 +22877,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22888,12 +22888,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22924,12 +22924,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22960,12 +22960,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22996,12 +22996,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23032,12 +23032,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23068,12 +23068,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23093,7 +23093,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23104,12 +23104,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23140,17 +23140,17 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E64" s="26" t="inlineStr">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23176,12 +23176,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23212,12 +23212,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23248,12 +23248,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23284,17 +23284,17 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E68" s="26" t="inlineStr">
@@ -23309,7 +23309,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23320,12 +23320,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23356,12 +23356,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23381,7 +23381,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23392,12 +23392,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23417,7 +23417,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23428,12 +23428,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23464,12 +23464,12 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -23500,17 +23500,17 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E74" s="26" t="inlineStr">
@@ -23525,7 +23525,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23536,12 +23536,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23572,12 +23572,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23608,12 +23608,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23644,17 +23644,17 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E78" s="26" t="inlineStr">
@@ -23664,12 +23664,12 @@
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23680,12 +23680,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23705,7 +23705,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23716,12 +23716,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23741,7 +23741,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23752,12 +23752,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23788,17 +23788,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E82" s="26" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23824,12 +23824,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23860,12 +23860,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23896,12 +23896,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23932,12 +23932,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23968,12 +23968,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -24004,12 +24004,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24040,12 +24040,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24076,17 +24076,17 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E90" s="26" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24112,12 +24112,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24148,12 +24148,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24184,12 +24184,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24220,12 +24220,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24256,17 +24256,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E95" s="26" t="inlineStr">
@@ -24281,7 +24281,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24292,12 +24292,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24317,7 +24317,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24328,17 +24328,17 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E97" s="26" t="inlineStr">
@@ -24353,7 +24353,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24364,12 +24364,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24389,7 +24389,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24400,12 +24400,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24436,12 +24436,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24472,12 +24472,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24508,12 +24508,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24544,17 +24544,17 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E103" s="26" t="inlineStr">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24580,12 +24580,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24605,7 +24605,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24616,17 +24616,17 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E105" s="26" t="inlineStr">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24652,12 +24652,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24677,7 +24677,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24688,17 +24688,17 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E107" s="26" t="inlineStr">
@@ -24713,7 +24713,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24724,12 +24724,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24749,7 +24749,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24760,12 +24760,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24785,7 +24785,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24796,12 +24796,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24821,7 +24821,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24832,12 +24832,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24852,12 +24852,12 @@
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24868,12 +24868,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24893,7 +24893,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24904,12 +24904,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24929,7 +24929,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24940,17 +24940,17 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E114" s="26" t="inlineStr">
@@ -24965,7 +24965,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24976,17 +24976,17 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E115" s="26" t="inlineStr">
@@ -25001,7 +25001,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25012,12 +25012,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25037,7 +25037,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25048,17 +25048,17 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E117" s="26" t="inlineStr">
@@ -25073,7 +25073,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25084,12 +25084,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25109,7 +25109,7 @@
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25120,17 +25120,17 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E119" s="26" t="inlineStr">
@@ -25145,7 +25145,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25156,12 +25156,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25181,7 +25181,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25192,12 +25192,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25228,12 +25228,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25253,7 +25253,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25264,12 +25264,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25289,7 +25289,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25300,12 +25300,12 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -25325,7 +25325,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25336,12 +25336,12 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25361,7 +25361,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25372,12 +25372,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25397,7 +25397,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25408,12 +25408,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25433,7 +25433,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25444,12 +25444,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25469,7 +25469,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25480,12 +25480,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25500,12 +25500,12 @@
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25516,12 +25516,12 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -25541,7 +25541,7 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25552,12 +25552,12 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -25577,7 +25577,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25588,12 +25588,12 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -25613,7 +25613,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25624,12 +25624,12 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -25644,12 +25644,12 @@
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25660,12 +25660,12 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -25696,12 +25696,12 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -25732,38 +25732,74 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C136" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D136" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E136" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G136" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H136" s="13" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="16" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C136" s="13" t="inlineStr">
+      <c r="C137" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D136" s="12" t="inlineStr">
+      <c r="D137" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E136" s="26" t="inlineStr">
+      <c r="E137" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F136" s="12" t="inlineStr">
+      <c r="F137" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G136" s="13" t="inlineStr">
+      <c r="G137" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H136" s="13" t="inlineStr"/>
+      <c r="H137" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H136"/>
+  <autoFilter ref="A1:H137"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T136, T137: xong; nhật ký, QD47, CHANGELOG, báo cáo hệ thống; tách việc T139, T140
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -829,7 +829,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>136 việc (T01 - T108)</t>
+          <t>142 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>115 việc (84.6%)</t>
+          <t>118 việc (83.1%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>21 việc</t>
+          <t>24 việc</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -21011,7 +21011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H137"/>
+  <dimension ref="A1:H143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21020,7 +21020,7 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="57" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -21072,15 +21072,19 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T120</t>
+          <t>T138</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr"/>
+          <t>Màn onboard khi bấm từ FABi sang IACC: khởi tạo đơn vị kế toán, điền sẵn từ FABi (chi nhánh, kho, cách đồng bộ, số dư đầu kỳ)</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
       <c r="E2" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21090,7 +21094,7 @@
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Phát hiện khi làm T112</t>
+          <t>Đã đề xuất luồng, chờ PhuongXT chốt 3 điểm, xem `2026-10-10-phuongxt-y-tuong-onboard-fabi.md`</t>
         </is>
       </c>
     </row>
@@ -21100,12 +21104,12 @@
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>T109</t>
+          <t>T139</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+          <t>Phiếu nhập, xuất, điều chuyển kho tự lấy mục chi phí, công việc ngầm định theo kho đã chọn</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr"/>
@@ -21118,7 +21122,7 @@
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
+          <t>Tách từ T136. Kho đã có ô `mucCp`, `congViec` ở `truong-dm.ts` 1.8. Sửa `ChungTuForm.tsx`</t>
         </is>
       </c>
     </row>
@@ -21128,12 +21132,12 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>T110</t>
+          <t>T140</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
+          <t>Đồng bộ POS có tích tự hạch toán theo phương thức thanh toán thì sinh phiếu thu thật vào danh sách Thu tiền mặt, Thu ngân hàng (hiện chỉ báo số phiếu bằng toast)</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
@@ -21146,7 +21150,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+          <t>Tách từ T137. Phiếu thu Nợ TK của phương thức / Có 131, lấy từ `DS_PTTT` ở `danh-muc/data.ts`</t>
         </is>
       </c>
     </row>
@@ -21156,19 +21160,15 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T120</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
+          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr"/>
       <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21178,7 +21178,7 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+          <t>Phát hiện khi làm T112</t>
         </is>
       </c>
     </row>
@@ -21188,19 +21188,15 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T109</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr"/>
       <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21210,7 +21206,7 @@
       <c r="G6" s="13" t="inlineStr"/>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T25</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21220,19 +21216,15 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21240,7 +21232,11 @@
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n">
@@ -21248,15 +21244,19 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T101</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr"/>
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21266,7 +21266,7 @@
       <c r="G8" s="13" t="inlineStr"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
         </is>
       </c>
     </row>
@@ -21276,15 +21276,19 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21294,7 +21298,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Chỉ máy Trum chạy được script</t>
+          <t>Tách từ T25</t>
         </is>
       </c>
     </row>
@@ -21304,15 +21308,19 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr"/>
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21320,11 +21328,7 @@
       </c>
       <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
-        </is>
-      </c>
+      <c r="H10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
@@ -21332,12 +21336,12 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr"/>
@@ -21350,7 +21354,7 @@
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
         </is>
       </c>
     </row>
@@ -21360,12 +21364,12 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
@@ -21376,7 +21380,11 @@
       </c>
       <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="13" t="inlineStr"/>
-      <c r="H12" s="13" t="inlineStr"/>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>Chỉ máy Trum chạy được script</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
@@ -21384,12 +21392,12 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
@@ -21402,7 +21410,7 @@
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
         </is>
       </c>
     </row>
@@ -21412,12 +21420,12 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
@@ -21430,7 +21438,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
         </is>
       </c>
     </row>
@@ -21440,12 +21448,12 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
@@ -21456,11 +21464,7 @@
       </c>
       <c r="F15" s="16" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
-        </is>
-      </c>
+      <c r="H15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n">
@@ -21468,12 +21472,12 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
@@ -21486,7 +21490,7 @@
       <c r="G16" s="13" t="inlineStr"/>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
         </is>
       </c>
     </row>
@@ -21496,12 +21500,12 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
@@ -21514,7 +21518,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
         </is>
       </c>
     </row>
@@ -21524,12 +21528,12 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
@@ -21542,7 +21546,7 @@
       <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -21552,12 +21556,12 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
@@ -21570,7 +21574,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -21580,12 +21584,12 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
@@ -21598,7 +21602,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -21608,12 +21612,12 @@
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
@@ -21626,7 +21630,7 @@
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -21636,12 +21640,12 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
@@ -21654,7 +21658,7 @@
       <c r="G22" s="13" t="inlineStr"/>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -21664,35 +21668,27 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E23" s="26" t="inlineStr">
-        <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>11/10/2026</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr"/>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr"/>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Chưa có file logo iPOS</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="n">
@@ -21700,35 +21696,27 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E24" s="26" t="inlineStr">
-        <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
-        </is>
-      </c>
-      <c r="H24" s="13" t="inlineStr"/>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr"/>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr"/>
+      <c r="G24" s="13" t="inlineStr"/>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="n">
@@ -21736,35 +21724,27 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E25" s="26" t="inlineStr">
-        <is>
-          <t>Xong</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>10/10/2026</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr"/>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr"/>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Chờ</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n">
@@ -21772,17 +21752,17 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E26" s="26" t="inlineStr">
@@ -21792,12 +21772,12 @@
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21808,17 +21788,17 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E27" s="26" t="inlineStr">
@@ -21828,12 +21808,12 @@
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21844,17 +21824,17 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E28" s="26" t="inlineStr">
@@ -21864,12 +21844,12 @@
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21880,17 +21860,17 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E29" s="26" t="inlineStr">
@@ -21900,12 +21880,12 @@
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21916,17 +21896,17 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E30" s="26" t="inlineStr">
@@ -21941,7 +21921,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21952,12 +21932,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21977,7 +21957,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21988,12 +21968,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22013,7 +21993,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22024,12 +22004,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22049,7 +22029,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22060,12 +22040,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22085,7 +22065,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22096,17 +22076,17 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E35" s="26" t="inlineStr">
@@ -22121,7 +22101,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22132,12 +22112,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22157,7 +22137,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22168,17 +22148,17 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E37" s="26" t="inlineStr">
@@ -22193,7 +22173,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22204,17 +22184,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E38" s="26" t="inlineStr">
@@ -22229,7 +22209,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22240,12 +22220,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22265,7 +22245,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22276,12 +22256,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22301,7 +22281,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22312,17 +22292,17 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E41" s="26" t="inlineStr">
@@ -22337,7 +22317,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22348,12 +22328,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22373,7 +22353,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22384,17 +22364,17 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E43" s="26" t="inlineStr">
@@ -22409,7 +22389,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22420,17 +22400,17 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E44" s="26" t="inlineStr">
@@ -22445,7 +22425,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22456,17 +22436,17 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E45" s="26" t="inlineStr">
@@ -22481,7 +22461,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22492,17 +22472,17 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E46" s="26" t="inlineStr">
@@ -22517,7 +22497,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22528,17 +22508,17 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E47" s="26" t="inlineStr">
@@ -22553,7 +22533,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22564,12 +22544,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22589,7 +22569,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22600,12 +22580,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22625,7 +22605,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22636,12 +22616,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22661,7 +22641,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22672,17 +22652,17 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E51" s="26" t="inlineStr">
@@ -22697,7 +22677,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22708,17 +22688,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E52" s="26" t="inlineStr">
@@ -22733,7 +22713,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22744,17 +22724,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E53" s="26" t="inlineStr">
@@ -22769,7 +22749,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22780,12 +22760,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22805,7 +22785,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22816,12 +22796,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22841,7 +22821,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22852,17 +22832,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E56" s="26" t="inlineStr">
@@ -22877,7 +22857,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22888,12 +22868,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22913,7 +22893,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22924,12 +22904,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22949,7 +22929,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22960,12 +22940,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22985,7 +22965,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22996,12 +22976,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23021,7 +23001,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23032,12 +23012,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23057,7 +23037,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23068,17 +23048,17 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E62" s="26" t="inlineStr">
@@ -23093,7 +23073,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23104,12 +23084,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23129,7 +23109,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23140,12 +23120,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23165,7 +23145,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23176,17 +23156,17 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E65" s="26" t="inlineStr">
@@ -23201,7 +23181,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23212,17 +23192,17 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E66" s="26" t="inlineStr">
@@ -23237,7 +23217,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23248,17 +23228,17 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E67" s="26" t="inlineStr">
@@ -23273,7 +23253,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23284,17 +23264,17 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E68" s="26" t="inlineStr">
@@ -23309,7 +23289,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23320,12 +23300,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23345,7 +23325,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23356,12 +23336,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23381,7 +23361,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23392,17 +23372,17 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E71" s="26" t="inlineStr">
@@ -23417,7 +23397,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23428,17 +23408,17 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E72" s="26" t="inlineStr">
@@ -23453,7 +23433,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23464,17 +23444,17 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E73" s="26" t="inlineStr">
@@ -23489,7 +23469,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23500,17 +23480,17 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E74" s="26" t="inlineStr">
@@ -23525,7 +23505,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23536,17 +23516,17 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E75" s="26" t="inlineStr">
@@ -23561,7 +23541,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23572,17 +23552,17 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E76" s="26" t="inlineStr">
@@ -23597,7 +23577,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23608,17 +23588,17 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E77" s="26" t="inlineStr">
@@ -23633,7 +23613,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23644,17 +23624,17 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E78" s="26" t="inlineStr">
@@ -23669,7 +23649,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23680,12 +23660,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23700,12 +23680,12 @@
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23716,12 +23696,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23736,12 +23716,12 @@
       </c>
       <c r="F80" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23752,17 +23732,17 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E81" s="26" t="inlineStr">
@@ -23772,12 +23752,12 @@
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23788,17 +23768,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E82" s="26" t="inlineStr">
@@ -23808,12 +23788,12 @@
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23824,12 +23804,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23844,12 +23824,12 @@
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23860,12 +23840,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23880,12 +23860,12 @@
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23896,17 +23876,17 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E85" s="26" t="inlineStr">
@@ -23921,7 +23901,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23932,17 +23912,17 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E86" s="26" t="inlineStr">
@@ -23957,7 +23937,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23968,17 +23948,17 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E87" s="26" t="inlineStr">
@@ -23993,7 +23973,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24004,17 +23984,17 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E88" s="26" t="inlineStr">
@@ -24029,7 +24009,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24040,12 +24020,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24076,12 +24056,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24112,17 +24092,17 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E91" s="26" t="inlineStr">
@@ -24137,7 +24117,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24148,17 +24128,17 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E92" s="26" t="inlineStr">
@@ -24173,7 +24153,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24184,17 +24164,17 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E93" s="26" t="inlineStr">
@@ -24209,7 +24189,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24220,17 +24200,17 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E94" s="26" t="inlineStr">
@@ -24245,7 +24225,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24256,17 +24236,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E95" s="26" t="inlineStr">
@@ -24281,7 +24261,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24292,12 +24272,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24317,7 +24297,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24328,17 +24308,17 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E97" s="26" t="inlineStr">
@@ -24353,7 +24333,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24364,12 +24344,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24389,7 +24369,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24400,12 +24380,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24425,7 +24405,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24436,12 +24416,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24461,7 +24441,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24472,12 +24452,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24497,7 +24477,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24508,17 +24488,17 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E102" s="26" t="inlineStr">
@@ -24533,7 +24513,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24544,17 +24524,17 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E103" s="26" t="inlineStr">
@@ -24569,7 +24549,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24580,17 +24560,17 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E104" s="26" t="inlineStr">
@@ -24605,7 +24585,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24616,17 +24596,17 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E105" s="26" t="inlineStr">
@@ -24641,7 +24621,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24652,12 +24632,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24677,7 +24657,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24688,12 +24668,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24713,7 +24693,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24724,17 +24704,17 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E108" s="26" t="inlineStr">
@@ -24749,7 +24729,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24760,17 +24740,17 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E109" s="26" t="inlineStr">
@@ -24785,7 +24765,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24796,12 +24776,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24821,7 +24801,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24832,12 +24812,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24857,7 +24837,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24868,17 +24848,17 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E112" s="26" t="inlineStr">
@@ -24888,12 +24868,12 @@
       </c>
       <c r="F112" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24904,17 +24884,17 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E113" s="26" t="inlineStr">
@@ -24924,12 +24904,12 @@
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24940,12 +24920,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24960,12 +24940,12 @@
       </c>
       <c r="F114" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24976,17 +24956,17 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E115" s="26" t="inlineStr">
@@ -24996,12 +24976,12 @@
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25012,12 +24992,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25032,12 +25012,12 @@
       </c>
       <c r="F116" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25048,12 +25028,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25068,12 +25048,12 @@
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25084,17 +25064,17 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E118" s="26" t="inlineStr">
@@ -25109,7 +25089,7 @@
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25120,17 +25100,17 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E119" s="26" t="inlineStr">
@@ -25145,7 +25125,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25156,12 +25136,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25181,7 +25161,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25192,17 +25172,17 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E121" s="26" t="inlineStr">
@@ -25217,7 +25197,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25228,12 +25208,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25253,7 +25233,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25264,12 +25244,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25289,7 +25269,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25300,17 +25280,17 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E124" s="26" t="inlineStr">
@@ -25325,7 +25305,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25336,17 +25316,17 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E125" s="26" t="inlineStr">
@@ -25361,7 +25341,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25372,12 +25352,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25397,7 +25377,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25408,12 +25388,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25433,7 +25413,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25444,12 +25424,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25469,7 +25449,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25480,12 +25460,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25505,7 +25485,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25516,12 +25496,12 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -25536,12 +25516,12 @@
       </c>
       <c r="F130" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25552,12 +25532,12 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -25572,12 +25552,12 @@
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25588,12 +25568,12 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -25608,12 +25588,12 @@
       </c>
       <c r="F132" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25624,12 +25604,12 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -25644,12 +25624,12 @@
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25660,12 +25640,12 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -25685,7 +25665,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25696,12 +25676,12 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -25721,7 +25701,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25732,12 +25712,12 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
@@ -25752,12 +25732,12 @@
       </c>
       <c r="F136" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25768,38 +25748,254 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+        </is>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E137" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F137" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+        </is>
+      </c>
+      <c r="H137" s="5" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="12" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="23" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="inlineStr">
+        <is>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+        </is>
+      </c>
+      <c r="D138" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E138" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G138" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+        </is>
+      </c>
+      <c r="H138" s="13" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="25" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+        </is>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E139" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F139" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+        </is>
+      </c>
+      <c r="H139" s="5" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="23" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E140" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G140" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H140" s="13" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="25" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D141" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E141" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F141" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H141" s="5" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="23" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E142" s="26" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G142" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H142" s="13" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C137" s="5" t="inlineStr">
+      <c r="C143" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D143" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E137" s="26" t="inlineStr">
+      <c r="E143" s="26" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F137" s="16" t="inlineStr">
+      <c r="F143" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G137" s="5" t="inlineStr">
+      <c r="G143" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H137" s="5" t="inlineStr"/>
+      <c r="H143" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H137"/>
+  <autoFilter ref="A1:H143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T146, T147, T148, T149: sơ đồ danh mục 7 làn đánh số, danh mục theo thông tư, chọn cột mọi danh mục, lịch chọn ngày
- T146: sơ đồ Khởi tạo danh mục kiểu làn, đánh số theo thứ tự thiết lập; danh mục TSCĐ 1.13 chuyển sang phân hệ TSCĐ
- T147: ScreenDef.cheDo, hienMan lọc theo thông tư; TT152, TT58 ẩn tài khoản, bút toán tự động, cột và ô TK
- T148: bỏ Thuộc nhóm; ô tích Tổng hợp ở tài khoản; Table chỉ ép minWidth khi cuộn ảo (hết giật cột); useCotDs + NutTuyChinhCot cho mọi danh mục, cột bổ sung từ trường form
- T149: ONgay dùng chung trong ChonNgay.tsx cho mọi ô một ngày
- QD48, nhật ký, CHANGELOG, báo cáo hệ thống

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,11 +80,17 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -141,6 +147,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
@@ -172,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -231,6 +243,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -829,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>142 việc (T01 - T108)</t>
+          <t>151 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -846,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>118 việc (83.1%)</t>
+          <t>127 việc (84.1%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -880,7 +895,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>24 việc</t>
+          <t>22 việc</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -21011,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21087,14 +21102,14 @@
       </c>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Đã đề xuất luồng, chờ PhuongXT chốt 3 điểm, xem `2026-10-10-phuongxt-y-tuong-onboard-fabi.md`</t>
+          <t>Popup khởi tạo dữ liệu 4 bước trong phần mềm (`OnboardFabi.tsx`, `Shell.tsx`) đã push, PhuongXT xem lại một lượt. Xem `2026-10-11-phuongxt-man-khoi-tao-fabi.md`</t>
         </is>
       </c>
     </row>
@@ -21113,7 +21128,7 @@
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr"/>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21141,7 +21156,7 @@
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21169,7 +21184,7 @@
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21197,7 +21212,7 @@
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21225,7 +21240,7 @@
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21257,7 +21272,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21291,14 +21306,14 @@
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>Chờ</t>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T25</t>
+          <t>11/10/2026 PhuongXT chốt gói Free không giới hạn chi nhánh (làm cùng T138): đã sửa mô tả gói Free, điểm nổi bật, câu hỏi đáp màn Gói thuê bao. Gói Standard còn ghi "1 điểm bán", chưa chốt</t>
         </is>
       </c>
     </row>
@@ -21321,7 +21336,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21345,7 +21360,7 @@
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr"/>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21373,7 +21388,7 @@
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21401,7 +21416,7 @@
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21429,7 +21444,7 @@
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21457,7 +21472,7 @@
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21481,7 +21496,7 @@
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21509,7 +21524,7 @@
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21537,7 +21552,7 @@
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21565,7 +21580,7 @@
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21593,7 +21608,7 @@
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21621,7 +21636,7 @@
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21649,7 +21664,7 @@
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21677,7 +21692,7 @@
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr"/>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21705,7 +21720,7 @@
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21733,7 +21748,7 @@
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21752,12 +21767,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21765,7 +21780,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E26" s="26" t="inlineStr">
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21777,7 +21792,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21788,12 +21803,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21801,7 +21816,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E27" s="26" t="inlineStr">
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21813,7 +21828,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21824,20 +21839,20 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
-        </is>
-      </c>
-      <c r="E28" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21849,7 +21864,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21860,12 +21875,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21873,7 +21888,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E29" s="26" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21885,7 +21900,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21896,32 +21911,32 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E30" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21932,12 +21947,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21945,19 +21960,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E31" s="26" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21968,12 +21983,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -21981,19 +21996,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E32" s="26" t="inlineStr">
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22004,12 +22019,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22017,19 +22032,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E33" s="26" t="inlineStr">
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22040,12 +22055,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22053,19 +22068,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E34" s="26" t="inlineStr">
+      <c r="E34" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22076,32 +22091,32 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E35" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22112,32 +22127,32 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E36" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22148,32 +22163,32 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E37" s="26" t="inlineStr">
+          <t>dinhlanphuongipacc</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22184,32 +22199,32 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E38" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E38" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22220,20 +22235,20 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E39" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22245,7 +22260,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22256,12 +22271,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22269,7 +22284,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E40" s="26" t="inlineStr">
+      <c r="E40" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22281,7 +22296,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22292,20 +22307,20 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E41" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22317,7 +22332,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22328,12 +22343,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22341,7 +22356,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E42" s="26" t="inlineStr">
+      <c r="E42" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22353,7 +22368,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22364,20 +22379,20 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E43" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22389,7 +22404,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22400,20 +22415,20 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E44" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E44" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22425,7 +22440,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22436,12 +22451,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22449,7 +22464,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E45" s="26" t="inlineStr">
+      <c r="E45" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22461,7 +22476,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22472,12 +22487,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22485,7 +22500,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E46" s="26" t="inlineStr">
+      <c r="E46" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22497,7 +22512,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22508,12 +22523,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22521,7 +22536,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E47" s="26" t="inlineStr">
+      <c r="E47" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22533,7 +22548,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22544,12 +22559,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22557,7 +22572,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E48" s="26" t="inlineStr">
+      <c r="E48" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22569,7 +22584,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22580,12 +22595,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22593,7 +22608,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E49" s="26" t="inlineStr">
+      <c r="E49" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22605,7 +22620,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22616,20 +22631,20 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E50" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22641,7 +22656,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22652,20 +22667,20 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E51" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22677,7 +22692,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22688,12 +22703,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22701,7 +22716,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E52" s="26" t="inlineStr">
+      <c r="E52" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22713,7 +22728,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22724,20 +22739,20 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
-        </is>
-      </c>
-      <c r="E53" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22749,7 +22764,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22760,12 +22775,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22773,7 +22788,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E54" s="26" t="inlineStr">
+      <c r="E54" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22785,7 +22800,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22796,12 +22811,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22809,7 +22824,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E55" s="26" t="inlineStr">
+      <c r="E55" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22821,7 +22836,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22832,12 +22847,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22845,7 +22860,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E56" s="26" t="inlineStr">
+      <c r="E56" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22857,7 +22872,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22868,12 +22883,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22881,7 +22896,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E57" s="26" t="inlineStr">
+      <c r="E57" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22893,7 +22908,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22904,12 +22919,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22917,7 +22932,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E58" s="26" t="inlineStr">
+      <c r="E58" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22929,7 +22944,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22940,12 +22955,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22953,7 +22968,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E59" s="26" t="inlineStr">
+      <c r="E59" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22965,7 +22980,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -22976,20 +22991,20 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E60" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E60" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23001,7 +23016,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23012,20 +23027,20 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E61" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23037,7 +23052,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23048,20 +23063,20 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E62" s="26" t="inlineStr">
+          <t>dinhlanphuongipacc</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23073,7 +23088,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23084,12 +23099,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23097,7 +23112,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E63" s="26" t="inlineStr">
+      <c r="E63" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23109,7 +23124,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23120,12 +23135,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23133,7 +23148,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E64" s="26" t="inlineStr">
+      <c r="E64" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23145,7 +23160,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23156,12 +23171,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23169,7 +23184,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E65" s="26" t="inlineStr">
+      <c r="E65" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23181,7 +23196,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23192,12 +23207,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23205,7 +23220,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E66" s="26" t="inlineStr">
+      <c r="E66" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23217,7 +23232,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23228,12 +23243,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23241,7 +23256,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E67" s="26" t="inlineStr">
+      <c r="E67" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23253,7 +23268,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23264,12 +23279,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23277,7 +23292,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E68" s="26" t="inlineStr">
+      <c r="E68" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23289,7 +23304,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23300,12 +23315,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23313,7 +23328,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E69" s="26" t="inlineStr">
+      <c r="E69" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23325,7 +23340,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23336,12 +23351,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23349,7 +23364,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E70" s="26" t="inlineStr">
+      <c r="E70" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23361,7 +23376,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23372,12 +23387,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23385,7 +23400,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E71" s="26" t="inlineStr">
+      <c r="E71" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23397,7 +23412,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23408,20 +23423,20 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E72" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E72" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23433,7 +23448,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23444,20 +23459,20 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E73" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E73" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23469,7 +23484,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23480,20 +23495,20 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E74" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23505,7 +23520,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23516,12 +23531,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23529,7 +23544,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E75" s="26" t="inlineStr">
+      <c r="E75" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23541,7 +23556,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23552,12 +23567,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23565,7 +23580,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E76" s="26" t="inlineStr">
+      <c r="E76" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23577,7 +23592,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23588,12 +23603,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23601,7 +23616,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E77" s="26" t="inlineStr">
+      <c r="E77" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23613,7 +23628,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23624,12 +23639,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23637,7 +23652,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E78" s="26" t="inlineStr">
+      <c r="E78" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23649,7 +23664,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23660,12 +23675,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23673,7 +23688,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E79" s="26" t="inlineStr">
+      <c r="E79" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23685,7 +23700,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23696,20 +23711,20 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E80" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E80" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23721,7 +23736,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23732,12 +23747,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23745,7 +23760,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E81" s="26" t="inlineStr">
+      <c r="E81" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23757,7 +23772,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23768,12 +23783,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23781,7 +23796,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E82" s="26" t="inlineStr">
+      <c r="E82" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23793,7 +23808,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23804,12 +23819,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23817,7 +23832,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E83" s="26" t="inlineStr">
+      <c r="E83" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23829,7 +23844,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23840,20 +23855,20 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E84" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E84" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23865,7 +23880,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23876,12 +23891,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23889,19 +23904,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E85" s="26" t="inlineStr">
+      <c r="E85" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23912,12 +23927,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23925,19 +23940,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E86" s="26" t="inlineStr">
+      <c r="E86" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F86" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23948,12 +23963,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23961,19 +23976,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E87" s="26" t="inlineStr">
+      <c r="E87" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -23984,12 +23999,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -23997,19 +24012,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E88" s="26" t="inlineStr">
+      <c r="E88" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24020,32 +24035,32 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E89" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E89" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24056,12 +24071,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24069,19 +24084,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E90" s="26" t="inlineStr">
+      <c r="E90" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F90" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24092,12 +24107,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24105,19 +24120,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E91" s="26" t="inlineStr">
+      <c r="E91" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24128,12 +24143,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24141,19 +24156,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E92" s="26" t="inlineStr">
+      <c r="E92" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F92" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24164,12 +24179,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24177,19 +24192,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E93" s="26" t="inlineStr">
+      <c r="E93" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24200,20 +24215,20 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E94" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E94" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24225,7 +24240,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24236,20 +24251,20 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E95" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E95" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24261,7 +24276,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24272,20 +24287,20 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E96" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E96" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24297,7 +24312,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24308,12 +24323,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24321,7 +24336,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E97" s="26" t="inlineStr">
+      <c r="E97" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24333,7 +24348,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24344,20 +24359,20 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E98" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E98" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24369,7 +24384,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24380,20 +24395,20 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E99" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E99" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24405,7 +24420,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24416,20 +24431,20 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E100" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E100" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24441,7 +24456,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24452,20 +24467,20 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E101" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E101" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24477,7 +24492,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24488,12 +24503,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24501,7 +24516,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E102" s="26" t="inlineStr">
+      <c r="E102" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24513,7 +24528,7 @@
       </c>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H102" s="13" t="inlineStr"/>
@@ -24524,12 +24539,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24537,7 +24552,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E103" s="26" t="inlineStr">
+      <c r="E103" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24549,7 +24564,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -24560,20 +24575,20 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E104" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E104" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24585,7 +24600,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -24596,20 +24611,20 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E105" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E105" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24621,7 +24636,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -24632,12 +24647,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24645,7 +24660,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E106" s="26" t="inlineStr">
+      <c r="E106" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24657,7 +24672,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24668,12 +24683,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24681,7 +24696,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E107" s="26" t="inlineStr">
+      <c r="E107" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24693,7 +24708,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24704,12 +24719,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24717,7 +24732,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E108" s="26" t="inlineStr">
+      <c r="E108" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24729,7 +24744,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24740,12 +24755,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24753,7 +24768,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E109" s="26" t="inlineStr">
+      <c r="E109" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24765,7 +24780,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24776,20 +24791,20 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E110" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E110" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24801,7 +24816,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -24812,12 +24827,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24825,7 +24840,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E111" s="26" t="inlineStr">
+      <c r="E111" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24837,7 +24852,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24848,20 +24863,20 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E112" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E112" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24873,7 +24888,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24884,12 +24899,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24897,7 +24912,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E113" s="26" t="inlineStr">
+      <c r="E113" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24920,20 +24935,20 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E114" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E114" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24945,7 +24960,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24956,20 +24971,20 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E115" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E115" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24981,7 +24996,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -24992,20 +25007,20 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E116" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E116" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25017,7 +25032,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25028,20 +25043,20 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E117" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E117" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25053,7 +25068,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25064,32 +25079,32 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E118" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E118" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F118" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25100,12 +25115,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25113,19 +25128,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E119" s="26" t="inlineStr">
+      <c r="E119" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25136,12 +25151,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25149,19 +25164,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E120" s="26" t="inlineStr">
+      <c r="E120" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25172,12 +25187,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25185,19 +25200,19 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E121" s="26" t="inlineStr">
+      <c r="E121" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25208,32 +25223,32 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E122" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E122" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F122" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25244,12 +25259,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25257,19 +25272,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E123" s="26" t="inlineStr">
+      <c r="E123" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F123" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25280,32 +25295,32 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E124" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E124" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F124" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25316,32 +25331,32 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E125" s="26" t="inlineStr">
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E125" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25352,12 +25367,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25365,19 +25380,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E126" s="26" t="inlineStr">
+      <c r="E126" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F126" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25388,12 +25403,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25401,7 +25416,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E127" s="26" t="inlineStr">
+      <c r="E127" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25413,7 +25428,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25424,12 +25439,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25437,7 +25452,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E128" s="26" t="inlineStr">
+      <c r="E128" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25449,7 +25464,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25460,12 +25475,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25473,7 +25488,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E129" s="26" t="inlineStr">
+      <c r="E129" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25485,7 +25500,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25496,20 +25511,20 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E130" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E130" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25521,7 +25536,7 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25532,12 +25547,12 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -25545,7 +25560,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E131" s="26" t="inlineStr">
+      <c r="E131" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25557,7 +25572,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25568,12 +25583,12 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -25581,7 +25596,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E132" s="26" t="inlineStr">
+      <c r="E132" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25593,7 +25608,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25604,20 +25619,20 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E133" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E133" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25629,7 +25644,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25640,20 +25655,20 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E134" s="26" t="inlineStr">
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E134" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25665,7 +25680,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25676,12 +25691,12 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -25689,7 +25704,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E135" s="26" t="inlineStr">
+      <c r="E135" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25701,7 +25716,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25712,12 +25727,12 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
@@ -25725,19 +25740,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E136" s="26" t="inlineStr">
+      <c r="E136" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F136" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25748,12 +25763,12 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -25761,19 +25776,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E137" s="26" t="inlineStr">
+      <c r="E137" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -25784,12 +25799,12 @@
       </c>
       <c r="B138" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
@@ -25797,19 +25812,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E138" s="26" t="inlineStr">
+      <c r="E138" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F138" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -25820,12 +25835,12 @@
       </c>
       <c r="B139" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -25833,19 +25848,19 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E139" s="26" t="inlineStr">
+      <c r="E139" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
       <c r="F139" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -25856,12 +25871,12 @@
       </c>
       <c r="B140" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -25869,7 +25884,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E140" s="26" t="inlineStr">
+      <c r="E140" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25881,7 +25896,7 @@
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr"/>
@@ -25892,12 +25907,12 @@
       </c>
       <c r="B141" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -25905,7 +25920,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E141" s="26" t="inlineStr">
+      <c r="E141" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25917,7 +25932,7 @@
       </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
@@ -25928,12 +25943,12 @@
       </c>
       <c r="B142" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -25941,7 +25956,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E142" s="26" t="inlineStr">
+      <c r="E142" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25953,7 +25968,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -25964,38 +25979,362 @@
       </c>
       <c r="B143" s="25" t="inlineStr">
         <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+        </is>
+      </c>
+      <c r="D143" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E143" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F143" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="23" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="inlineStr">
+        <is>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+        </is>
+      </c>
+      <c r="D144" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E144" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G144" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+        </is>
+      </c>
+      <c r="H144" s="13" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="25" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+        </is>
+      </c>
+      <c r="D145" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E145" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F145" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-khung-web.md`</t>
+        </is>
+      </c>
+      <c r="H145" s="5" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="23" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+        </is>
+      </c>
+      <c r="D146" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E146" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G146" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+        </is>
+      </c>
+      <c r="H146" s="13" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="25" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+        </is>
+      </c>
+      <c r="D147" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E147" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+        </is>
+      </c>
+      <c r="H147" s="5" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="23" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="inlineStr">
+        <is>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+        </is>
+      </c>
+      <c r="D148" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E148" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G148" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+        </is>
+      </c>
+      <c r="H148" s="13" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="16" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="25" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+        </is>
+      </c>
+      <c r="D149" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E149" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H149" s="5" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="23" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="inlineStr">
+        <is>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+        </is>
+      </c>
+      <c r="D150" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E150" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G150" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H150" s="13" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="25" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D151" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E151" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F151" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H151" s="5" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="23" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C143" s="5" t="inlineStr">
+      <c r="C152" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D143" s="16" t="inlineStr">
+      <c r="D152" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E143" s="26" t="inlineStr">
+      <c r="E152" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F143" s="16" t="inlineStr">
+      <c r="F152" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G143" s="5" t="inlineStr">
+      <c r="G152" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H143" s="5" t="inlineStr"/>
+      <c r="H152" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H143"/>
+  <autoFilter ref="A1:H152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T150: danh mục vừa một trang, bảng cuộn trong khung, chân phân trang 50-1000 dòng như danh sách chứng từ
- CatalogScreen, Chi nhánh: khung page-voucher + dm-bang, phân trang mặc định 50 (CO_TRANG_DM), về trang 1 khi đổi danh mục, tìm, lọc
- Hệ thống tài khoản: cùng khung, không phân trang, chân đếm số tài khoản
- PhanTrang nhận dsCoTrang, danh sách chứng từ giữ 20, 50, 100
- BAY: không mượn class voucher-top cho khung không phải chứng từ

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -844,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>151 việc (T01 - T108)</t>
+          <t>152 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>127 việc (84.1%)</t>
+          <t>128 việc (84.2%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21026,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21767,12 +21767,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21803,12 +21803,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21839,12 +21839,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21875,12 +21875,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21911,17 +21911,17 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
@@ -21936,7 +21936,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -21947,12 +21947,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21972,7 +21972,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21983,12 +21983,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22008,7 +22008,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22019,12 +22019,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22055,12 +22055,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22080,7 +22080,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22091,17 +22091,17 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22127,12 +22127,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22163,17 +22163,17 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E37" s="27" t="inlineStr">
@@ -22188,7 +22188,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22199,17 +22199,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22235,12 +22235,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22255,12 +22255,12 @@
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22271,17 +22271,17 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22307,12 +22307,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22332,7 +22332,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22343,12 +22343,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22368,7 +22368,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22379,12 +22379,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22415,12 +22415,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22451,12 +22451,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22487,12 +22487,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22523,12 +22523,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22559,12 +22559,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22595,12 +22595,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22620,7 +22620,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22631,17 +22631,17 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E50" s="27" t="inlineStr">
@@ -22656,7 +22656,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22667,17 +22667,17 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22703,17 +22703,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E52" s="27" t="inlineStr">
@@ -22728,7 +22728,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22739,12 +22739,12 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -22775,17 +22775,17 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E54" s="27" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22811,12 +22811,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22847,12 +22847,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22883,12 +22883,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22919,12 +22919,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22955,12 +22955,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22991,17 +22991,17 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E60" s="27" t="inlineStr">
@@ -23016,7 +23016,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23027,12 +23027,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23063,17 +23063,17 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23099,17 +23099,17 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E63" s="27" t="inlineStr">
@@ -23124,7 +23124,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23135,12 +23135,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23171,12 +23171,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23207,12 +23207,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23243,12 +23243,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23279,12 +23279,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23304,7 +23304,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23315,12 +23315,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23351,12 +23351,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23387,17 +23387,17 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E71" s="27" t="inlineStr">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23423,17 +23423,17 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr">
@@ -23448,7 +23448,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23459,12 +23459,12 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -23495,12 +23495,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23531,12 +23531,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23567,12 +23567,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23603,12 +23603,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23639,12 +23639,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23664,7 +23664,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23675,12 +23675,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23711,17 +23711,17 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E80" s="27" t="inlineStr">
@@ -23736,7 +23736,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23747,12 +23747,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23772,7 +23772,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23783,12 +23783,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23819,12 +23819,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23855,17 +23855,17 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E84" s="27" t="inlineStr">
@@ -23880,7 +23880,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23891,12 +23891,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23927,12 +23927,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23963,12 +23963,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -23999,12 +23999,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24035,12 +24035,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24071,17 +24071,17 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E90" s="27" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24107,12 +24107,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24143,12 +24143,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24179,12 +24179,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24215,17 +24215,17 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E94" s="27" t="inlineStr">
@@ -24235,12 +24235,12 @@
       </c>
       <c r="F94" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24251,12 +24251,12 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -24276,7 +24276,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24287,12 +24287,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24323,12 +24323,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24359,17 +24359,17 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E98" s="27" t="inlineStr">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24395,12 +24395,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24431,12 +24431,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24467,12 +24467,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24503,12 +24503,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24539,12 +24539,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24575,12 +24575,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24611,12 +24611,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24647,17 +24647,17 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E106" s="27" t="inlineStr">
@@ -24672,7 +24672,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -24683,12 +24683,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24719,12 +24719,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24755,12 +24755,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24791,12 +24791,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24827,17 +24827,17 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E111" s="27" t="inlineStr">
@@ -24852,7 +24852,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -24863,12 +24863,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24888,7 +24888,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24899,17 +24899,17 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E113" s="27" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24935,12 +24935,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24971,12 +24971,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25007,12 +25007,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25043,12 +25043,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25068,7 +25068,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25104,7 +25104,7 @@
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25115,17 +25115,17 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E119" s="27" t="inlineStr">
@@ -25140,7 +25140,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25151,12 +25151,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25187,17 +25187,17 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E121" s="27" t="inlineStr">
@@ -25212,7 +25212,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25223,12 +25223,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25248,7 +25248,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25259,17 +25259,17 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E123" s="27" t="inlineStr">
@@ -25284,7 +25284,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25295,12 +25295,12 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25331,12 +25331,12 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25356,7 +25356,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25367,12 +25367,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25392,7 +25392,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25403,12 +25403,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25423,12 +25423,12 @@
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25439,12 +25439,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25475,12 +25475,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25511,17 +25511,17 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E130" s="27" t="inlineStr">
@@ -25536,7 +25536,7 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25547,17 +25547,17 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E131" s="27" t="inlineStr">
@@ -25572,7 +25572,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25583,12 +25583,12 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -25608,7 +25608,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25619,17 +25619,17 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E133" s="27" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25655,12 +25655,12 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -25680,7 +25680,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25691,17 +25691,17 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E135" s="27" t="inlineStr">
@@ -25716,7 +25716,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25727,12 +25727,12 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
@@ -25752,7 +25752,7 @@
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25763,12 +25763,12 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -25799,12 +25799,12 @@
       </c>
       <c r="B138" s="23" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
@@ -25824,7 +25824,7 @@
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -25835,12 +25835,12 @@
       </c>
       <c r="B139" s="25" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -25860,7 +25860,7 @@
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -25871,12 +25871,12 @@
       </c>
       <c r="B140" s="23" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -25896,7 +25896,7 @@
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr"/>
@@ -25907,12 +25907,12 @@
       </c>
       <c r="B141" s="25" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -25932,7 +25932,7 @@
       </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
@@ -25943,12 +25943,12 @@
       </c>
       <c r="B142" s="23" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -25968,7 +25968,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -25979,12 +25979,12 @@
       </c>
       <c r="B143" s="25" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26015,12 +26015,12 @@
       </c>
       <c r="B144" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
@@ -26040,7 +26040,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26051,12 +26051,12 @@
       </c>
       <c r="B145" s="25" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
@@ -26071,12 +26071,12 @@
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26087,12 +26087,12 @@
       </c>
       <c r="B146" s="23" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26123,12 +26123,12 @@
       </c>
       <c r="B147" s="25" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26159,12 +26159,12 @@
       </c>
       <c r="B148" s="23" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
@@ -26184,7 +26184,7 @@
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26195,12 +26195,12 @@
       </c>
       <c r="B149" s="25" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
@@ -26215,12 +26215,12 @@
       </c>
       <c r="F149" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26231,12 +26231,12 @@
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26267,12 +26267,12 @@
       </c>
       <c r="B151" s="25" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26303,38 +26303,74 @@
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C152" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D152" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E152" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F152" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G152" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H152" s="13" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="16" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C152" s="13" t="inlineStr">
+      <c r="C153" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D152" s="12" t="inlineStr">
+      <c r="D153" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E152" s="27" t="inlineStr">
+      <c r="E153" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F152" s="12" t="inlineStr">
+      <c r="F153" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G152" s="13" t="inlineStr">
+      <c r="G153" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H152" s="13" t="inlineStr"/>
+      <c r="H153" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H152"/>
+  <autoFilter ref="A1:H153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T151: hàng hoá theo iFaster: thuế theo 37 ngành nghề (TT152, TT58), thương hiệu, kho theo dõi, nhà cung cấp, quy đổi ĐVT có hộp thêm sửa
- nganh-nghe.ts: 4 nhóm, 37 ngành nghề con, % GTGT, TNCN chép từ iFaster
- Form hàng hoá, nhóm hàng: ngành nghề con tự điền nhóm, tỷ lệ; TT133, TT99 giữ thuế suất GTGT
- Danh mục Thương hiệu; thương hiệu trên hàng hoá, kho
- QuyDoiDvt.tsx: bảng và hộp quy đổi ĐVT trong form hàng hoá
- QD49, nhật ký, CHANGELOG, báo cáo hệ thống

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$154</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -844,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>152 việc (T01 - T108)</t>
+          <t>153 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>128 việc (84.2%)</t>
+          <t>129 việc (84.3%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21026,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21767,12 +21767,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T150</t>
+          <t>T151</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
+          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
+          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21803,12 +21803,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21828,7 +21828,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21839,12 +21839,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21875,12 +21875,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21911,12 +21911,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21947,17 +21947,17 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E31" s="27" t="inlineStr">
@@ -21972,7 +21972,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -21983,12 +21983,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22008,7 +22008,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22019,12 +22019,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22055,12 +22055,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22080,7 +22080,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22091,12 +22091,12 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22127,17 +22127,17 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
@@ -22152,7 +22152,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22163,12 +22163,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22199,17 +22199,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22235,17 +22235,17 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
@@ -22260,7 +22260,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22271,12 +22271,12 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22291,12 +22291,12 @@
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22307,17 +22307,17 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr">
@@ -22332,7 +22332,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22343,12 +22343,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22368,7 +22368,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22379,12 +22379,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22415,12 +22415,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22451,12 +22451,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22487,12 +22487,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22523,12 +22523,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22559,12 +22559,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22595,12 +22595,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22620,7 +22620,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22631,12 +22631,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22656,7 +22656,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22667,17 +22667,17 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22703,17 +22703,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E52" s="27" t="inlineStr">
@@ -22728,7 +22728,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22739,17 +22739,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22775,12 +22775,12 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -22811,17 +22811,17 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22847,12 +22847,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22872,7 +22872,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22883,12 +22883,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22919,12 +22919,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22955,12 +22955,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22991,12 +22991,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23027,17 +23027,17 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E61" s="27" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23063,12 +23063,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23099,17 +23099,17 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E63" s="27" t="inlineStr">
@@ -23124,7 +23124,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23135,17 +23135,17 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr">
@@ -23160,7 +23160,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23171,12 +23171,12 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23207,12 +23207,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23243,12 +23243,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23279,12 +23279,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23315,12 +23315,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23340,7 +23340,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23351,12 +23351,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23387,12 +23387,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23423,17 +23423,17 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr">
@@ -23448,7 +23448,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23459,17 +23459,17 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E73" s="27" t="inlineStr">
@@ -23484,7 +23484,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23495,12 +23495,12 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -23531,12 +23531,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23567,12 +23567,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23592,7 +23592,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -23603,12 +23603,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23639,12 +23639,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23675,12 +23675,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23700,7 +23700,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -23711,12 +23711,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23747,17 +23747,17 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E81" s="27" t="inlineStr">
@@ -23772,7 +23772,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23783,12 +23783,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23808,7 +23808,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23819,12 +23819,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23855,12 +23855,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23891,17 +23891,17 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E85" s="27" t="inlineStr">
@@ -23916,7 +23916,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -23927,12 +23927,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23963,12 +23963,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -23999,12 +23999,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24035,12 +24035,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24071,12 +24071,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24107,17 +24107,17 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E91" s="27" t="inlineStr">
@@ -24132,7 +24132,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr"/>
@@ -24143,12 +24143,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24179,12 +24179,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24215,12 +24215,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24251,17 +24251,17 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E95" s="27" t="inlineStr">
@@ -24271,12 +24271,12 @@
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H95" s="5" t="inlineStr"/>
@@ -24287,12 +24287,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24323,12 +24323,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24348,7 +24348,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24359,12 +24359,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24395,17 +24395,17 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E99" s="27" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24431,12 +24431,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24467,12 +24467,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24503,12 +24503,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24539,12 +24539,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24575,12 +24575,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24611,12 +24611,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24647,12 +24647,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24683,17 +24683,17 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E107" s="27" t="inlineStr">
@@ -24708,7 +24708,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -24719,12 +24719,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24755,12 +24755,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24791,12 +24791,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24827,12 +24827,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24863,17 +24863,17 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E112" s="27" t="inlineStr">
@@ -24888,7 +24888,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -24899,12 +24899,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24935,17 +24935,17 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E114" s="27" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24971,12 +24971,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -24996,7 +24996,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25007,12 +25007,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25043,12 +25043,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25079,12 +25079,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25104,7 +25104,7 @@
       </c>
       <c r="G118" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr"/>
@@ -25115,12 +25115,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25140,7 +25140,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25151,17 +25151,17 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E120" s="27" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25187,12 +25187,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25212,7 +25212,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25223,17 +25223,17 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E122" s="27" t="inlineStr">
@@ -25248,7 +25248,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25259,12 +25259,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25284,7 +25284,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25295,17 +25295,17 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E124" s="27" t="inlineStr">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25331,12 +25331,12 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25356,7 +25356,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25367,12 +25367,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25392,7 +25392,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25403,12 +25403,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25439,12 +25439,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25459,12 +25459,12 @@
       </c>
       <c r="F128" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25475,12 +25475,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25511,12 +25511,12 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -25536,7 +25536,7 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25547,17 +25547,17 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E131" s="27" t="inlineStr">
@@ -25572,7 +25572,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25583,17 +25583,17 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E132" s="27" t="inlineStr">
@@ -25608,7 +25608,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25619,12 +25619,12 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25655,17 +25655,17 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E134" s="27" t="inlineStr">
@@ -25680,7 +25680,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25691,12 +25691,12 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -25716,7 +25716,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25727,17 +25727,17 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E136" s="27" t="inlineStr">
@@ -25752,7 +25752,7 @@
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25763,12 +25763,12 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -25788,7 +25788,7 @@
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -25799,12 +25799,12 @@
       </c>
       <c r="B138" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
@@ -25835,12 +25835,12 @@
       </c>
       <c r="B139" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -25860,7 +25860,7 @@
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -25871,12 +25871,12 @@
       </c>
       <c r="B140" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -25896,7 +25896,7 @@
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr"/>
@@ -25907,12 +25907,12 @@
       </c>
       <c r="B141" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -25932,7 +25932,7 @@
       </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
@@ -25943,12 +25943,12 @@
       </c>
       <c r="B142" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -25968,7 +25968,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -25979,12 +25979,12 @@
       </c>
       <c r="B143" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26015,12 +26015,12 @@
       </c>
       <c r="B144" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
@@ -26040,7 +26040,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26051,12 +26051,12 @@
       </c>
       <c r="B145" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
@@ -26076,7 +26076,7 @@
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26087,12 +26087,12 @@
       </c>
       <c r="B146" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
@@ -26107,12 +26107,12 @@
       </c>
       <c r="F146" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26123,12 +26123,12 @@
       </c>
       <c r="B147" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26159,12 +26159,12 @@
       </c>
       <c r="B148" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
@@ -26184,7 +26184,7 @@
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26195,12 +26195,12 @@
       </c>
       <c r="B149" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
@@ -26220,7 +26220,7 @@
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26231,12 +26231,12 @@
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26251,12 +26251,12 @@
       </c>
       <c r="F150" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr"/>
@@ -26267,12 +26267,12 @@
       </c>
       <c r="B151" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26303,12 +26303,12 @@
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D152" s="12" t="inlineStr">
@@ -26339,38 +26339,74 @@
       </c>
       <c r="B153" s="25" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D153" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E153" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F153" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H153" s="5" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="23" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C153" s="5" t="inlineStr">
+      <c r="C154" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D153" s="16" t="inlineStr">
+      <c r="D154" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E153" s="27" t="inlineStr">
+      <c r="E154" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F153" s="16" t="inlineStr">
+      <c r="F154" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G153" s="5" t="inlineStr">
+      <c r="G154" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H153" s="5" t="inlineStr"/>
+      <c r="H154" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H153"/>
+  <autoFilter ref="A1:H154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T152: sản xuất ở Kho theo iPOS Inventory: 4 tab xuất, nhập sơ chế, chế biến; công thức sơ chế, chế biến làm lại
- 5.1.6, 5.1.6-2, 5.1.3, 5.1.3-2: chip Chờ nhập, Đã nhập, Đã huỷ; phiếu nhập tham chiếu phiếu xuất; Kế hoạch, Thực tế; hạch toán qua 154; chưa có số lô
- ChungTuForm nhánh sanXuat, BangSanXuat, PhieuSanXuat, CongThuc, san-xuat.ts
- QD50, nhật ký, CHANGELOG, báo cáo hệ thống

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$155</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -844,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>153 việc (T01 - T108)</t>
+          <t>154 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>129 việc (84.3%)</t>
+          <t>130 việc (84.4%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21026,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H154"/>
+  <dimension ref="A1:H155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21767,12 +21767,12 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T151</t>
+          <t>T152</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
+          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
+          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21803,12 +21803,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T150</t>
+          <t>T151</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
+          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21828,7 +21828,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
+          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21839,12 +21839,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21864,7 +21864,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21875,12 +21875,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21911,12 +21911,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21947,12 +21947,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21983,17 +21983,17 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
@@ -22008,7 +22008,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22019,12 +22019,12 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22055,12 +22055,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22080,7 +22080,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22091,12 +22091,12 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22127,12 +22127,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22152,7 +22152,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22163,17 +22163,17 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E37" s="27" t="inlineStr">
@@ -22188,7 +22188,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22199,12 +22199,12 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22235,17 +22235,17 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
@@ -22260,7 +22260,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22271,17 +22271,17 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22307,12 +22307,12 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22327,12 +22327,12 @@
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22343,17 +22343,17 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E42" s="27" t="inlineStr">
@@ -22368,7 +22368,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22379,12 +22379,12 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22415,12 +22415,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22451,12 +22451,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22487,12 +22487,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22523,12 +22523,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22559,12 +22559,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22595,12 +22595,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22620,7 +22620,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22631,12 +22631,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22656,7 +22656,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22667,12 +22667,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22703,17 +22703,17 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E52" s="27" t="inlineStr">
@@ -22728,7 +22728,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22739,17 +22739,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22775,17 +22775,17 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E54" s="27" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22811,12 +22811,12 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -22847,17 +22847,17 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E56" s="27" t="inlineStr">
@@ -22872,7 +22872,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -22883,12 +22883,12 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -22908,7 +22908,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22919,12 +22919,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22955,12 +22955,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22991,12 +22991,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23027,12 +23027,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23063,17 +23063,17 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23099,12 +23099,12 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -23124,7 +23124,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23135,17 +23135,17 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr">
@@ -23160,7 +23160,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23171,17 +23171,17 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E65" s="27" t="inlineStr">
@@ -23196,7 +23196,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23207,12 +23207,12 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23243,12 +23243,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23279,12 +23279,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23315,12 +23315,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23351,12 +23351,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23376,7 +23376,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23387,12 +23387,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23423,12 +23423,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23459,17 +23459,17 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E73" s="27" t="inlineStr">
@@ -23484,7 +23484,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -23495,17 +23495,17 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E74" s="27" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23531,12 +23531,12 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -23567,12 +23567,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23603,12 +23603,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23628,7 +23628,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -23639,12 +23639,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23675,12 +23675,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23711,12 +23711,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23736,7 +23736,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -23747,12 +23747,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23783,17 +23783,17 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E82" s="27" t="inlineStr">
@@ -23808,7 +23808,7 @@
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr"/>
@@ -23819,12 +23819,12 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -23844,7 +23844,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23855,12 +23855,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23891,12 +23891,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23927,17 +23927,17 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E86" s="27" t="inlineStr">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -23963,12 +23963,12 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -23999,12 +23999,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24035,12 +24035,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24060,7 +24060,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24071,12 +24071,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24107,12 +24107,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24143,17 +24143,17 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E92" s="27" t="inlineStr">
@@ -24168,7 +24168,7 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr"/>
@@ -24179,12 +24179,12 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24215,12 +24215,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24251,12 +24251,12 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -24287,17 +24287,17 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E96" s="27" t="inlineStr">
@@ -24307,12 +24307,12 @@
       </c>
       <c r="F96" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24323,12 +24323,12 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
@@ -24348,7 +24348,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24359,12 +24359,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24395,12 +24395,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24431,17 +24431,17 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E100" s="27" t="inlineStr">
@@ -24456,7 +24456,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24467,12 +24467,12 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -24503,12 +24503,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24539,12 +24539,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24575,12 +24575,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24611,12 +24611,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24647,12 +24647,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24683,12 +24683,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24719,17 +24719,17 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E108" s="27" t="inlineStr">
@@ -24744,7 +24744,7 @@
       </c>
       <c r="G108" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr"/>
@@ -24755,12 +24755,12 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -24791,12 +24791,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24827,12 +24827,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24863,12 +24863,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24899,17 +24899,17 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E113" s="27" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -24935,12 +24935,12 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24971,17 +24971,17 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E115" s="27" t="inlineStr">
@@ -24996,7 +24996,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25007,12 +25007,12 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25032,7 +25032,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25043,12 +25043,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25079,12 +25079,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25115,12 +25115,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25140,7 +25140,7 @@
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25151,12 +25151,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25187,17 +25187,17 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E121" s="27" t="inlineStr">
@@ -25212,7 +25212,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25223,12 +25223,12 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25248,7 +25248,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25259,17 +25259,17 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E123" s="27" t="inlineStr">
@@ -25284,7 +25284,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25295,12 +25295,12 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25331,17 +25331,17 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E125" s="27" t="inlineStr">
@@ -25356,7 +25356,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25367,12 +25367,12 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25392,7 +25392,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25403,12 +25403,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25439,12 +25439,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25475,12 +25475,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25495,12 +25495,12 @@
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25511,12 +25511,12 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -25536,7 +25536,7 @@
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25547,12 +25547,12 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -25572,7 +25572,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25583,17 +25583,17 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E132" s="27" t="inlineStr">
@@ -25608,7 +25608,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25619,17 +25619,17 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E133" s="27" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25655,12 +25655,12 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -25680,7 +25680,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25691,17 +25691,17 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E135" s="27" t="inlineStr">
@@ -25716,7 +25716,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25727,12 +25727,12 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
@@ -25752,7 +25752,7 @@
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25763,17 +25763,17 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E137" s="27" t="inlineStr">
@@ -25788,7 +25788,7 @@
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -25799,12 +25799,12 @@
       </c>
       <c r="B138" s="23" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
@@ -25824,7 +25824,7 @@
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -25835,12 +25835,12 @@
       </c>
       <c r="B139" s="25" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -25871,12 +25871,12 @@
       </c>
       <c r="B140" s="23" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -25896,7 +25896,7 @@
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr"/>
@@ -25907,12 +25907,12 @@
       </c>
       <c r="B141" s="25" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -25932,7 +25932,7 @@
       </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
@@ -25943,12 +25943,12 @@
       </c>
       <c r="B142" s="23" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -25968,7 +25968,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -25979,12 +25979,12 @@
       </c>
       <c r="B143" s="25" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26015,12 +26015,12 @@
       </c>
       <c r="B144" s="23" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
@@ -26040,7 +26040,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26051,12 +26051,12 @@
       </c>
       <c r="B145" s="25" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
@@ -26076,7 +26076,7 @@
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26087,12 +26087,12 @@
       </c>
       <c r="B146" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26123,12 +26123,12 @@
       </c>
       <c r="B147" s="25" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
@@ -26143,12 +26143,12 @@
       </c>
       <c r="F147" s="16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26159,12 +26159,12 @@
       </c>
       <c r="B148" s="23" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
@@ -26184,7 +26184,7 @@
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26195,12 +26195,12 @@
       </c>
       <c r="B149" s="25" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
@@ -26220,7 +26220,7 @@
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26231,12 +26231,12 @@
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26256,7 +26256,7 @@
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr"/>
@@ -26267,12 +26267,12 @@
       </c>
       <c r="B151" s="25" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26287,12 +26287,12 @@
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
@@ -26303,12 +26303,12 @@
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D152" s="12" t="inlineStr">
@@ -26339,12 +26339,12 @@
       </c>
       <c r="B153" s="25" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D153" s="16" t="inlineStr">
@@ -26375,38 +26375,74 @@
       </c>
       <c r="B154" s="23" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D154" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E154" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F154" s="12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G154" s="13" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H154" s="13" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="16" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C154" s="13" t="inlineStr">
+      <c r="C155" s="5" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D154" s="12" t="inlineStr">
+      <c r="D155" s="16" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E154" s="27" t="inlineStr">
+      <c r="E155" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F154" s="12" t="inlineStr">
+      <c r="F155" s="16" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G154" s="13" t="inlineStr">
+      <c r="G155" s="5" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H154" s="13" t="inlineStr"/>
+      <c r="H155" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H154"/>
+  <autoFilter ref="A1:H155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T153: đổi mã việc danh mục vừa một trang từ T150 sang T153 (trùng mã với việc của dinhlanphuongipacc)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$K$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -844,7 +844,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>154 việc (T01 - T108)</t>
+          <t>155 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>130 việc (84.4%)</t>
+          <t>131 việc (84.5%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21026,7 +21026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H155"/>
+  <dimension ref="A1:H156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21767,17 +21767,17 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T152</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
+          <t>Danh sách thẻ chi phí: số thẻ link xanh mở thẻ; thẻ mở ở chế độ xem, bấm Sửa (Ctrl+E) mới sửa, Huỷ về xem như phiếu chi. Thông tin đơn vị: phương pháp thuế GTGT, TNCN, TNDN lên khối Thông tin kê khai, khoá theo loại hình, nhóm doanh thu, gói</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
@@ -21792,7 +21792,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
+          <t>`2026-10-11-dinhlanphuongipacc-xem-the-thue.md`</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr"/>
@@ -21803,12 +21803,12 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>T151</t>
+          <t>T152</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
+          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -21828,7 +21828,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
+          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -21839,12 +21839,12 @@
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>T150</t>
+          <t>T151</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
+          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -21864,7 +21864,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
+          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -21875,12 +21875,12 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T153</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -21900,7 +21900,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -21911,12 +21911,12 @@
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -21947,12 +21947,12 @@
       </c>
       <c r="B31" s="25" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -21983,12 +21983,12 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -22019,17 +22019,17 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22055,12 +22055,12 @@
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22080,7 +22080,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22091,12 +22091,12 @@
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22127,12 +22127,12 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22152,7 +22152,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22163,12 +22163,12 @@
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22188,7 +22188,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22199,17 +22199,17 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22235,12 +22235,12 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22271,17 +22271,17 @@
       </c>
       <c r="B40" s="23" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
@@ -22296,7 +22296,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22307,17 +22307,17 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr">
@@ -22332,7 +22332,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22343,12 +22343,12 @@
       </c>
       <c r="B42" s="23" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -22363,12 +22363,12 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22379,17 +22379,17 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E43" s="27" t="inlineStr">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22415,12 +22415,12 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22451,12 +22451,12 @@
       </c>
       <c r="B45" s="25" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -22487,12 +22487,12 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -22523,12 +22523,12 @@
       </c>
       <c r="B47" s="25" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -22559,12 +22559,12 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -22584,7 +22584,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -22595,12 +22595,12 @@
       </c>
       <c r="B49" s="25" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -22620,7 +22620,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -22631,12 +22631,12 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -22656,7 +22656,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -22667,12 +22667,12 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -22703,12 +22703,12 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -22728,7 +22728,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -22739,17 +22739,17 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr"/>
@@ -22775,17 +22775,17 @@
       </c>
       <c r="B54" s="23" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E54" s="27" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H54" s="13" t="inlineStr"/>
@@ -22811,17 +22811,17 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -22847,12 +22847,12 @@
       </c>
       <c r="B56" s="23" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -22883,17 +22883,17 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E57" s="27" t="inlineStr">
@@ -22908,7 +22908,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -22919,12 +22919,12 @@
       </c>
       <c r="B58" s="23" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -22944,7 +22944,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -22955,12 +22955,12 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -22991,12 +22991,12 @@
       </c>
       <c r="B60" s="23" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23027,12 +23027,12 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23063,12 +23063,12 @@
       </c>
       <c r="B62" s="23" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23099,17 +23099,17 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E63" s="27" t="inlineStr">
@@ -23124,7 +23124,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23135,12 +23135,12 @@
       </c>
       <c r="B64" s="23" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23160,7 +23160,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23171,17 +23171,17 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E65" s="27" t="inlineStr">
@@ -23196,7 +23196,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23207,17 +23207,17 @@
       </c>
       <c r="B66" s="23" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E66" s="27" t="inlineStr">
@@ -23232,7 +23232,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23243,12 +23243,12 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23279,12 +23279,12 @@
       </c>
       <c r="B68" s="23" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23315,12 +23315,12 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23351,12 +23351,12 @@
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23387,12 +23387,12 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23423,12 +23423,12 @@
       </c>
       <c r="B72" s="23" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23459,12 +23459,12 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -23495,17 +23495,17 @@
       </c>
       <c r="B74" s="23" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E74" s="27" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -23531,17 +23531,17 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E75" s="27" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -23567,12 +23567,12 @@
       </c>
       <c r="B76" s="23" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -23603,12 +23603,12 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -23639,12 +23639,12 @@
       </c>
       <c r="B78" s="23" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -23664,7 +23664,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -23675,12 +23675,12 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -23711,12 +23711,12 @@
       </c>
       <c r="B80" s="23" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -23747,12 +23747,12 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -23772,7 +23772,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -23783,12 +23783,12 @@
       </c>
       <c r="B82" s="23" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -23819,17 +23819,17 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E83" s="27" t="inlineStr">
@@ -23844,7 +23844,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr"/>
@@ -23855,12 +23855,12 @@
       </c>
       <c r="B84" s="23" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -23880,7 +23880,7 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr"/>
@@ -23891,12 +23891,12 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -23927,12 +23927,12 @@
       </c>
       <c r="B86" s="23" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -23963,17 +23963,17 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E87" s="27" t="inlineStr">
@@ -23988,7 +23988,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -23999,12 +23999,12 @@
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -24035,12 +24035,12 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24060,7 +24060,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24071,12 +24071,12 @@
       </c>
       <c r="B90" s="23" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr"/>
@@ -24107,12 +24107,12 @@
       </c>
       <c r="B91" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24143,12 +24143,12 @@
       </c>
       <c r="B92" s="23" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24179,17 +24179,17 @@
       </c>
       <c r="B93" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E93" s="27" t="inlineStr">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24215,12 +24215,12 @@
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24251,12 +24251,12 @@
       </c>
       <c r="B95" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -24287,12 +24287,12 @@
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24323,17 +24323,17 @@
       </c>
       <c r="B97" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E97" s="27" t="inlineStr">
@@ -24343,12 +24343,12 @@
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24359,12 +24359,12 @@
       </c>
       <c r="B98" s="23" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24395,12 +24395,12 @@
       </c>
       <c r="B99" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
@@ -24431,12 +24431,12 @@
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24467,17 +24467,17 @@
       </c>
       <c r="B101" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E101" s="27" t="inlineStr">
@@ -24492,7 +24492,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -24503,12 +24503,12 @@
       </c>
       <c r="B102" s="23" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -24539,12 +24539,12 @@
       </c>
       <c r="B103" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -24575,12 +24575,12 @@
       </c>
       <c r="B104" s="23" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -24611,12 +24611,12 @@
       </c>
       <c r="B105" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -24647,12 +24647,12 @@
       </c>
       <c r="B106" s="23" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -24683,12 +24683,12 @@
       </c>
       <c r="B107" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -24719,12 +24719,12 @@
       </c>
       <c r="B108" s="23" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -24755,17 +24755,17 @@
       </c>
       <c r="B109" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E109" s="27" t="inlineStr">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -24791,12 +24791,12 @@
       </c>
       <c r="B110" s="23" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -24827,12 +24827,12 @@
       </c>
       <c r="B111" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -24863,12 +24863,12 @@
       </c>
       <c r="B112" s="23" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -24899,12 +24899,12 @@
       </c>
       <c r="B113" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -24935,17 +24935,17 @@
       </c>
       <c r="B114" s="23" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E114" s="27" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr"/>
@@ -24971,12 +24971,12 @@
       </c>
       <c r="B115" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -24996,7 +24996,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25007,17 +25007,17 @@
       </c>
       <c r="B116" s="23" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E116" s="27" t="inlineStr">
@@ -25032,7 +25032,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25043,12 +25043,12 @@
       </c>
       <c r="B117" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25068,7 +25068,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="B118" s="23" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25115,12 +25115,12 @@
       </c>
       <c r="B119" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25151,12 +25151,12 @@
       </c>
       <c r="B120" s="23" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25187,12 +25187,12 @@
       </c>
       <c r="B121" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25212,7 +25212,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25223,17 +25223,17 @@
       </c>
       <c r="B122" s="23" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E122" s="27" t="inlineStr">
@@ -25248,7 +25248,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25259,12 +25259,12 @@
       </c>
       <c r="B123" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25284,7 +25284,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25295,17 +25295,17 @@
       </c>
       <c r="B124" s="23" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E124" s="27" t="inlineStr">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25331,12 +25331,12 @@
       </c>
       <c r="B125" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25356,7 +25356,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
@@ -25367,17 +25367,17 @@
       </c>
       <c r="B126" s="23" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E126" s="27" t="inlineStr">
@@ -25392,7 +25392,7 @@
       </c>
       <c r="G126" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr"/>
@@ -25403,12 +25403,12 @@
       </c>
       <c r="B127" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
@@ -25439,12 +25439,12 @@
       </c>
       <c r="B128" s="23" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="G128" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr"/>
@@ -25475,12 +25475,12 @@
       </c>
       <c r="B129" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -25500,7 +25500,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
@@ -25511,12 +25511,12 @@
       </c>
       <c r="B130" s="23" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -25531,12 +25531,12 @@
       </c>
       <c r="F130" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G130" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H130" s="13" t="inlineStr"/>
@@ -25547,12 +25547,12 @@
       </c>
       <c r="B131" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -25572,7 +25572,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -25583,12 +25583,12 @@
       </c>
       <c r="B132" s="23" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -25608,7 +25608,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -25619,17 +25619,17 @@
       </c>
       <c r="B133" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E133" s="27" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
@@ -25655,17 +25655,17 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E134" s="27" t="inlineStr">
@@ -25680,7 +25680,7 @@
       </c>
       <c r="G134" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr"/>
@@ -25691,12 +25691,12 @@
       </c>
       <c r="B135" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -25716,7 +25716,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
@@ -25727,17 +25727,17 @@
       </c>
       <c r="B136" s="23" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E136" s="27" t="inlineStr">
@@ -25752,7 +25752,7 @@
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -25763,12 +25763,12 @@
       </c>
       <c r="B137" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -25788,7 +25788,7 @@
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -25799,17 +25799,17 @@
       </c>
       <c r="B138" s="23" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E138" s="27" t="inlineStr">
@@ -25824,7 +25824,7 @@
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -25835,12 +25835,12 @@
       </c>
       <c r="B139" s="25" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -25860,7 +25860,7 @@
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -25871,12 +25871,12 @@
       </c>
       <c r="B140" s="23" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -25907,12 +25907,12 @@
       </c>
       <c r="B141" s="25" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -25932,7 +25932,7 @@
       </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
@@ -25943,12 +25943,12 @@
       </c>
       <c r="B142" s="23" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -25968,7 +25968,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -25979,12 +25979,12 @@
       </c>
       <c r="B143" s="25" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26015,12 +26015,12 @@
       </c>
       <c r="B144" s="23" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
@@ -26040,7 +26040,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26051,12 +26051,12 @@
       </c>
       <c r="B145" s="25" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
@@ -26076,7 +26076,7 @@
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26087,12 +26087,12 @@
       </c>
       <c r="B146" s="23" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26123,12 +26123,12 @@
       </c>
       <c r="B147" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26159,12 +26159,12 @@
       </c>
       <c r="B148" s="23" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
@@ -26179,12 +26179,12 @@
       </c>
       <c r="F148" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26195,12 +26195,12 @@
       </c>
       <c r="B149" s="25" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
@@ -26220,7 +26220,7 @@
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26231,12 +26231,12 @@
       </c>
       <c r="B150" s="23" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26256,7 +26256,7 @@
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr"/>
@@ -26267,12 +26267,12 @@
       </c>
       <c r="B151" s="25" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26292,7 +26292,7 @@
       </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
@@ -26303,12 +26303,12 @@
       </c>
       <c r="B152" s="23" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D152" s="12" t="inlineStr">
@@ -26323,12 +26323,12 @@
       </c>
       <c r="F152" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G152" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr"/>
@@ -26339,12 +26339,12 @@
       </c>
       <c r="B153" s="25" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D153" s="16" t="inlineStr">
@@ -26375,12 +26375,12 @@
       </c>
       <c r="B154" s="23" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C154" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D154" s="12" t="inlineStr">
@@ -26411,38 +26411,74 @@
       </c>
       <c r="B155" s="25" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D155" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E155" s="27" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F155" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H155" s="5" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="23" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C155" s="5" t="inlineStr">
+      <c r="C156" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D155" s="16" t="inlineStr">
+      <c r="D156" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E155" s="27" t="inlineStr">
+      <c r="E156" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F155" s="16" t="inlineStr">
+      <c r="F156" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G155" s="5" t="inlineStr">
+      <c r="G156" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H155" s="5" t="inlineStr"/>
+      <c r="H156" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H155"/>
+  <autoFilter ref="A1:H156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T155: kho tách xuất điều chuyển, nhập điều chuyển (tham chiếu nhau, 1368, 3368) và chuyển kho không hạch toán
- 5.1.4, 5-1-4-2, 5-1-4-3; dùng lại cơ chế tham chiếu phiếu sản xuất
- báo cáo nhập, xuất có phiếu điều chuyển; sơ đồ, menu bay, tìm nhanh trỏ đúng tab
- QD53, nhật ký, CHANGELOG, báo cáo hệ thống

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,12 +81,6 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00854D0E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
@@ -96,7 +90,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -153,12 +147,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-        <bgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
       </patternFill>
@@ -196,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -258,9 +246,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -652,7 +637,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ngày xuất: 11/10/2026 | Bản mẫu iaccdemo (React 19 + TypeScript + Vite) | Deploy: https://iaccdemo.pages.dev</t>
+          <t>Ngày xuất: 12/10/2026 | Bản mẫu iaccdemo (React 19 + TypeScript + Vite) | Deploy: https://iaccdemo.pages.dev</t>
         </is>
       </c>
     </row>
@@ -876,7 +861,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>134 việc (84.3%)</t>
+          <t>135 việc (84.9%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -893,7 +878,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>1 việc</t>
+          <t>0 việc</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -21102,29 +21087,29 @@
       </c>
       <c r="B2" s="23" t="inlineStr">
         <is>
-          <t>T155</t>
+          <t>T138</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
+          <t>Màn onboard khi bấm từ FABi sang IACC: khởi tạo đơn vị kế toán, điền sẵn từ FABi (chi nhánh, kho, cách đồng bộ, số dư đầu kỳ)</t>
         </is>
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E2" s="24" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Làm sau T157. Sửa `kho/index.ts`, `ChungTuForm.tsx`, `app.css`</t>
+          <t>Popup khởi tạo dữ liệu 4 bước trong phần mềm (`OnboardFabi.tsx`, `Shell.tsx`) đã push, PhuongXT xem lại một lượt. Xem `2026-10-11-phuongxt-man-khoi-tao-fabi.md`</t>
         </is>
       </c>
     </row>
@@ -21134,29 +21119,25 @@
       </c>
       <c r="B3" s="25" t="inlineStr">
         <is>
-          <t>T138</t>
+          <t>T139</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Màn onboard khi bấm từ FABi sang IACC: khởi tạo đơn vị kế toán, điền sẵn từ FABi (chi nhánh, kho, cách đồng bộ, số dư đầu kỳ)</t>
-        </is>
-      </c>
-      <c r="D3" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
+          <t>Phiếu nhập, xuất, điều chuyển kho tự lấy mục chi phí, công việc ngầm định theo kho đã chọn</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr"/>
       <c r="E3" s="26" t="inlineStr">
         <is>
-          <t>Dở dang</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Popup khởi tạo dữ liệu 4 bước trong phần mềm (`OnboardFabi.tsx`, `Shell.tsx`) đã push, PhuongXT xem lại một lượt. Xem `2026-10-11-phuongxt-man-khoi-tao-fabi.md`</t>
+          <t>Tách từ T136. Kho đã có ô `mucCp`, `congViec` ở `truong-dm.ts` 1.8. Sửa `ChungTuForm.tsx`</t>
         </is>
       </c>
     </row>
@@ -21166,16 +21147,16 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>T139</t>
+          <t>T140</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Phiếu nhập, xuất, điều chuyển kho tự lấy mục chi phí, công việc ngầm định theo kho đã chọn</t>
+          <t>Đồng bộ POS có tích tự hạch toán theo phương thức thanh toán thì sinh phiếu thu thật vào danh sách Thu tiền mặt, Thu ngân hàng (hiện chỉ báo số phiếu bằng toast)</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21184,7 +21165,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T136. Kho đã có ô `mucCp`, `congViec` ở `truong-dm.ts` 1.8. Sửa `ChungTuForm.tsx`</t>
+          <t>Tách từ T137. Phiếu thu Nợ TK của phương thức / Có 131, lấy từ `DS_PTTT` ở `danh-muc/data.ts`</t>
         </is>
       </c>
     </row>
@@ -21194,16 +21175,16 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>T140</t>
+          <t>T120</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Đồng bộ POS có tích tự hạch toán theo phương thức thanh toán thì sinh phiếu thu thật vào danh sách Thu tiền mặt, Thu ngân hàng (hiện chỉ báo số phiếu bằng toast)</t>
+          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr"/>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21212,7 +21193,7 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T137. Phiếu thu Nợ TK của phương thức / Có 131, lấy từ `DS_PTTT` ở `danh-muc/data.ts`</t>
+          <t>Phát hiện khi làm T112</t>
         </is>
       </c>
     </row>
@@ -21222,16 +21203,16 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>T120</t>
+          <t>T109</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="E6" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21240,7 +21221,7 @@
       <c r="G6" s="13" t="inlineStr"/>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Phát hiện khi làm T112</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21250,16 +21231,16 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>T109</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21268,7 +21249,7 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
         </is>
       </c>
     </row>
@@ -21278,16 +21259,20 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>T110</t>
+          <t>T101</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="27" t="inlineStr">
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21296,7 +21281,7 @@
       <c r="G8" s="13" t="inlineStr"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
         </is>
       </c>
     </row>
@@ -21306,12 +21291,12 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -21319,16 +21304,16 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E9" s="27" t="inlineStr">
-        <is>
-          <t>Chờ</t>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
+          <t>11/10/2026 PhuongXT chốt gói Free không giới hạn chi nhánh (làm cùng T138): đã sửa mô tả gói Free, điểm nổi bật, câu hỏi đáp màn Gói thuê bao. Gói Standard còn ghi "1 điểm bán", chưa chốt</t>
         </is>
       </c>
     </row>
@@ -21338,31 +21323,27 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
         <is>
-          <t>Dở dang</t>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>11/10/2026 PhuongXT chốt gói Free không giới hạn chi nhánh (làm cùng T138): đã sửa mô tả gói Free, điểm nổi bật, câu hỏi đáp màn Gói thuê bao. Gói Standard còn ghi "1 điểm bán", chưa chốt</t>
-        </is>
-      </c>
+      <c r="H10" s="13" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
@@ -21370,27 +21351,27 @@
       </c>
       <c r="B11" s="25" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E11" s="27" t="inlineStr">
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr"/>
+      <c r="E11" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -21398,16 +21379,16 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T33</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="27" t="inlineStr">
+      <c r="E12" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21416,7 +21397,7 @@
       <c r="G12" s="13" t="inlineStr"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+          <t>Chỉ máy Trum chạy được script</t>
         </is>
       </c>
     </row>
@@ -21426,16 +21407,16 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>T33</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
-      <c r="E13" s="27" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21444,7 +21425,7 @@
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Chỉ máy Trum chạy được script</t>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
         </is>
       </c>
     </row>
@@ -21454,16 +21435,16 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21472,7 +21453,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
         </is>
       </c>
     </row>
@@ -21482,27 +21463,23 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="27" t="inlineStr">
+      <c r="E15" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
-        </is>
-      </c>
+      <c r="H15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="n">
@@ -21510,23 +21487,27 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T07</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr"/>
       <c r="G16" s="13" t="inlineStr"/>
-      <c r="H16" s="13" t="inlineStr"/>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n">
@@ -21534,16 +21515,16 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>T07</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
-      <c r="E17" s="27" t="inlineStr">
+      <c r="E17" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21552,7 +21533,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
         </is>
       </c>
     </row>
@@ -21562,16 +21543,16 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T09</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="27" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21580,7 +21561,7 @@
       <c r="G18" s="13" t="inlineStr"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -21590,16 +21571,16 @@
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>T09</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21608,7 +21589,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -21618,16 +21599,16 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T11</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="27" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21636,7 +21617,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -21646,16 +21627,16 @@
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
-      <c r="E21" s="27" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21664,7 +21645,7 @@
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -21674,16 +21655,16 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T13</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="27" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21692,7 +21673,7 @@
       <c r="G22" s="13" t="inlineStr"/>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -21702,16 +21683,16 @@
       </c>
       <c r="B23" s="25" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr"/>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21720,7 +21701,7 @@
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>Chưa có file logo iPOS</t>
         </is>
       </c>
     </row>
@@ -21730,16 +21711,16 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21748,7 +21729,7 @@
       <c r="G24" s="13" t="inlineStr"/>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
         </is>
       </c>
     </row>
@@ -21758,16 +21739,16 @@
       </c>
       <c r="B25" s="25" t="inlineStr">
         <is>
-          <t>T19</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
-      <c r="E25" s="27" t="inlineStr">
+      <c r="E25" s="26" t="inlineStr">
         <is>
           <t>Chờ</t>
         </is>
@@ -21776,7 +21757,7 @@
       <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
         </is>
       </c>
     </row>
@@ -21786,27 +21767,35 @@
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T155</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr"/>
+          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Chờ</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr"/>
-      <c r="G26" s="13" t="inlineStr"/>
-      <c r="H26" s="13" t="inlineStr">
-        <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
-        </is>
-      </c>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>[2026-10-12-trum-dieu-chuyen-chuyen-kho](nhat-ky/2026-10-12-trum-dieu-chuyen-chuyen-kho.md)</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n">
@@ -21827,7 +21816,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E27" s="28" t="inlineStr">
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21863,7 +21852,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E28" s="28" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21899,7 +21888,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E29" s="28" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21935,7 +21924,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E30" s="28" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -21971,7 +21960,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E31" s="28" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22007,7 +21996,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E32" s="28" t="inlineStr">
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22043,7 +22032,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E33" s="28" t="inlineStr">
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22079,7 +22068,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E34" s="28" t="inlineStr">
+      <c r="E34" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22115,7 +22104,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E35" s="28" t="inlineStr">
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22151,7 +22140,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E36" s="28" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22187,7 +22176,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E37" s="28" t="inlineStr">
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22223,7 +22212,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E38" s="28" t="inlineStr">
+      <c r="E38" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22259,7 +22248,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E39" s="28" t="inlineStr">
+      <c r="E39" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22295,7 +22284,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E40" s="28" t="inlineStr">
+      <c r="E40" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22331,7 +22320,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E41" s="28" t="inlineStr">
+      <c r="E41" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22367,7 +22356,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E42" s="28" t="inlineStr">
+      <c r="E42" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22403,7 +22392,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E43" s="28" t="inlineStr">
+      <c r="E43" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22439,7 +22428,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E44" s="28" t="inlineStr">
+      <c r="E44" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22475,7 +22464,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E45" s="28" t="inlineStr">
+      <c r="E45" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22511,7 +22500,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E46" s="28" t="inlineStr">
+      <c r="E46" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22547,7 +22536,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E47" s="28" t="inlineStr">
+      <c r="E47" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22583,7 +22572,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E48" s="28" t="inlineStr">
+      <c r="E48" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22619,7 +22608,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E49" s="28" t="inlineStr">
+      <c r="E49" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22655,7 +22644,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E50" s="28" t="inlineStr">
+      <c r="E50" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22691,7 +22680,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E51" s="28" t="inlineStr">
+      <c r="E51" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22727,7 +22716,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E52" s="28" t="inlineStr">
+      <c r="E52" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22763,7 +22752,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E53" s="28" t="inlineStr">
+      <c r="E53" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22799,7 +22788,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E54" s="28" t="inlineStr">
+      <c r="E54" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22835,7 +22824,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E55" s="28" t="inlineStr">
+      <c r="E55" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22871,7 +22860,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E56" s="28" t="inlineStr">
+      <c r="E56" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22907,7 +22896,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E57" s="28" t="inlineStr">
+      <c r="E57" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22943,7 +22932,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E58" s="28" t="inlineStr">
+      <c r="E58" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22979,7 +22968,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E59" s="28" t="inlineStr">
+      <c r="E59" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23015,7 +23004,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E60" s="28" t="inlineStr">
+      <c r="E60" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23051,7 +23040,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E61" s="28" t="inlineStr">
+      <c r="E61" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23087,7 +23076,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E62" s="28" t="inlineStr">
+      <c r="E62" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23123,7 +23112,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E63" s="28" t="inlineStr">
+      <c r="E63" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23159,7 +23148,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E64" s="28" t="inlineStr">
+      <c r="E64" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23195,7 +23184,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E65" s="28" t="inlineStr">
+      <c r="E65" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23231,7 +23220,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E66" s="28" t="inlineStr">
+      <c r="E66" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23267,7 +23256,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E67" s="28" t="inlineStr">
+      <c r="E67" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23303,7 +23292,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E68" s="28" t="inlineStr">
+      <c r="E68" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23339,7 +23328,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E69" s="28" t="inlineStr">
+      <c r="E69" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23375,7 +23364,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E70" s="28" t="inlineStr">
+      <c r="E70" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23411,7 +23400,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E71" s="28" t="inlineStr">
+      <c r="E71" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23447,7 +23436,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E72" s="28" t="inlineStr">
+      <c r="E72" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23483,7 +23472,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E73" s="28" t="inlineStr">
+      <c r="E73" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23519,7 +23508,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E74" s="28" t="inlineStr">
+      <c r="E74" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23555,7 +23544,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E75" s="28" t="inlineStr">
+      <c r="E75" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23591,7 +23580,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E76" s="28" t="inlineStr">
+      <c r="E76" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23627,7 +23616,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E77" s="28" t="inlineStr">
+      <c r="E77" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23663,7 +23652,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E78" s="28" t="inlineStr">
+      <c r="E78" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23699,7 +23688,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E79" s="28" t="inlineStr">
+      <c r="E79" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23735,7 +23724,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E80" s="28" t="inlineStr">
+      <c r="E80" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23771,7 +23760,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E81" s="28" t="inlineStr">
+      <c r="E81" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23807,7 +23796,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E82" s="28" t="inlineStr">
+      <c r="E82" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23843,7 +23832,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E83" s="28" t="inlineStr">
+      <c r="E83" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23879,7 +23868,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E84" s="28" t="inlineStr">
+      <c r="E84" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23915,7 +23904,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E85" s="28" t="inlineStr">
+      <c r="E85" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23951,7 +23940,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E86" s="28" t="inlineStr">
+      <c r="E86" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23987,7 +23976,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E87" s="28" t="inlineStr">
+      <c r="E87" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24023,7 +24012,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E88" s="28" t="inlineStr">
+      <c r="E88" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24059,7 +24048,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E89" s="28" t="inlineStr">
+      <c r="E89" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24095,7 +24084,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E90" s="28" t="inlineStr">
+      <c r="E90" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24131,7 +24120,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E91" s="28" t="inlineStr">
+      <c r="E91" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24167,7 +24156,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E92" s="28" t="inlineStr">
+      <c r="E92" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24203,7 +24192,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E93" s="28" t="inlineStr">
+      <c r="E93" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24239,7 +24228,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E94" s="28" t="inlineStr">
+      <c r="E94" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24275,7 +24264,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E95" s="28" t="inlineStr">
+      <c r="E95" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24311,7 +24300,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E96" s="28" t="inlineStr">
+      <c r="E96" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24347,7 +24336,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E97" s="28" t="inlineStr">
+      <c r="E97" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24383,7 +24372,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E98" s="28" t="inlineStr">
+      <c r="E98" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24419,7 +24408,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E99" s="28" t="inlineStr">
+      <c r="E99" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24455,7 +24444,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E100" s="28" t="inlineStr">
+      <c r="E100" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24491,7 +24480,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E101" s="28" t="inlineStr">
+      <c r="E101" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24527,7 +24516,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E102" s="28" t="inlineStr">
+      <c r="E102" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24563,7 +24552,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E103" s="28" t="inlineStr">
+      <c r="E103" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24599,7 +24588,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E104" s="28" t="inlineStr">
+      <c r="E104" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24635,7 +24624,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E105" s="28" t="inlineStr">
+      <c r="E105" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24671,7 +24660,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E106" s="28" t="inlineStr">
+      <c r="E106" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24707,7 +24696,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E107" s="28" t="inlineStr">
+      <c r="E107" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24743,7 +24732,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E108" s="28" t="inlineStr">
+      <c r="E108" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24779,7 +24768,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E109" s="28" t="inlineStr">
+      <c r="E109" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24815,7 +24804,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E110" s="28" t="inlineStr">
+      <c r="E110" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24851,7 +24840,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E111" s="28" t="inlineStr">
+      <c r="E111" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24887,7 +24876,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E112" s="28" t="inlineStr">
+      <c r="E112" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24923,7 +24912,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E113" s="28" t="inlineStr">
+      <c r="E113" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24959,7 +24948,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E114" s="28" t="inlineStr">
+      <c r="E114" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24995,7 +24984,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E115" s="28" t="inlineStr">
+      <c r="E115" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25031,7 +25020,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E116" s="28" t="inlineStr">
+      <c r="E116" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25067,7 +25056,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E117" s="28" t="inlineStr">
+      <c r="E117" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25103,7 +25092,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E118" s="28" t="inlineStr">
+      <c r="E118" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25139,7 +25128,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E119" s="28" t="inlineStr">
+      <c r="E119" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25175,7 +25164,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E120" s="28" t="inlineStr">
+      <c r="E120" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25211,7 +25200,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E121" s="28" t="inlineStr">
+      <c r="E121" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25247,7 +25236,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E122" s="28" t="inlineStr">
+      <c r="E122" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25283,7 +25272,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E123" s="28" t="inlineStr">
+      <c r="E123" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25319,7 +25308,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E124" s="28" t="inlineStr">
+      <c r="E124" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25355,7 +25344,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E125" s="28" t="inlineStr">
+      <c r="E125" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25391,7 +25380,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E126" s="28" t="inlineStr">
+      <c r="E126" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25427,7 +25416,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E127" s="28" t="inlineStr">
+      <c r="E127" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25463,7 +25452,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E128" s="28" t="inlineStr">
+      <c r="E128" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25499,7 +25488,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E129" s="28" t="inlineStr">
+      <c r="E129" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25535,7 +25524,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E130" s="28" t="inlineStr">
+      <c r="E130" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25571,7 +25560,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E131" s="28" t="inlineStr">
+      <c r="E131" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25607,7 +25596,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E132" s="28" t="inlineStr">
+      <c r="E132" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25643,7 +25632,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E133" s="28" t="inlineStr">
+      <c r="E133" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25679,7 +25668,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E134" s="28" t="inlineStr">
+      <c r="E134" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25715,7 +25704,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E135" s="28" t="inlineStr">
+      <c r="E135" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25751,7 +25740,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E136" s="28" t="inlineStr">
+      <c r="E136" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25787,7 +25776,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E137" s="28" t="inlineStr">
+      <c r="E137" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25823,7 +25812,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E138" s="28" t="inlineStr">
+      <c r="E138" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25859,7 +25848,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E139" s="28" t="inlineStr">
+      <c r="E139" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25895,7 +25884,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E140" s="28" t="inlineStr">
+      <c r="E140" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25931,7 +25920,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E141" s="28" t="inlineStr">
+      <c r="E141" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25967,7 +25956,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E142" s="28" t="inlineStr">
+      <c r="E142" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26003,7 +25992,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E143" s="28" t="inlineStr">
+      <c r="E143" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26039,7 +26028,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E144" s="28" t="inlineStr">
+      <c r="E144" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26075,7 +26064,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E145" s="28" t="inlineStr">
+      <c r="E145" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26111,7 +26100,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E146" s="28" t="inlineStr">
+      <c r="E146" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26147,7 +26136,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E147" s="28" t="inlineStr">
+      <c r="E147" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26183,7 +26172,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E148" s="28" t="inlineStr">
+      <c r="E148" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26219,7 +26208,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E149" s="28" t="inlineStr">
+      <c r="E149" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26255,7 +26244,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E150" s="28" t="inlineStr">
+      <c r="E150" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26291,7 +26280,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E151" s="28" t="inlineStr">
+      <c r="E151" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26327,7 +26316,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E152" s="28" t="inlineStr">
+      <c r="E152" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26363,7 +26352,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E153" s="28" t="inlineStr">
+      <c r="E153" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26399,7 +26388,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E154" s="28" t="inlineStr">
+      <c r="E154" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26435,7 +26424,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E155" s="28" t="inlineStr">
+      <c r="E155" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26471,7 +26460,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E156" s="28" t="inlineStr">
+      <c r="E156" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26507,7 +26496,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E157" s="28" t="inlineStr">
+      <c r="E157" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26543,7 +26532,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E158" s="28" t="inlineStr">
+      <c r="E158" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26579,7 +26568,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E159" s="28" t="inlineStr">
+      <c r="E159" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26615,7 +26604,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E160" s="28" t="inlineStr">
+      <c r="E160" s="27" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>

</xml_diff>

<commit_message>
T173: làm mới Excel báo cáo hệ thống sau khi gộp T171, T174
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ma trận tính năng" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chi tiết màn hình" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Báo cáo &amp; Mẫu in" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tiến độ công việc" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma trận tính năng" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiết màn hình" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Báo cáo &amp; Mẫu in" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ công việc" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,17 +86,11 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00854D0E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -159,12 +153,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-        <bgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
       </patternFill>
@@ -196,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -257,13 +245,10 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -879,7 +864,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>149 việc (84.7%)</t>
+          <t>151 việc (85.8%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -896,7 +881,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>1 việc</t>
+          <t>0 việc</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -913,7 +898,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>24 việc</t>
+          <t>23 việc</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -21641,29 +21626,25 @@
       </c>
       <c r="B2" s="25" t="inlineStr">
         <is>
-          <t>T173</t>
+          <t>T169</t>
         </is>
       </c>
       <c r="C2" s="13" t="inlineStr">
         <is>
-          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên, thanh dưới 4 tab, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E2" s="26" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
+          <t>Form chứng từ: gõ đổi địa chỉ từ phiếu này sang phiếu khác (vd `#/app/tien/2-1-1/chi-3` sang `chi-6`) thì form giữ số phiếu, đối tượng của phiếu cũ; mở từ danh sách, Trước, Sau thì đúng</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr"/>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr"/>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Theo `docs/ke-hoach-mobile-ivt.md` mục 7 đợt 1. Điều phối Anti A, Anti B. Sửa `App.tsx`, `Screen.tsx`, `index.html`, `app.css` (mục cuối), `tools/kiem_tra.py`, file mới ở `src/ui/mobile/`</t>
+          <t>Phát hiện ở T168. Sửa `ChungTuForm.tsx`, có thể `VoucherScreen.tsx` (key của form)</t>
         </is>
       </c>
     </row>
@@ -21671,31 +21652,31 @@
       <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="27" t="inlineStr">
-        <is>
-          <t>T172</t>
+      <c r="B3" s="26" t="inlineStr">
+        <is>
+          <t>T138</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` trên máy có thư mục `Present` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
+          <t>Màn onboard khi bấm từ FABi sang IACC: khởi tạo đơn vị kế toán, điền sẵn từ FABi (chi nhánh, kho, cách đồng bộ, số dư đầu kỳ)</t>
         </is>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
-        </is>
-      </c>
-      <c r="E3" s="23" t="inlineStr">
-        <is>
-          <t>Chờ</t>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Máy PhuongXT thiếu `../Present/tools/build_present.py` nên không chạy được</t>
+          <t>Popup khởi tạo dữ liệu 4 bước trong phần mềm (`OnboardFabi.tsx`, `Shell.tsx`) đã push, PhuongXT xem lại một lượt. Xem `2026-10-11-phuongxt-man-khoi-tao-fabi.md`</t>
         </is>
       </c>
     </row>
@@ -21705,12 +21686,12 @@
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>T169</t>
+          <t>T139</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ: gõ đổi địa chỉ từ phiếu này sang phiếu khác (vd `#/app/tien/2-1-1/chi-3` sang `chi-6`) thì form giữ số phiếu, đối tượng của phiếu cũ; mở từ danh sách, Trước, Sau thì đúng</t>
+          <t>Phiếu nhập, xuất, điều chuyển kho tự lấy mục chi phí, công việc ngầm định theo kho đã chọn</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr"/>
@@ -21723,7 +21704,7 @@
       <c r="G4" s="13" t="inlineStr"/>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Phát hiện ở T168. Sửa `ChungTuForm.tsx`, có thể `VoucherScreen.tsx` (key của form)</t>
+          <t>Tách từ T136. Kho đã có ô `mucCp`, `congViec` ở `truong-dm.ts` 1.8. Sửa `ChungTuForm.tsx`</t>
         </is>
       </c>
     </row>
@@ -21731,31 +21712,27 @@
       <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>T138</t>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>T140</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Màn onboard khi bấm từ FABi sang IACC: khởi tạo đơn vị kế toán, điền sẵn từ FABi (chi nhánh, kho, cách đồng bộ, số dư đầu kỳ)</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E5" s="28" t="inlineStr">
-        <is>
-          <t>Dở dang</t>
+          <t>Đồng bộ POS có tích tự hạch toán theo phương thức thanh toán thì sinh phiếu thu thật vào danh sách Thu tiền mặt, Thu ngân hàng (hiện chỉ báo số phiếu bằng toast)</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr"/>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Popup khởi tạo dữ liệu 4 bước trong phần mềm (`OnboardFabi.tsx`, `Shell.tsx`) đã push, PhuongXT xem lại một lượt. Xem `2026-10-11-phuongxt-man-khoi-tao-fabi.md`</t>
+          <t>Tách từ T137. Phiếu thu Nợ TK của phương thức / Có 131, lấy từ `DS_PTTT` ở `danh-muc/data.ts`</t>
         </is>
       </c>
     </row>
@@ -21765,12 +21742,12 @@
       </c>
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>T139</t>
+          <t>T120</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Phiếu nhập, xuất, điều chuyển kho tự lấy mục chi phí, công việc ngầm định theo kho đã chọn</t>
+          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr"/>
@@ -21783,7 +21760,7 @@
       <c r="G6" s="13" t="inlineStr"/>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T136. Kho đã có ô `mucCp`, `congViec` ở `truong-dm.ts` 1.8. Sửa `ChungTuForm.tsx`</t>
+          <t>Phát hiện khi làm T112</t>
         </is>
       </c>
     </row>
@@ -21791,14 +21768,14 @@
       <c r="A7" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>T140</t>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>T109</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Đồng bộ POS có tích tự hạch toán theo phương thức thanh toán thì sinh phiếu thu thật vào danh sách Thu tiền mặt, Thu ngân hàng (hiện chỉ báo số phiếu bằng toast)</t>
+          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
@@ -21811,7 +21788,7 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Tách từ T137. Phiếu thu Nợ TK của phương thức / Có 131, lấy từ `DS_PTTT` ở `danh-muc/data.ts`</t>
+          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
         </is>
       </c>
     </row>
@@ -21821,12 +21798,12 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>T120</t>
+          <t>T110</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>In phiếu từ form chứng từ: hàm `moIn` ở `ChungTuForm.tsx` (khoảng dòng 317–321) chưa truyền dòng chi tiết đang có trên form vào phiếu in, nên phiếu mới hoặc đang sửa in theo dòng đã lưu hoặc dòng sinh lại</t>
+          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr"/>
@@ -21839,7 +21816,7 @@
       <c r="G8" s="13" t="inlineStr"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Phát hiện khi làm T112</t>
+          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
         </is>
       </c>
     </row>
@@ -21847,17 +21824,21 @@
       <c r="A9" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>T109</t>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>T101</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Sổ S2c-DNSN (5.2.8, TT58): bộ lọc Mặt hàng, Kho để mở sổ theo từng cặp mặt hàng – kho</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr"/>
+          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21867,7 +21848,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>T108 đang in cố định Thịt bò thăn, kho Phố Mây Lê Lợi. `CauHinhBC.loc` chưa đổi theo chế độ, lọc thêm sẽ hiện cả ở TT133, TT99</t>
+          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
         </is>
       </c>
     </row>
@@ -21877,25 +21858,29 @@
       </c>
       <c r="B10" s="25" t="inlineStr">
         <is>
-          <t>T110</t>
+          <t>T60</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>TT58: tên sổ ghi trong phần Hạch toán của phiếu (`soTT58` ở `tien/index.ts`, `ban-hang`, `kho`, `mua-hang`) theo bộ sổ TT58 (Sổ chi tiết tiền S2d thay Sổ quỹ tiền mặt, Sổ tiền gửi ngân hàng); tờ khai GTGT, Thông tin đơn vị đọc phương pháp thuế GTGT từ `s.ppGtgt` thay vì suy từ chế độ</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>Chờ</t>
+          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Dở dang</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr"/>
       <c r="G10" s="13" t="inlineStr"/>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Tách từ T108. `ToKhaiGTGT.tsx:18` còn `s.cheDo === 'TT58'`</t>
+          <t>11/10/2026 PhuongXT chốt gói Free không giới hạn chi nhánh (làm cùng T138): đã sửa mô tả gói Free, điểm nổi bật, câu hỏi đáp màn Gói thuê bao. Gói Standard còn ghi "1 điểm bán", chưa chốt</t>
         </is>
       </c>
     </row>
@@ -21903,19 +21888,19 @@
       <c r="A11" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>T101</t>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>T02</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Chuyển tiện ích về phân hệ của nó (tiện ích của phân hệ nào nằm trong phân hệ đó); tiện ích chung như Thiết kế mẫu in tính sau. Rồi xem lại có mở phân hệ Tiện ích cho gói Free không</t>
+          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
@@ -21925,11 +21910,7 @@
       </c>
       <c r="F11" s="16" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Ý của PhuongXT 10/10/2026, khi làm T100. Gói Free đang ẩn tạm phân hệ Tiện ích</t>
-        </is>
-      </c>
+      <c r="H11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n">
@@ -21937,29 +21918,25 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>T60</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>Mô tả gói Free, Standard trong `GOI` (`src/app/plan.ts`) đang ghi "1 điểm bán"; theo Roadmap gói Free là mỗi chi nhánh một kho, không giới hạn một chi nhánh. Chốt câu chữ rồi sửa</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>PhuongXT</t>
-        </is>
-      </c>
-      <c r="E12" s="28" t="inlineStr">
-        <is>
-          <t>Dở dang</t>
+          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr"/>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>Chờ</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr"/>
       <c r="G12" s="13" t="inlineStr"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>11/10/2026 PhuongXT chốt gói Free không giới hạn chi nhánh (làm cùng T138): đã sửa mô tả gói Free, điểm nổi bật, câu hỏi đáp màn Gói thuê bao. Gói Standard còn ghi "1 điểm bán", chưa chốt</t>
+          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
         </is>
       </c>
     </row>
@@ -21967,21 +21944,17 @@
       <c r="A13" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>T02</t>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>T33</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Chốt nghiệp vụ trên từng sơ đồ Quy trình: ô nào, nối thế nào, câu chữ. Sửa ở `src/modules/&lt;phân hệ&gt;/quy-trinh.ts`</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>Trum</t>
-        </is>
-      </c>
+          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="23" t="inlineStr">
         <is>
           <t>Chờ</t>
@@ -21989,7 +21962,11 @@
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Chỉ máy Trum chạy được script</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="n">
@@ -21997,12 +21974,12 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Nối sổ quỹ, sổ tài khoản 2.2.2, sổ ngân hàng 2.2.3, sổ công nợ 2.2.5 vào `so-cai.ts` để mọi sổ khớp báo cáo tài chính</t>
+          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr"/>
@@ -22015,7 +21992,7 @@
       <c r="G14" s="13" t="inlineStr"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Sổ quỹ đang tính riêng từ tiền mặt FABi từng chi nhánh. Tổng 3 quỹ chưa bằng dư TK 1111 trên cân đối kế toán</t>
+          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
         </is>
       </c>
     </row>
@@ -22023,14 +22000,14 @@
       <c r="A15" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>T33</t>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>T05</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Cập nhật Excel tính năng theo sheet Roadmap rồi chạy lại `tools/xuat_tinh_nang.py`: 1.12 và 2.2.3 có ở gói Free; thêm 1.17, S1a-HKD, S2a-HKD. Xong thì xoá các dòng tương ứng trong `THEO_ROADMAP` ở `src/app/plan.ts`</t>
+          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr"/>
@@ -22043,7 +22020,7 @@
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Chỉ máy Trum chạy được script</t>
+          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
         </is>
       </c>
     </row>
@@ -22053,12 +22030,12 @@
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="C16" s="13" t="inlineStr">
         <is>
-          <t>Kế toán trưởng duyệt mẫu sổ, báo cáo tài chính, tờ khai theo TT58, TT133, TT99. Sửa ký hiệu mẫu theo kết quả duyệt</t>
+          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr"/>
@@ -22069,24 +22046,20 @@
       </c>
       <c r="F16" s="12" t="inlineStr"/>
       <c r="G16" s="13" t="inlineStr"/>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>Ký hiệu mẫu (S03a-DNN, B01-DNN, 01/GTGT...) ghi theo hiểu biết, chưa đối chiếu văn bản gốc. Mẫu dạng tinh gọn TT58 chưa có. TT58 (T108) dựng theo bản dựng lại `D:\IACC-CLOUD\TT58`, cần đối chiếu Công báo số 323: 6 mục chi phí S2b, cột Nguyên giá S4b thuộc nhóm Ghi tăng hay Khấu hao, bố cục 01-TT, 02-TT; tỷ lệ % GTGT, TNDN nhóm ngành ở `tt58.ts` là tỷ lệ mẫu</t>
-        </is>
-      </c>
+      <c r="H16" s="13" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t>T05</t>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>T07</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Làm màn hoá đơn điện tử 3.1.5 riêng: danh sách theo trạng thái, ký số, gửi, huỷ, thay thế</t>
+          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr"/>
@@ -22099,7 +22072,7 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Hiện chưa có trạng thái phát hành, ký số, gửi cơ quan thuế. DB iPOS lưu trạng thái ở `SALE.EVAT_STATUS`: chưa ký, đã ký, đã gửi, đã xoá</t>
+          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
         </is>
       </c>
     </row>
@@ -22109,12 +22082,12 @@
       </c>
       <c r="B18" s="25" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>T08</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Thống nhất API với Dev (BR-18 trong spec DEV), thay `data/mock.ts` bằng lớp gọi API, giữ nguyên màn</t>
+          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr"/>
@@ -22125,20 +22098,24 @@
       </c>
       <c r="F18" s="12" t="inlineStr"/>
       <c r="G18" s="13" t="inlineStr"/>
-      <c r="H18" s="13" t="inlineStr"/>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="27" t="inlineStr">
-        <is>
-          <t>T07</t>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>T09</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo TSCĐ, CCDC làm khớp báo cáo tài chính</t>
+          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
@@ -22151,7 +22128,7 @@
       <c r="G19" s="5" t="inlineStr"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Đang dùng màn sổ chung, số sinh ngẫu nhiên theo hạt giống. T47 đã thêm thẻ TSCĐ, sổ theo dõi nơi sử dụng; số liệu TSCĐ, CCDC vẫn chưa nối sổ cái</t>
+          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
         </is>
       </c>
     </row>
@@ -22161,12 +22138,12 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>T08</t>
+          <t>T10</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Bảng kê mua vào 6.2.1, báo cáo mua hàng 4.2.1, bảng kê điều chuyển 3.2.4 làm màn riêng</t>
+          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
@@ -22179,7 +22156,7 @@
       <c r="G20" s="13" t="inlineStr"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Đang dùng bảng kê hoá đơn chung. T47 đã thêm bộ lọc, gom nhóm cho 4.2.1, 6.2.1, 3.2.4; màn riêng vẫn chưa làm</t>
+          <t>Hiện đường nối là nét đứt</t>
         </is>
       </c>
     </row>
@@ -22187,14 +22164,14 @@
       <c r="A21" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>T09</t>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>T11</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Form kiểm tra dữ liệu nhập. Nút Lưu thật sự lưu</t>
+          <t>Thuế TNDN tính đúng theo kỳ</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr"/>
@@ -22207,7 +22184,7 @@
       <c r="G21" s="5" t="inlineStr"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Hiện nút chỉ hiện thông báo. Chỉ màn đăng nhập có kiểm tra</t>
+          <t>Đang tạm tính 20% mỗi tháng</t>
         </is>
       </c>
     </row>
@@ -22217,12 +22194,12 @@
       </c>
       <c r="B22" s="25" t="inlineStr">
         <is>
-          <t>T10</t>
+          <t>T12</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Ô trên sơ đồ Quy trình hiện số đếm (vd "3 phiếu chưa ghi sổ"). Đường nối ô phụ có mũi tên chiều nghiệp vụ</t>
+          <t>Giao diện cho màn hẹp hơn 1280px</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
@@ -22235,7 +22212,7 @@
       <c r="G22" s="13" t="inlineStr"/>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Hiện đường nối là nét đứt</t>
+          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
         </is>
       </c>
     </row>
@@ -22243,14 +22220,14 @@
       <c r="A23" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>T11</t>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>T13</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Thuế TNDN tính đúng theo kỳ</t>
+          <t>Tách gói JS khi build</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr"/>
@@ -22263,7 +22240,7 @@
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Đang tạm tính 20% mỗi tháng</t>
+          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
         </is>
       </c>
     </row>
@@ -22273,12 +22250,12 @@
       </c>
       <c r="B24" s="25" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Giao diện cho màn hẹp hơn 1280px</t>
+          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr"/>
@@ -22291,7 +22268,7 @@
       <c r="G24" s="13" t="inlineStr"/>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Khung có min-width 1180px. Ở 1280px ô tìm kiếm trên thanh trên co còn khoảng 160px</t>
+          <t>Chưa có file logo iPOS</t>
         </is>
       </c>
     </row>
@@ -22299,14 +22276,14 @@
       <c r="A25" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="27" t="inlineStr">
-        <is>
-          <t>T13</t>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>T19</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Tách gói JS khi build</t>
+          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
@@ -22319,7 +22296,7 @@
       <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>`npm run build` cảnh báo gói JS hơn 500 kB</t>
+          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
         </is>
       </c>
     </row>
@@ -22329,12 +22306,12 @@
       </c>
       <c r="B26" s="25" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Thay biểu tượng chìa khoá ở nút "Đăng nhập bằng tài khoản iPOS" bằng logo iPOS</t>
+          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr"/>
@@ -22347,7 +22324,7 @@
       <c r="G26" s="13" t="inlineStr"/>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Chưa có file logo iPOS</t>
+          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
         </is>
       </c>
     </row>
@@ -22355,29 +22332,37 @@
       <c r="A27" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t>T19</t>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>T173</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Khoá sổ theo từng đơn vị, chi nhánh</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr"/>
-      <c r="E27" s="23" t="inlineStr">
-        <is>
-          <t>Chờ</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>DB iPOS lưu ngày khoá ở `DM_ORGANIZATION.DATE_LOCK`, màn Khoá sổ đang khoá chung</t>
-        </is>
-      </c>
+          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên (tên màn, chọn chi nhánh), thanh dưới 4 tab theo IVT Pro, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>[2026-10-13-trum-dien-thoai-dot-1](nhat-ky/2026-10-13-trum-dien-thoai-dot-1.md)</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n">
@@ -22385,33 +22370,41 @@
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>T172</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Cột trạng thái duyệt trong danh sách chứng từ, tách khỏi ghi sổ</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr"/>
-      <c r="E28" s="23" t="inlineStr">
-        <is>
-          <t>Chờ</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr"/>
-      <c r="G28" s="13" t="inlineStr"/>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>DB iPOS có `REVIEW_STATUS` CHECKED/UNCHECKED riêng với `STATUS` DRAFT/POSTED</t>
-        </is>
-      </c>
+          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>PhuongXT</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>[2026-10-13-phuongxt-xuat-excel](nhat-ky/2026-10-13-phuongxt-xuat-excel.md)</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>T174</t>
         </is>
@@ -22426,7 +22419,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E29" s="29" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22462,7 +22455,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E30" s="29" t="inlineStr">
+      <c r="E30" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22483,7 +22476,7 @@
       <c r="A31" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="27" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>T170</t>
         </is>
@@ -22498,7 +22491,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E31" s="29" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22534,7 +22527,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E32" s="29" t="inlineStr">
+      <c r="E32" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22555,7 +22548,7 @@
       <c r="A33" s="16" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="27" t="inlineStr">
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>T165</t>
         </is>
@@ -22570,7 +22563,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E33" s="29" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22606,7 +22599,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E34" s="29" t="inlineStr">
+      <c r="E34" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22627,7 +22620,7 @@
       <c r="A35" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="27" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>T166</t>
         </is>
@@ -22642,7 +22635,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E35" s="29" t="inlineStr">
+      <c r="E35" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22678,7 +22671,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E36" s="29" t="inlineStr">
+      <c r="E36" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22699,7 +22692,7 @@
       <c r="A37" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="27" t="inlineStr">
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>T163</t>
         </is>
@@ -22714,7 +22707,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E37" s="29" t="inlineStr">
+      <c r="E37" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22750,7 +22743,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E38" s="29" t="inlineStr">
+      <c r="E38" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22771,7 +22764,7 @@
       <c r="A39" s="16" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="27" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>T161</t>
         </is>
@@ -22786,7 +22779,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E39" s="29" t="inlineStr">
+      <c r="E39" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22822,7 +22815,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E40" s="29" t="inlineStr">
+      <c r="E40" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22843,7 +22836,7 @@
       <c r="A41" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="27" t="inlineStr">
+      <c r="B41" s="26" t="inlineStr">
         <is>
           <t>T159</t>
         </is>
@@ -22858,7 +22851,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E41" s="29" t="inlineStr">
+      <c r="E41" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22894,7 +22887,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E42" s="29" t="inlineStr">
+      <c r="E42" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22915,7 +22908,7 @@
       <c r="A43" s="16" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="27" t="inlineStr">
+      <c r="B43" s="26" t="inlineStr">
         <is>
           <t>T155</t>
         </is>
@@ -22930,7 +22923,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E43" s="29" t="inlineStr">
+      <c r="E43" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22966,7 +22959,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E44" s="29" t="inlineStr">
+      <c r="E44" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -22987,7 +22980,7 @@
       <c r="A45" s="16" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="27" t="inlineStr">
+      <c r="B45" s="26" t="inlineStr">
         <is>
           <t>T154</t>
         </is>
@@ -23002,7 +22995,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E45" s="29" t="inlineStr">
+      <c r="E45" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23038,7 +23031,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E46" s="29" t="inlineStr">
+      <c r="E46" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23059,7 +23052,7 @@
       <c r="A47" s="16" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="27" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>T150</t>
         </is>
@@ -23074,7 +23067,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E47" s="29" t="inlineStr">
+      <c r="E47" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23110,7 +23103,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E48" s="29" t="inlineStr">
+      <c r="E48" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23131,7 +23124,7 @@
       <c r="A49" s="16" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="27" t="inlineStr">
+      <c r="B49" s="26" t="inlineStr">
         <is>
           <t>T151</t>
         </is>
@@ -23146,7 +23139,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E49" s="29" t="inlineStr">
+      <c r="E49" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23182,7 +23175,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E50" s="29" t="inlineStr">
+      <c r="E50" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23203,7 +23196,7 @@
       <c r="A51" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="27" t="inlineStr">
+      <c r="B51" s="26" t="inlineStr">
         <is>
           <t>T149</t>
         </is>
@@ -23218,7 +23211,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E51" s="29" t="inlineStr">
+      <c r="E51" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23254,7 +23247,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E52" s="29" t="inlineStr">
+      <c r="E52" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23275,7 +23268,7 @@
       <c r="A53" s="16" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="27" t="inlineStr">
+      <c r="B53" s="26" t="inlineStr">
         <is>
           <t>T147</t>
         </is>
@@ -23290,7 +23283,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E53" s="29" t="inlineStr">
+      <c r="E53" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23326,7 +23319,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E54" s="29" t="inlineStr">
+      <c r="E54" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23347,7 +23340,7 @@
       <c r="A55" s="16" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="27" t="inlineStr">
+      <c r="B55" s="26" t="inlineStr">
         <is>
           <t>T145</t>
         </is>
@@ -23362,7 +23355,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E55" s="29" t="inlineStr">
+      <c r="E55" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23398,7 +23391,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E56" s="29" t="inlineStr">
+      <c r="E56" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23419,7 +23412,7 @@
       <c r="A57" s="16" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="27" t="inlineStr">
+      <c r="B57" s="26" t="inlineStr">
         <is>
           <t>T143</t>
         </is>
@@ -23434,7 +23427,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E57" s="29" t="inlineStr">
+      <c r="E57" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23470,7 +23463,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E58" s="29" t="inlineStr">
+      <c r="E58" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23491,7 +23484,7 @@
       <c r="A59" s="16" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="27" t="inlineStr">
+      <c r="B59" s="26" t="inlineStr">
         <is>
           <t>T141</t>
         </is>
@@ -23506,7 +23499,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E59" s="29" t="inlineStr">
+      <c r="E59" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23542,7 +23535,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E60" s="29" t="inlineStr">
+      <c r="E60" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23563,7 +23556,7 @@
       <c r="A61" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="27" t="inlineStr">
+      <c r="B61" s="26" t="inlineStr">
         <is>
           <t>T137</t>
         </is>
@@ -23578,7 +23571,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E61" s="29" t="inlineStr">
+      <c r="E61" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23614,7 +23607,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E62" s="29" t="inlineStr">
+      <c r="E62" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23635,7 +23628,7 @@
       <c r="A63" s="16" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="27" t="inlineStr">
+      <c r="B63" s="26" t="inlineStr">
         <is>
           <t>T134</t>
         </is>
@@ -23650,7 +23643,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E63" s="29" t="inlineStr">
+      <c r="E63" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23686,7 +23679,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E64" s="29" t="inlineStr">
+      <c r="E64" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23707,7 +23700,7 @@
       <c r="A65" s="16" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="27" t="inlineStr">
+      <c r="B65" s="26" t="inlineStr">
         <is>
           <t>T132</t>
         </is>
@@ -23722,7 +23715,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E65" s="29" t="inlineStr">
+      <c r="E65" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23758,7 +23751,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E66" s="29" t="inlineStr">
+      <c r="E66" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23779,7 +23772,7 @@
       <c r="A67" s="16" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="27" t="inlineStr">
+      <c r="B67" s="26" t="inlineStr">
         <is>
           <t>T130</t>
         </is>
@@ -23794,7 +23787,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E67" s="29" t="inlineStr">
+      <c r="E67" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23830,7 +23823,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E68" s="29" t="inlineStr">
+      <c r="E68" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23851,7 +23844,7 @@
       <c r="A69" s="16" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="27" t="inlineStr">
+      <c r="B69" s="26" t="inlineStr">
         <is>
           <t>T128</t>
         </is>
@@ -23866,7 +23859,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E69" s="29" t="inlineStr">
+      <c r="E69" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23902,7 +23895,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E70" s="29" t="inlineStr">
+      <c r="E70" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23923,7 +23916,7 @@
       <c r="A71" s="16" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="27" t="inlineStr">
+      <c r="B71" s="26" t="inlineStr">
         <is>
           <t>T126</t>
         </is>
@@ -23938,7 +23931,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E71" s="29" t="inlineStr">
+      <c r="E71" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23974,7 +23967,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E72" s="29" t="inlineStr">
+      <c r="E72" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -23995,7 +23988,7 @@
       <c r="A73" s="16" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="27" t="inlineStr">
+      <c r="B73" s="26" t="inlineStr">
         <is>
           <t>T124</t>
         </is>
@@ -24010,7 +24003,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E73" s="29" t="inlineStr">
+      <c r="E73" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24046,7 +24039,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E74" s="29" t="inlineStr">
+      <c r="E74" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24067,7 +24060,7 @@
       <c r="A75" s="16" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="27" t="inlineStr">
+      <c r="B75" s="26" t="inlineStr">
         <is>
           <t>T122</t>
         </is>
@@ -24082,7 +24075,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E75" s="29" t="inlineStr">
+      <c r="E75" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24118,7 +24111,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E76" s="29" t="inlineStr">
+      <c r="E76" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24139,7 +24132,7 @@
       <c r="A77" s="16" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="27" t="inlineStr">
+      <c r="B77" s="26" t="inlineStr">
         <is>
           <t>T111</t>
         </is>
@@ -24154,7 +24147,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E77" s="29" t="inlineStr">
+      <c r="E77" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24190,7 +24183,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E78" s="29" t="inlineStr">
+      <c r="E78" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24211,7 +24204,7 @@
       <c r="A79" s="16" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="27" t="inlineStr">
+      <c r="B79" s="26" t="inlineStr">
         <is>
           <t>T118</t>
         </is>
@@ -24226,7 +24219,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E79" s="29" t="inlineStr">
+      <c r="E79" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24262,7 +24255,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E80" s="29" t="inlineStr">
+      <c r="E80" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24283,7 +24276,7 @@
       <c r="A81" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="B81" s="27" t="inlineStr">
+      <c r="B81" s="26" t="inlineStr">
         <is>
           <t>T116</t>
         </is>
@@ -24298,7 +24291,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E81" s="29" t="inlineStr">
+      <c r="E81" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24334,7 +24327,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E82" s="29" t="inlineStr">
+      <c r="E82" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24355,7 +24348,7 @@
       <c r="A83" s="16" t="n">
         <v>82</v>
       </c>
-      <c r="B83" s="27" t="inlineStr">
+      <c r="B83" s="26" t="inlineStr">
         <is>
           <t>T114</t>
         </is>
@@ -24370,7 +24363,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E83" s="29" t="inlineStr">
+      <c r="E83" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24406,7 +24399,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E84" s="29" t="inlineStr">
+      <c r="E84" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24427,7 +24420,7 @@
       <c r="A85" s="16" t="n">
         <v>84</v>
       </c>
-      <c r="B85" s="27" t="inlineStr">
+      <c r="B85" s="26" t="inlineStr">
         <is>
           <t>T119</t>
         </is>
@@ -24442,7 +24435,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E85" s="29" t="inlineStr">
+      <c r="E85" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24478,7 +24471,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E86" s="29" t="inlineStr">
+      <c r="E86" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24499,7 +24492,7 @@
       <c r="A87" s="16" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="27" t="inlineStr">
+      <c r="B87" s="26" t="inlineStr">
         <is>
           <t>T107</t>
         </is>
@@ -24514,7 +24507,7 @@
           <t>dinhlanphuongipacc</t>
         </is>
       </c>
-      <c r="E87" s="29" t="inlineStr">
+      <c r="E87" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24550,7 +24543,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E88" s="29" t="inlineStr">
+      <c r="E88" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24571,7 +24564,7 @@
       <c r="A89" s="16" t="n">
         <v>88</v>
       </c>
-      <c r="B89" s="27" t="inlineStr">
+      <c r="B89" s="26" t="inlineStr">
         <is>
           <t>T103</t>
         </is>
@@ -24586,7 +24579,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E89" s="29" t="inlineStr">
+      <c r="E89" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24622,7 +24615,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E90" s="29" t="inlineStr">
+      <c r="E90" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24643,7 +24636,7 @@
       <c r="A91" s="16" t="n">
         <v>90</v>
       </c>
-      <c r="B91" s="27" t="inlineStr">
+      <c r="B91" s="26" t="inlineStr">
         <is>
           <t>T104</t>
         </is>
@@ -24658,7 +24651,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E91" s="29" t="inlineStr">
+      <c r="E91" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24694,7 +24687,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E92" s="29" t="inlineStr">
+      <c r="E92" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24715,7 +24708,7 @@
       <c r="A93" s="16" t="n">
         <v>92</v>
       </c>
-      <c r="B93" s="27" t="inlineStr">
+      <c r="B93" s="26" t="inlineStr">
         <is>
           <t>T100</t>
         </is>
@@ -24730,7 +24723,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E93" s="29" t="inlineStr">
+      <c r="E93" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24766,7 +24759,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E94" s="29" t="inlineStr">
+      <c r="E94" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24787,7 +24780,7 @@
       <c r="A95" s="16" t="n">
         <v>94</v>
       </c>
-      <c r="B95" s="27" t="inlineStr">
+      <c r="B95" s="26" t="inlineStr">
         <is>
           <t>T98</t>
         </is>
@@ -24802,7 +24795,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E95" s="29" t="inlineStr">
+      <c r="E95" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24838,7 +24831,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E96" s="29" t="inlineStr">
+      <c r="E96" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24859,7 +24852,7 @@
       <c r="A97" s="16" t="n">
         <v>96</v>
       </c>
-      <c r="B97" s="27" t="inlineStr">
+      <c r="B97" s="26" t="inlineStr">
         <is>
           <t>T96</t>
         </is>
@@ -24874,7 +24867,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E97" s="29" t="inlineStr">
+      <c r="E97" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24910,7 +24903,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E98" s="29" t="inlineStr">
+      <c r="E98" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24931,7 +24924,7 @@
       <c r="A99" s="16" t="n">
         <v>98</v>
       </c>
-      <c r="B99" s="27" t="inlineStr">
+      <c r="B99" s="26" t="inlineStr">
         <is>
           <t>T94</t>
         </is>
@@ -24946,7 +24939,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E99" s="29" t="inlineStr">
+      <c r="E99" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -24982,7 +24975,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E100" s="29" t="inlineStr">
+      <c r="E100" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25003,7 +24996,7 @@
       <c r="A101" s="16" t="n">
         <v>100</v>
       </c>
-      <c r="B101" s="27" t="inlineStr">
+      <c r="B101" s="26" t="inlineStr">
         <is>
           <t>T92</t>
         </is>
@@ -25018,7 +25011,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E101" s="29" t="inlineStr">
+      <c r="E101" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25054,7 +25047,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E102" s="29" t="inlineStr">
+      <c r="E102" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25075,7 +25068,7 @@
       <c r="A103" s="16" t="n">
         <v>102</v>
       </c>
-      <c r="B103" s="27" t="inlineStr">
+      <c r="B103" s="26" t="inlineStr">
         <is>
           <t>T90</t>
         </is>
@@ -25090,7 +25083,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E103" s="29" t="inlineStr">
+      <c r="E103" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25126,7 +25119,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E104" s="29" t="inlineStr">
+      <c r="E104" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25147,7 +25140,7 @@
       <c r="A105" s="16" t="n">
         <v>104</v>
       </c>
-      <c r="B105" s="27" t="inlineStr">
+      <c r="B105" s="26" t="inlineStr">
         <is>
           <t>T88</t>
         </is>
@@ -25162,7 +25155,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E105" s="29" t="inlineStr">
+      <c r="E105" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25198,7 +25191,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E106" s="29" t="inlineStr">
+      <c r="E106" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25219,7 +25212,7 @@
       <c r="A107" s="16" t="n">
         <v>106</v>
       </c>
-      <c r="B107" s="27" t="inlineStr">
+      <c r="B107" s="26" t="inlineStr">
         <is>
           <t>T87</t>
         </is>
@@ -25234,7 +25227,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E107" s="29" t="inlineStr">
+      <c r="E107" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25270,7 +25263,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E108" s="29" t="inlineStr">
+      <c r="E108" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25291,7 +25284,7 @@
       <c r="A109" s="16" t="n">
         <v>108</v>
       </c>
-      <c r="B109" s="27" t="inlineStr">
+      <c r="B109" s="26" t="inlineStr">
         <is>
           <t>T86</t>
         </is>
@@ -25306,7 +25299,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E109" s="29" t="inlineStr">
+      <c r="E109" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25342,7 +25335,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E110" s="29" t="inlineStr">
+      <c r="E110" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25363,7 +25356,7 @@
       <c r="A111" s="16" t="n">
         <v>110</v>
       </c>
-      <c r="B111" s="27" t="inlineStr">
+      <c r="B111" s="26" t="inlineStr">
         <is>
           <t>T84</t>
         </is>
@@ -25378,7 +25371,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E111" s="29" t="inlineStr">
+      <c r="E111" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25414,7 +25407,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E112" s="29" t="inlineStr">
+      <c r="E112" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25435,7 +25428,7 @@
       <c r="A113" s="16" t="n">
         <v>112</v>
       </c>
-      <c r="B113" s="27" t="inlineStr">
+      <c r="B113" s="26" t="inlineStr">
         <is>
           <t>T82</t>
         </is>
@@ -25450,7 +25443,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E113" s="29" t="inlineStr">
+      <c r="E113" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25486,7 +25479,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E114" s="29" t="inlineStr">
+      <c r="E114" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25507,7 +25500,7 @@
       <c r="A115" s="16" t="n">
         <v>114</v>
       </c>
-      <c r="B115" s="27" t="inlineStr">
+      <c r="B115" s="26" t="inlineStr">
         <is>
           <t>T81</t>
         </is>
@@ -25522,7 +25515,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E115" s="29" t="inlineStr">
+      <c r="E115" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25558,7 +25551,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E116" s="29" t="inlineStr">
+      <c r="E116" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25579,7 +25572,7 @@
       <c r="A117" s="16" t="n">
         <v>116</v>
       </c>
-      <c r="B117" s="27" t="inlineStr">
+      <c r="B117" s="26" t="inlineStr">
         <is>
           <t>T70</t>
         </is>
@@ -25594,7 +25587,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E117" s="29" t="inlineStr">
+      <c r="E117" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25630,7 +25623,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E118" s="29" t="inlineStr">
+      <c r="E118" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25651,7 +25644,7 @@
       <c r="A119" s="16" t="n">
         <v>118</v>
       </c>
-      <c r="B119" s="27" t="inlineStr">
+      <c r="B119" s="26" t="inlineStr">
         <is>
           <t>T78</t>
         </is>
@@ -25666,7 +25659,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E119" s="29" t="inlineStr">
+      <c r="E119" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25702,7 +25695,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E120" s="29" t="inlineStr">
+      <c r="E120" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25723,7 +25716,7 @@
       <c r="A121" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="B121" s="27" t="inlineStr">
+      <c r="B121" s="26" t="inlineStr">
         <is>
           <t>T69</t>
         </is>
@@ -25738,7 +25731,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E121" s="29" t="inlineStr">
+      <c r="E121" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25774,7 +25767,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E122" s="29" t="inlineStr">
+      <c r="E122" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25795,7 +25788,7 @@
       <c r="A123" s="16" t="n">
         <v>122</v>
       </c>
-      <c r="B123" s="27" t="inlineStr">
+      <c r="B123" s="26" t="inlineStr">
         <is>
           <t>T74</t>
         </is>
@@ -25810,7 +25803,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E123" s="29" t="inlineStr">
+      <c r="E123" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25846,7 +25839,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E124" s="29" t="inlineStr">
+      <c r="E124" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25867,7 +25860,7 @@
       <c r="A125" s="16" t="n">
         <v>124</v>
       </c>
-      <c r="B125" s="27" t="inlineStr">
+      <c r="B125" s="26" t="inlineStr">
         <is>
           <t>T71</t>
         </is>
@@ -25882,7 +25875,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E125" s="29" t="inlineStr">
+      <c r="E125" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25918,7 +25911,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E126" s="29" t="inlineStr">
+      <c r="E126" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25939,7 +25932,7 @@
       <c r="A127" s="16" t="n">
         <v>126</v>
       </c>
-      <c r="B127" s="27" t="inlineStr">
+      <c r="B127" s="26" t="inlineStr">
         <is>
           <t>T59</t>
         </is>
@@ -25954,7 +25947,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E127" s="29" t="inlineStr">
+      <c r="E127" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -25990,7 +25983,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E128" s="29" t="inlineStr">
+      <c r="E128" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26011,7 +26004,7 @@
       <c r="A129" s="16" t="n">
         <v>128</v>
       </c>
-      <c r="B129" s="27" t="inlineStr">
+      <c r="B129" s="26" t="inlineStr">
         <is>
           <t>T67</t>
         </is>
@@ -26026,7 +26019,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E129" s="29" t="inlineStr">
+      <c r="E129" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26062,7 +26055,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E130" s="29" t="inlineStr">
+      <c r="E130" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26083,7 +26076,7 @@
       <c r="A131" s="16" t="n">
         <v>130</v>
       </c>
-      <c r="B131" s="27" t="inlineStr">
+      <c r="B131" s="26" t="inlineStr">
         <is>
           <t>T65</t>
         </is>
@@ -26098,7 +26091,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E131" s="29" t="inlineStr">
+      <c r="E131" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26134,7 +26127,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E132" s="29" t="inlineStr">
+      <c r="E132" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26155,7 +26148,7 @@
       <c r="A133" s="16" t="n">
         <v>132</v>
       </c>
-      <c r="B133" s="27" t="inlineStr">
+      <c r="B133" s="26" t="inlineStr">
         <is>
           <t>T63</t>
         </is>
@@ -26170,7 +26163,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E133" s="29" t="inlineStr">
+      <c r="E133" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26206,7 +26199,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E134" s="29" t="inlineStr">
+      <c r="E134" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26227,7 +26220,7 @@
       <c r="A135" s="16" t="n">
         <v>134</v>
       </c>
-      <c r="B135" s="27" t="inlineStr">
+      <c r="B135" s="26" t="inlineStr">
         <is>
           <t>T61</t>
         </is>
@@ -26242,7 +26235,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E135" s="29" t="inlineStr">
+      <c r="E135" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26278,7 +26271,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E136" s="29" t="inlineStr">
+      <c r="E136" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26299,7 +26292,7 @@
       <c r="A137" s="16" t="n">
         <v>136</v>
       </c>
-      <c r="B137" s="27" t="inlineStr">
+      <c r="B137" s="26" t="inlineStr">
         <is>
           <t>T56</t>
         </is>
@@ -26314,7 +26307,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E137" s="29" t="inlineStr">
+      <c r="E137" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26350,7 +26343,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E138" s="29" t="inlineStr">
+      <c r="E138" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26371,7 +26364,7 @@
       <c r="A139" s="16" t="n">
         <v>138</v>
       </c>
-      <c r="B139" s="27" t="inlineStr">
+      <c r="B139" s="26" t="inlineStr">
         <is>
           <t>T55</t>
         </is>
@@ -26386,7 +26379,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E139" s="29" t="inlineStr">
+      <c r="E139" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26422,7 +26415,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E140" s="29" t="inlineStr">
+      <c r="E140" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26443,7 +26436,7 @@
       <c r="A141" s="16" t="n">
         <v>140</v>
       </c>
-      <c r="B141" s="27" t="inlineStr">
+      <c r="B141" s="26" t="inlineStr">
         <is>
           <t>T53</t>
         </is>
@@ -26458,7 +26451,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E141" s="29" t="inlineStr">
+      <c r="E141" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26494,7 +26487,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E142" s="29" t="inlineStr">
+      <c r="E142" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26515,7 +26508,7 @@
       <c r="A143" s="16" t="n">
         <v>142</v>
       </c>
-      <c r="B143" s="27" t="inlineStr">
+      <c r="B143" s="26" t="inlineStr">
         <is>
           <t>T51</t>
         </is>
@@ -26530,7 +26523,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E143" s="29" t="inlineStr">
+      <c r="E143" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26566,7 +26559,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E144" s="29" t="inlineStr">
+      <c r="E144" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26587,7 +26580,7 @@
       <c r="A145" s="16" t="n">
         <v>144</v>
       </c>
-      <c r="B145" s="27" t="inlineStr">
+      <c r="B145" s="26" t="inlineStr">
         <is>
           <t>T47</t>
         </is>
@@ -26602,7 +26595,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E145" s="29" t="inlineStr">
+      <c r="E145" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26638,7 +26631,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E146" s="29" t="inlineStr">
+      <c r="E146" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26659,7 +26652,7 @@
       <c r="A147" s="16" t="n">
         <v>146</v>
       </c>
-      <c r="B147" s="27" t="inlineStr">
+      <c r="B147" s="26" t="inlineStr">
         <is>
           <t>T48</t>
         </is>
@@ -26674,7 +26667,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E147" s="29" t="inlineStr">
+      <c r="E147" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26710,7 +26703,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E148" s="29" t="inlineStr">
+      <c r="E148" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26731,7 +26724,7 @@
       <c r="A149" s="16" t="n">
         <v>148</v>
       </c>
-      <c r="B149" s="27" t="inlineStr">
+      <c r="B149" s="26" t="inlineStr">
         <is>
           <t>T43</t>
         </is>
@@ -26746,7 +26739,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E149" s="29" t="inlineStr">
+      <c r="E149" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26782,7 +26775,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E150" s="29" t="inlineStr">
+      <c r="E150" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26803,7 +26796,7 @@
       <c r="A151" s="16" t="n">
         <v>150</v>
       </c>
-      <c r="B151" s="27" t="inlineStr">
+      <c r="B151" s="26" t="inlineStr">
         <is>
           <t>T44</t>
         </is>
@@ -26818,7 +26811,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E151" s="29" t="inlineStr">
+      <c r="E151" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26854,7 +26847,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E152" s="29" t="inlineStr">
+      <c r="E152" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26875,7 +26868,7 @@
       <c r="A153" s="16" t="n">
         <v>152</v>
       </c>
-      <c r="B153" s="27" t="inlineStr">
+      <c r="B153" s="26" t="inlineStr">
         <is>
           <t>T41</t>
         </is>
@@ -26890,7 +26883,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E153" s="29" t="inlineStr">
+      <c r="E153" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26926,7 +26919,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E154" s="29" t="inlineStr">
+      <c r="E154" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26947,7 +26940,7 @@
       <c r="A155" s="16" t="n">
         <v>154</v>
       </c>
-      <c r="B155" s="27" t="inlineStr">
+      <c r="B155" s="26" t="inlineStr">
         <is>
           <t>T39</t>
         </is>
@@ -26962,7 +26955,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E155" s="29" t="inlineStr">
+      <c r="E155" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -26998,7 +26991,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E156" s="29" t="inlineStr">
+      <c r="E156" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27019,7 +27012,7 @@
       <c r="A157" s="16" t="n">
         <v>156</v>
       </c>
-      <c r="B157" s="27" t="inlineStr">
+      <c r="B157" s="26" t="inlineStr">
         <is>
           <t>T37</t>
         </is>
@@ -27034,7 +27027,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E157" s="29" t="inlineStr">
+      <c r="E157" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27070,7 +27063,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E158" s="29" t="inlineStr">
+      <c r="E158" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27091,7 +27084,7 @@
       <c r="A159" s="16" t="n">
         <v>158</v>
       </c>
-      <c r="B159" s="27" t="inlineStr">
+      <c r="B159" s="26" t="inlineStr">
         <is>
           <t>T32</t>
         </is>
@@ -27106,7 +27099,7 @@
           <t>PhuongXT</t>
         </is>
       </c>
-      <c r="E159" s="29" t="inlineStr">
+      <c r="E159" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27142,7 +27135,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E160" s="29" t="inlineStr">
+      <c r="E160" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27163,7 +27156,7 @@
       <c r="A161" s="16" t="n">
         <v>160</v>
       </c>
-      <c r="B161" s="27" t="inlineStr">
+      <c r="B161" s="26" t="inlineStr">
         <is>
           <t>T30</t>
         </is>
@@ -27178,7 +27171,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E161" s="29" t="inlineStr">
+      <c r="E161" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27214,7 +27207,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E162" s="29" t="inlineStr">
+      <c r="E162" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27235,7 +27228,7 @@
       <c r="A163" s="16" t="n">
         <v>162</v>
       </c>
-      <c r="B163" s="27" t="inlineStr">
+      <c r="B163" s="26" t="inlineStr">
         <is>
           <t>T35</t>
         </is>
@@ -27250,7 +27243,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E163" s="29" t="inlineStr">
+      <c r="E163" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27286,7 +27279,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E164" s="29" t="inlineStr">
+      <c r="E164" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27307,7 +27300,7 @@
       <c r="A165" s="16" t="n">
         <v>164</v>
       </c>
-      <c r="B165" s="27" t="inlineStr">
+      <c r="B165" s="26" t="inlineStr">
         <is>
           <t>T29</t>
         </is>
@@ -27322,7 +27315,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E165" s="29" t="inlineStr">
+      <c r="E165" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27358,7 +27351,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E166" s="29" t="inlineStr">
+      <c r="E166" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27379,7 +27372,7 @@
       <c r="A167" s="16" t="n">
         <v>166</v>
       </c>
-      <c r="B167" s="27" t="inlineStr">
+      <c r="B167" s="26" t="inlineStr">
         <is>
           <t>T26</t>
         </is>
@@ -27394,7 +27387,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E167" s="29" t="inlineStr">
+      <c r="E167" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27430,7 +27423,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E168" s="29" t="inlineStr">
+      <c r="E168" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27451,7 +27444,7 @@
       <c r="A169" s="16" t="n">
         <v>168</v>
       </c>
-      <c r="B169" s="27" t="inlineStr">
+      <c r="B169" s="26" t="inlineStr">
         <is>
           <t>T25</t>
         </is>
@@ -27466,7 +27459,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E169" s="29" t="inlineStr">
+      <c r="E169" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27502,7 +27495,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E170" s="29" t="inlineStr">
+      <c r="E170" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27523,7 +27516,7 @@
       <c r="A171" s="16" t="n">
         <v>170</v>
       </c>
-      <c r="B171" s="27" t="inlineStr">
+      <c r="B171" s="26" t="inlineStr">
         <is>
           <t>T15</t>
         </is>
@@ -27538,7 +27531,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E171" s="29" t="inlineStr">
+      <c r="E171" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27574,7 +27567,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E172" s="29" t="inlineStr">
+      <c r="E172" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27595,7 +27588,7 @@
       <c r="A173" s="16" t="n">
         <v>172</v>
       </c>
-      <c r="B173" s="27" t="inlineStr">
+      <c r="B173" s="26" t="inlineStr">
         <is>
           <t>T17</t>
         </is>
@@ -27610,7 +27603,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E173" s="29" t="inlineStr">
+      <c r="E173" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27646,7 +27639,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E174" s="29" t="inlineStr">
+      <c r="E174" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27667,7 +27660,7 @@
       <c r="A175" s="16" t="n">
         <v>174</v>
       </c>
-      <c r="B175" s="27" t="inlineStr">
+      <c r="B175" s="26" t="inlineStr">
         <is>
           <t>T22</t>
         </is>
@@ -27682,7 +27675,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E175" s="29" t="inlineStr">
+      <c r="E175" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27718,7 +27711,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E176" s="29" t="inlineStr">
+      <c r="E176" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
@@ -27739,7 +27732,7 @@
       <c r="A177" s="16" t="n">
         <v>176</v>
       </c>
-      <c r="B177" s="27" t="inlineStr">
+      <c r="B177" s="26" t="inlineStr">
         <is>
           <t>T18</t>
         </is>
@@ -27754,7 +27747,7 @@
           <t>Trum</t>
         </is>
       </c>
-      <c r="E177" s="29" t="inlineStr">
+      <c r="E177" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>

</xml_diff>

<commit_message>
T175: giao diện điện thoại đợt 2, Trang chủ, Nghiệp vụ, Khác, thanh dưới nổi theo số đo IVT
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$L$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$178</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -847,7 +847,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>176 việc (T01 - T108)</t>
+          <t>177 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>151 việc (85.8%)</t>
+          <t>152 việc (85.9%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21565,7 +21565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H177"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22334,12 +22334,12 @@
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>T173</t>
+          <t>T175</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên (tên màn, chọn chi nhánh), thanh dưới 4 tab theo IVT Pro, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
+          <t>Điện thoại đợt 2: Trang chủ (thao tác nhanh, thẻ số liệu), Nghiệp vụ (lưới phân hệ, danh sách màn), Khác (tài khoản, danh mục, hệ thống, đơn vị, gói, đăng xuất); số đo IVT, thanh dưới nổi</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-13-trum-dien-thoai-dot-1](nhat-ky/2026-10-13-trum-dien-thoai-dot-1.md)</t>
+          <t>[2026-10-13-trum-dien-thoai-dot-2](nhat-ky/2026-10-13-trum-dien-thoai-dot-2.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -22370,17 +22370,17 @@
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>T172</t>
+          <t>T173</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
+          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên (tên màn, chọn chi nhánh), thanh dưới 4 tab theo IVT Pro, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E28" s="28" t="inlineStr">
@@ -22395,7 +22395,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-xuat-excel](nhat-ky/2026-10-13-phuongxt-xuat-excel.md)</t>
+          <t>[2026-10-13-trum-dien-thoai-dot-1](nhat-ky/2026-10-13-trum-dien-thoai-dot-1.md)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -22406,12 +22406,12 @@
       </c>
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>T174</t>
+          <t>T172</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Doanh nghiệp siêu nhỏ TT58 chọn 1 trong 4 nhóm ở popup khởi tạo, Thông tin đơn vị. PhuongXT bỏ chia nhóm, trả code về như cũ; chỉ giữ ô Thông tư áp dụng ở Thông tin đơn vị chuyển lên cạnh Loại hình, doanh nghiệp gói Standard khoá ở TT58, ô thuế TNDN mở cho chọn</t>
+          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -22431,7 +22431,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-nhom-dnsn](nhat-ky/2026-10-13-phuongxt-nhom-dnsn.md)</t>
+          <t>[2026-10-13-phuongxt-xuat-excel](nhat-ky/2026-10-13-phuongxt-xuat-excel.md)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -22442,12 +22442,12 @@
       </c>
       <c r="B30" s="25" t="inlineStr">
         <is>
-          <t>T171</t>
+          <t>T174</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Bỏ mọi báo cáo ở mọi gói, chỉ giữ Sổ quỹ tiền mặt, Sổ ngân hàng và bộ sổ, báo cáo tài chính TT58; gói Standard (TT58) hiện bộ sổ theo trường hợp thuế của đơn vị</t>
+          <t>Doanh nghiệp siêu nhỏ TT58 chọn 1 trong 4 nhóm ở popup khởi tạo, Thông tin đơn vị. PhuongXT bỏ chia nhóm, trả code về như cũ; chỉ giữ ô Thông tư áp dụng ở Thông tin đơn vị chuyển lên cạnh Loại hình, doanh nghiệp gói Standard khoá ở TT58, ô thuế TNDN mở cho chọn</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-bo-bao-cao](nhat-ky/2026-10-13-phuongxt-bo-bao-cao.md)</t>
+          <t>[2026-10-13-phuongxt-nhom-dnsn](nhat-ky/2026-10-13-phuongxt-nhom-dnsn.md)</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -22478,17 +22478,17 @@
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>T170</t>
+          <t>T171</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Lập kế hoạch giao diện điện thoại theo app IVT Pro: đọc APK, bộ nhận diện, khung màn, 9 đợt làm, danh sách ảnh cần chụp</t>
+          <t>Bỏ mọi báo cáo ở mọi gói, chỉ giữ Sổ quỹ tiền mặt, Sổ ngân hàng và bộ sổ, báo cáo tài chính TT58; gói Standard (TT58) hiện bộ sổ theo trường hợp thuế của đơn vị</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E31" s="28" t="inlineStr">
@@ -22498,12 +22498,12 @@
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-12-trum-ke-hoach-mobile-ivt](nhat-ky/2026-10-12-trum-ke-hoach-mobile-ivt.md)</t>
+          <t>[2026-10-13-phuongxt-bo-bao-cao](nhat-ky/2026-10-13-phuongxt-bo-bao-cao.md)</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -22514,17 +22514,17 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>T168</t>
+          <t>T170</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: phiếu chi mẫu Chi phí chờ phân bổ (Tiền nhà 6 tháng, 72 triệu) có dòng tham chiếu Thẻ chi phí mở thẻ; phiếu thu, chi bỏ Mã số thuế, Ghi chú lên cột giữa, đầu phiếu 3 hàng; cột danh sách Lý do</t>
+          <t>Lập kế hoạch giao diện điện thoại theo app IVT Pro: đọc APK, bộ nhận diện, khung màn, 9 đợt làm, danh sách ảnh cần chụp</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E32" s="28" t="inlineStr">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb](nhat-ky/2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb.md)</t>
+          <t>[2026-10-12-trum-ke-hoach-mobile-ivt](nhat-ky/2026-10-12-trum-ke-hoach-mobile-ivt.md)</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22550,12 +22550,12 @@
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>T165</t>
+          <t>T168</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Form thẻ chi phí: bỏ thanh tiêu đề Thông tin chung; thẻ ghi tăng không xoá, thêm dòng, sửa thì Ngày ghi tăng, Số tiền chỉ đọc; thẻ dư đầu kỳ giữ nút; Free, Standard ngừng theo tháng (bảng 12 tháng); danh sách bỏ cột Số kỳ, Trạng thái</t>
+          <t>Thu chi: phiếu chi mẫu Chi phí chờ phân bổ (Tiền nhà 6 tháng, 72 triệu) có dòng tham chiếu Thẻ chi phí mở thẻ; phiếu thu, chi bỏ Mã số thuế, Ghi chú lên cột giữa, đầu phiếu 3 hàng; cột danh sách Lý do</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -22586,17 +22586,17 @@
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>T167</t>
+          <t>T165</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Kho: tab Kiểm kê chia 3 tab con Kiểm kê, Xuất điều chỉnh, Nhập điều chỉnh; bỏ tab Điều chỉnh kho trên thanh tab</t>
+          <t>Form thẻ chi phí: bỏ thanh tiêu đề Thông tin chung; thẻ ghi tăng không xoá, thêm dòng, sửa thì Ngày ghi tăng, Số tiền chỉ đọc; thẻ dư đầu kỳ giữ nút; Free, Standard ngừng theo tháng (bảng 12 tháng); danh sách bỏ cột Số kỳ, Trạng thái</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E34" s="28" t="inlineStr">
@@ -22611,7 +22611,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-tab-kiem-ke.md`</t>
+          <t>[2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb](nhat-ky/2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb.md)</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr"/>
@@ -22622,12 +22622,12 @@
       </c>
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>T166</t>
+          <t>T167</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Bỏ danh mục Thương hiệu cho mọi đơn vị; ô, cột Thương hiệu ở Hàng hoá, Kho, Bảng giá giữ nguyên</t>
+          <t>Kho: tab Kiểm kê chia 3 tab con Kiểm kê, Xuất điều chỉnh, Nhập điều chỉnh; bỏ tab Điều chỉnh kho trên thanh tab</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -22647,7 +22647,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-bo-thuong-hieu.md`</t>
+          <t>`2026-10-12-phuongxt-tab-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22658,12 +22658,12 @@
       </c>
       <c r="B36" s="25" t="inlineStr">
         <is>
-          <t>T164</t>
+          <t>T166</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng của hộ kinh doanh: Giá trị nhập kho = tiền trước thuế + tiền thuế GTGT</t>
+          <t>Bỏ danh mục Thương hiệu cho mọi đơn vị; ô, cột Thương hiệu ở Hàng hoá, Kho, Bảng giá giữ nguyên</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-nhap-kho-hkd.md`</t>
+          <t>`2026-10-12-phuongxt-bo-thuong-hieu.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22694,12 +22694,12 @@
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>T163</t>
+          <t>T164</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: đơn vị hộ kinh doanh bỏ cột Thuế suất, Tiền thuế, hiện cột Giảm thuế GTGT; doanh nghiệp luôn hiện Thuế suất, Tiền thuế</t>
+          <t>Mua hàng của hộ kinh doanh: Giá trị nhập kho = tiền trước thuế + tiền thuế GTGT</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22719,7 +22719,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-thue-xuat-ban-pos.md`</t>
+          <t>`2026-10-12-phuongxt-nhap-kho-hkd.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22730,12 +22730,12 @@
       </c>
       <c r="B38" s="25" t="inlineStr">
         <is>
-          <t>T162</t>
+          <t>T163</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng gói Plus, Pro tích nhận kèm hoá đơn thì dòng chi tiết có cột Nhóm HHDV mua vào; xem chi tiết phiếu mua, bán bỏ ô tích kèm hoá đơn; danh sách mua bỏ cột Nhận hoá đơn; nút Tổng hợp, Chi tiết ở danh sách bán hàng chỉ xem</t>
+          <t>Xuất bán POS: đơn vị hộ kinh doanh bỏ cột Thuế suất, Tiền thuế, hiện cột Giảm thuế GTGT; doanh nghiệp luôn hiện Thuế suất, Tiền thuế</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22755,7 +22755,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-nhom-hhdv-mua-vao.md`</t>
+          <t>`2026-10-12-phuongxt-thue-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22766,12 +22766,12 @@
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>T161</t>
+          <t>T162</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Mọi form chứng từ khi thêm mới, sửa có nút Tuỳ chỉnh giao diện như lúc xem chi tiết</t>
+          <t>Mua hàng gói Plus, Pro tích nhận kèm hoá đơn thì dòng chi tiết có cột Nhóm HHDV mua vào; xem chi tiết phiếu mua, bán bỏ ô tích kèm hoá đơn; danh sách mua bỏ cột Nhận hoá đơn; nút Tổng hợp, Chi tiết ở danh sách bán hàng chỉ xem</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22791,7 +22791,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-tuy-chinh-khi-sua.md`</t>
+          <t>`2026-10-12-phuongxt-nhom-hhdv-mua-vao.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22802,12 +22802,12 @@
       </c>
       <c r="B40" s="25" t="inlineStr">
         <is>
-          <t>T160</t>
+          <t>T161</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Số dư ban đầu tab tiền: bỏ Thêm mới, hiện đủ mọi quỹ của đơn vị, gõ số dư rồi Lưu (lưu theo đơn vị)</t>
+          <t>Mọi form chứng từ khi thêm mới, sửa có nút Tuỳ chỉnh giao diện như lúc xem chi tiết</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22827,7 +22827,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-12-phuongxt-tuy-chinh-khi-sua.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22838,17 +22838,17 @@
       </c>
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>T159</t>
+          <t>T160</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí: mọi gói chỉ còn Ghi tăng (đổi tên từ Ghi tăng hàng loạt) và Ghi tăng dư đầu kỳ; ngày bắt đầu, ngừng phân bổ theo từng dòng (Standard, Plus chọn tháng); Thông tin mua của thẻ ghi tăng có link chứng từ gốc</t>
+          <t>Số dư ban đầu tab tiền: bỏ Thêm mới, hiện đủ mọi quỹ của đơn vị, gõ số dư rồi Lưu (lưu theo đơn vị)</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E41" s="28" t="inlineStr">
@@ -22863,7 +22863,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong](nhat-ky/2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22874,17 +22874,17 @@
       </c>
       <c r="B42" s="25" t="inlineStr">
         <is>
-          <t>T158</t>
+          <t>T159</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Khởi tạo từ FABi: bỏ bước Đồng bộ bán hàng, popup 3 bước bắt buộc; dùng thử 30 ngày cho mọi gói, hiện ở màn chào, giới thiệu, popup và thanh trên (còn N ngày)</t>
+          <t>Thẻ chi phí: mọi gói chỉ còn Ghi tăng (đổi tên từ Ghi tăng hàng loạt) và Ghi tăng dư đầu kỳ; ngày bắt đầu, ngừng phân bổ theo từng dòng (Standard, Plus chọn tháng); Thông tin mua của thẻ ghi tăng có link chứng từ gốc</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E42" s="28" t="inlineStr">
@@ -22899,7 +22899,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-dung-thu-30-ngay.md`</t>
+          <t>[2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong](nhat-ky/2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong.md)</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22910,17 +22910,17 @@
       </c>
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>T155</t>
+          <t>T158</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
+          <t>Khởi tạo từ FABi: bỏ bước Đồng bộ bán hàng, popup 3 bước bắt buộc; dùng thử 30 ngày cho mọi gói, hiện ở màn chào, giới thiệu, popup và thanh trên (còn N ngày)</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E43" s="28" t="inlineStr">
@@ -22935,7 +22935,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-12-trum-dieu-chuyen-chuyen-kho](nhat-ky/2026-10-12-trum-dieu-chuyen-chuyen-kho.md)</t>
+          <t>`2026-10-12-phuongxt-dung-thu-30-ngay.md`</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22946,12 +22946,12 @@
       </c>
       <c r="B44" s="25" t="inlineStr">
         <is>
-          <t>T157</t>
+          <t>T155</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: bán hàng theo ngày, tổng hợp, chi tiết bán hàng; kho: xuất nhập tồn (mã hàng mở thẻ kho), tổng hợp, chi tiết nhập, xuất, hàng trả</t>
+          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -22966,12 +22966,12 @@
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-bao-cao-ban-hang-kho](nhat-ky/2026-10-11-trum-bao-cao-ban-hang-kho.md)</t>
+          <t>[2026-10-12-trum-dieu-chuyen-chuyen-kho](nhat-ky/2026-10-12-trum-dieu-chuyen-chuyen-kho.md)</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22982,12 +22982,12 @@
       </c>
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>T154</t>
+          <t>T157</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Danh mục sửa theo iFaster: form tài khoản (cấp, loại tài khoản chọn, ô Tổng hợp), hộp quy đổi ĐVT trong hàng hoá, ô chọn nhiều kiểu iFaster toàn hệ thống, thuế ngành nghề chỉ đọc, form Quy đổi ĐVT (hàng áp dụng chọn nhiều, diễn giải tự sinh), lịch chọn ngày hết khoảng trống, nhóm hàng bỏ loại hàng và tồn kho, công việc chỉ mã tên mô tả trạng thái, form bảng giá như iFaster</t>
+          <t>Báo cáo: bán hàng theo ngày, tổng hợp, chi tiết bán hàng; kho: xuất nhập tồn (mã hàng mở thẻ kho), tổng hợp, chi tiết nhập, xuất, hàng trả</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-ifaster-cong-thuc](nhat-ky/2026-10-11-trum-danh-muc-ifaster-cong-thuc.md)</t>
+          <t>[2026-10-11-trum-bao-cao-ban-hang-kho](nhat-ky/2026-10-11-trum-bao-cao-ban-hang-kho.md)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -23018,12 +23018,12 @@
       </c>
       <c r="B46" s="25" t="inlineStr">
         <is>
-          <t>T156</t>
+          <t>T154</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Công thức sơ chế, chế biến: form chi tiết bố cục như iPOS Inventory, bỏ mức tăng, giảm tối đa</t>
+          <t>Danh mục sửa theo iFaster: form tài khoản (cấp, loại tài khoản chọn, ô Tổng hợp), hộp quy đổi ĐVT trong hàng hoá, ô chọn nhiều kiểu iFaster toàn hệ thống, thuế ngành nghề chỉ đọc, form Quy đổi ĐVT (hàng áp dụng chọn nhiều, diễn giải tự sinh), lịch chọn ngày hết khoảng trống, nhóm hàng bỏ loại hàng và tồn kho, công việc chỉ mã tên mô tả trạng thái, form bảng giá như iFaster</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -23054,17 +23054,17 @@
       </c>
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>T150</t>
+          <t>T156</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thẻ chi phí: số thẻ link xanh mở thẻ; thẻ mở ở chế độ xem, bấm Sửa (Ctrl+E) mới sửa, Huỷ về xem như phiếu chi. Thông tin đơn vị: phương pháp thuế GTGT, TNCN, TNDN lên khối Thông tin kê khai, khoá theo loại hình, nhóm doanh thu, gói</t>
+          <t>Công thức sơ chế, chế biến: form chi tiết bố cục như iPOS Inventory, bỏ mức tăng, giảm tối đa</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E47" s="28" t="inlineStr">
@@ -23079,7 +23079,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-xem-the-thue.md`</t>
+          <t>[2026-10-11-trum-danh-muc-ifaster-cong-thuc](nhat-ky/2026-10-11-trum-danh-muc-ifaster-cong-thuc.md)</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
@@ -23090,17 +23090,17 @@
       </c>
       <c r="B48" s="25" t="inlineStr">
         <is>
-          <t>T152</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
+          <t>Danh sách thẻ chi phí: số thẻ link xanh mở thẻ; thẻ mở ở chế độ xem, bấm Sửa (Ctrl+E) mới sửa, Huỷ về xem như phiếu chi. Thông tin đơn vị: phương pháp thuế GTGT, TNCN, TNDN lên khối Thông tin kê khai, khoá theo loại hình, nhóm doanh thu, gói</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E48" s="28" t="inlineStr">
@@ -23115,7 +23115,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
+          <t>`2026-10-11-dinhlanphuongipacc-xem-the-thue.md`</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -23126,12 +23126,12 @@
       </c>
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>T151</t>
+          <t>T152</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
+          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
+          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -23162,12 +23162,12 @@
       </c>
       <c r="B50" s="25" t="inlineStr">
         <is>
-          <t>T153</t>
+          <t>T151</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
+          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -23187,7 +23187,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
+          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -23198,12 +23198,12 @@
       </c>
       <c r="B51" s="26" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T153</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -23234,12 +23234,12 @@
       </c>
       <c r="B52" s="25" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -23270,12 +23270,12 @@
       </c>
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -23306,12 +23306,12 @@
       </c>
       <c r="B54" s="25" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -23342,17 +23342,17 @@
       </c>
       <c r="B55" s="26" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E55" s="28" t="inlineStr">
@@ -23367,7 +23367,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -23378,12 +23378,12 @@
       </c>
       <c r="B56" s="25" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -23403,7 +23403,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -23414,12 +23414,12 @@
       </c>
       <c r="B57" s="26" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -23439,7 +23439,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -23450,12 +23450,12 @@
       </c>
       <c r="B58" s="25" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -23475,7 +23475,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -23486,12 +23486,12 @@
       </c>
       <c r="B59" s="26" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -23511,7 +23511,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -23522,17 +23522,17 @@
       </c>
       <c r="B60" s="25" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E60" s="28" t="inlineStr">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23558,12 +23558,12 @@
       </c>
       <c r="B61" s="26" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -23594,17 +23594,17 @@
       </c>
       <c r="B62" s="25" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E62" s="28" t="inlineStr">
@@ -23619,7 +23619,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr"/>
@@ -23630,17 +23630,17 @@
       </c>
       <c r="B63" s="26" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E63" s="28" t="inlineStr">
@@ -23655,7 +23655,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23666,12 +23666,12 @@
       </c>
       <c r="B64" s="25" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -23686,12 +23686,12 @@
       </c>
       <c r="F64" s="12" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23702,17 +23702,17 @@
       </c>
       <c r="B65" s="26" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E65" s="28" t="inlineStr">
@@ -23727,7 +23727,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23738,12 +23738,12 @@
       </c>
       <c r="B66" s="25" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -23763,7 +23763,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23774,12 +23774,12 @@
       </c>
       <c r="B67" s="26" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23799,7 +23799,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23810,12 +23810,12 @@
       </c>
       <c r="B68" s="25" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23846,12 +23846,12 @@
       </c>
       <c r="B69" s="26" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23871,7 +23871,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23882,12 +23882,12 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23918,12 +23918,12 @@
       </c>
       <c r="B71" s="26" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23954,12 +23954,12 @@
       </c>
       <c r="B72" s="25" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23990,12 +23990,12 @@
       </c>
       <c r="B73" s="26" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -24026,12 +24026,12 @@
       </c>
       <c r="B74" s="25" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -24051,7 +24051,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -24062,17 +24062,17 @@
       </c>
       <c r="B75" s="26" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E75" s="28" t="inlineStr">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -24098,17 +24098,17 @@
       </c>
       <c r="B76" s="25" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E76" s="28" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -24134,17 +24134,17 @@
       </c>
       <c r="B77" s="26" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E77" s="28" t="inlineStr">
@@ -24159,7 +24159,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -24170,12 +24170,12 @@
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -24206,17 +24206,17 @@
       </c>
       <c r="B79" s="26" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E79" s="28" t="inlineStr">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr"/>
@@ -24242,12 +24242,12 @@
       </c>
       <c r="B80" s="25" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -24267,7 +24267,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -24278,12 +24278,12 @@
       </c>
       <c r="B81" s="26" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -24314,12 +24314,12 @@
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -24350,12 +24350,12 @@
       </c>
       <c r="B83" s="26" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -24386,12 +24386,12 @@
       </c>
       <c r="B84" s="25" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -24422,17 +24422,17 @@
       </c>
       <c r="B85" s="26" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E85" s="28" t="inlineStr">
@@ -24447,7 +24447,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr"/>
@@ -24458,12 +24458,12 @@
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -24483,7 +24483,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -24494,17 +24494,17 @@
       </c>
       <c r="B87" s="26" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E87" s="28" t="inlineStr">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24530,17 +24530,17 @@
       </c>
       <c r="B88" s="25" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E88" s="28" t="inlineStr">
@@ -24555,7 +24555,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24566,12 +24566,12 @@
       </c>
       <c r="B89" s="26" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -24602,12 +24602,12 @@
       </c>
       <c r="B90" s="25" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24638,12 +24638,12 @@
       </c>
       <c r="B91" s="26" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24674,12 +24674,12 @@
       </c>
       <c r="B92" s="25" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24710,12 +24710,12 @@
       </c>
       <c r="B93" s="26" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24735,7 +24735,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr"/>
@@ -24746,12 +24746,12 @@
       </c>
       <c r="B94" s="25" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24782,12 +24782,12 @@
       </c>
       <c r="B95" s="26" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -24818,17 +24818,17 @@
       </c>
       <c r="B96" s="25" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E96" s="28" t="inlineStr">
@@ -24843,7 +24843,7 @@
       </c>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr"/>
@@ -24854,17 +24854,17 @@
       </c>
       <c r="B97" s="26" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E97" s="28" t="inlineStr">
@@ -24879,7 +24879,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24890,12 +24890,12 @@
       </c>
       <c r="B98" s="25" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
@@ -24926,12 +24926,12 @@
       </c>
       <c r="B99" s="26" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24962,12 +24962,12 @@
       </c>
       <c r="B100" s="25" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24987,7 +24987,7 @@
       </c>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr"/>
@@ -24998,12 +24998,12 @@
       </c>
       <c r="B101" s="26" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -25034,12 +25034,12 @@
       </c>
       <c r="B102" s="25" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -25070,12 +25070,12 @@
       </c>
       <c r="B103" s="26" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -25095,7 +25095,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
@@ -25106,12 +25106,12 @@
       </c>
       <c r="B104" s="25" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -25142,17 +25142,17 @@
       </c>
       <c r="B105" s="26" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E105" s="28" t="inlineStr">
@@ -25167,7 +25167,7 @@
       </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
@@ -25178,12 +25178,12 @@
       </c>
       <c r="B106" s="25" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -25214,12 +25214,12 @@
       </c>
       <c r="B107" s="26" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -25250,12 +25250,12 @@
       </c>
       <c r="B108" s="25" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -25286,17 +25286,17 @@
       </c>
       <c r="B109" s="26" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E109" s="28" t="inlineStr">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
@@ -25322,12 +25322,12 @@
       </c>
       <c r="B110" s="25" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
@@ -25358,12 +25358,12 @@
       </c>
       <c r="B111" s="26" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -25383,7 +25383,7 @@
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
@@ -25394,12 +25394,12 @@
       </c>
       <c r="B112" s="25" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -25419,7 +25419,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -25430,12 +25430,12 @@
       </c>
       <c r="B113" s="26" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -25466,12 +25466,12 @@
       </c>
       <c r="B114" s="25" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -25502,17 +25502,17 @@
       </c>
       <c r="B115" s="26" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E115" s="28" t="inlineStr">
@@ -25527,7 +25527,7 @@
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
@@ -25538,12 +25538,12 @@
       </c>
       <c r="B116" s="25" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
@@ -25574,12 +25574,12 @@
       </c>
       <c r="B117" s="26" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25610,12 +25610,12 @@
       </c>
       <c r="B118" s="25" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25646,17 +25646,17 @@
       </c>
       <c r="B119" s="26" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E119" s="28" t="inlineStr">
@@ -25666,12 +25666,12 @@
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H119" s="5" t="inlineStr"/>
@@ -25682,12 +25682,12 @@
       </c>
       <c r="B120" s="25" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
@@ -25707,7 +25707,7 @@
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25718,12 +25718,12 @@
       </c>
       <c r="B121" s="26" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25743,7 +25743,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25754,12 +25754,12 @@
       </c>
       <c r="B122" s="25" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25790,17 +25790,17 @@
       </c>
       <c r="B123" s="26" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E123" s="28" t="inlineStr">
@@ -25815,7 +25815,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
@@ -25826,12 +25826,12 @@
       </c>
       <c r="B124" s="25" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
@@ -25862,12 +25862,12 @@
       </c>
       <c r="B125" s="26" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25898,12 +25898,12 @@
       </c>
       <c r="B126" s="25" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25934,12 +25934,12 @@
       </c>
       <c r="B127" s="26" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25970,12 +25970,12 @@
       </c>
       <c r="B128" s="25" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -26006,12 +26006,12 @@
       </c>
       <c r="B129" s="26" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -26042,12 +26042,12 @@
       </c>
       <c r="B130" s="25" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -26078,17 +26078,17 @@
       </c>
       <c r="B131" s="26" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E131" s="28" t="inlineStr">
@@ -26103,7 +26103,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr"/>
@@ -26114,12 +26114,12 @@
       </c>
       <c r="B132" s="25" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
@@ -26150,12 +26150,12 @@
       </c>
       <c r="B133" s="26" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -26186,12 +26186,12 @@
       </c>
       <c r="B134" s="25" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -26222,12 +26222,12 @@
       </c>
       <c r="B135" s="26" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -26258,17 +26258,17 @@
       </c>
       <c r="B136" s="25" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E136" s="28" t="inlineStr">
@@ -26283,7 +26283,7 @@
       </c>
       <c r="G136" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr"/>
@@ -26294,12 +26294,12 @@
       </c>
       <c r="B137" s="26" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -26319,7 +26319,7 @@
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -26330,17 +26330,17 @@
       </c>
       <c r="B138" s="25" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E138" s="28" t="inlineStr">
@@ -26355,7 +26355,7 @@
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -26366,12 +26366,12 @@
       </c>
       <c r="B139" s="26" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -26402,12 +26402,12 @@
       </c>
       <c r="B140" s="25" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -26438,12 +26438,12 @@
       </c>
       <c r="B141" s="26" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -26474,12 +26474,12 @@
       </c>
       <c r="B142" s="25" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -26499,7 +26499,7 @@
       </c>
       <c r="G142" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr"/>
@@ -26510,12 +26510,12 @@
       </c>
       <c r="B143" s="26" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26535,7 +26535,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26546,17 +26546,17 @@
       </c>
       <c r="B144" s="25" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E144" s="28" t="inlineStr">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26582,12 +26582,12 @@
       </c>
       <c r="B145" s="26" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
@@ -26607,7 +26607,7 @@
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26618,17 +26618,17 @@
       </c>
       <c r="B146" s="25" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E146" s="28" t="inlineStr">
@@ -26643,7 +26643,7 @@
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26654,12 +26654,12 @@
       </c>
       <c r="B147" s="26" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26690,17 +26690,17 @@
       </c>
       <c r="B148" s="25" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E148" s="28" t="inlineStr">
@@ -26715,7 +26715,7 @@
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26726,12 +26726,12 @@
       </c>
       <c r="B149" s="26" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
@@ -26751,7 +26751,7 @@
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26762,12 +26762,12 @@
       </c>
       <c r="B150" s="25" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26787,7 +26787,7 @@
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr"/>
@@ -26798,12 +26798,12 @@
       </c>
       <c r="B151" s="26" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
@@ -26834,12 +26834,12 @@
       </c>
       <c r="B152" s="25" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D152" s="12" t="inlineStr">
@@ -26854,12 +26854,12 @@
       </c>
       <c r="F152" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G152" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr"/>
@@ -26870,12 +26870,12 @@
       </c>
       <c r="B153" s="26" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D153" s="16" t="inlineStr">
@@ -26895,7 +26895,7 @@
       </c>
       <c r="G153" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H153" s="5" t="inlineStr"/>
@@ -26906,12 +26906,12 @@
       </c>
       <c r="B154" s="25" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C154" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D154" s="12" t="inlineStr">
@@ -26931,7 +26931,7 @@
       </c>
       <c r="G154" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr"/>
@@ -26942,17 +26942,17 @@
       </c>
       <c r="B155" s="26" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D155" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E155" s="28" t="inlineStr">
@@ -26967,7 +26967,7 @@
       </c>
       <c r="G155" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H155" s="5" t="inlineStr"/>
@@ -26978,17 +26978,17 @@
       </c>
       <c r="B156" s="25" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C156" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D156" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E156" s="28" t="inlineStr">
@@ -27003,7 +27003,7 @@
       </c>
       <c r="G156" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H156" s="13" t="inlineStr"/>
@@ -27014,12 +27014,12 @@
       </c>
       <c r="B157" s="26" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D157" s="16" t="inlineStr">
@@ -27039,7 +27039,7 @@
       </c>
       <c r="G157" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H157" s="5" t="inlineStr"/>
@@ -27050,17 +27050,17 @@
       </c>
       <c r="B158" s="25" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C158" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D158" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E158" s="28" t="inlineStr">
@@ -27075,7 +27075,7 @@
       </c>
       <c r="G158" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H158" s="13" t="inlineStr"/>
@@ -27086,12 +27086,12 @@
       </c>
       <c r="B159" s="26" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
       <c r="D159" s="16" t="inlineStr">
@@ -27111,7 +27111,7 @@
       </c>
       <c r="G159" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
+          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
         </is>
       </c>
       <c r="H159" s="5" t="inlineStr"/>
@@ -27122,17 +27122,17 @@
       </c>
       <c r="B160" s="25" t="inlineStr">
         <is>
-          <t>T31</t>
+          <t>T32</t>
         </is>
       </c>
       <c r="C160" s="13" t="inlineStr">
         <is>
-          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
+          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
         </is>
       </c>
       <c r="D160" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E160" s="28" t="inlineStr">
@@ -27147,7 +27147,7 @@
       </c>
       <c r="G160" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
+          <t>`2026-10-08-phuongxt-thu-chi-free.md`</t>
         </is>
       </c>
       <c r="H160" s="13" t="inlineStr"/>
@@ -27158,12 +27158,12 @@
       </c>
       <c r="B161" s="26" t="inlineStr">
         <is>
-          <t>T30</t>
+          <t>T31</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
+          <t>Luật mới: agent kiểm bản mới trên GitHub trước mỗi lần push (QD16)</t>
         </is>
       </c>
       <c r="D161" s="16" t="inlineStr">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="G161" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bao-telegram.md`</t>
+          <t>`2026-10-08-trum-kiem-truoc-push.md`</t>
         </is>
       </c>
       <c r="H161" s="5" t="inlineStr"/>
@@ -27194,12 +27194,12 @@
       </c>
       <c r="B162" s="25" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T30</t>
         </is>
       </c>
       <c r="C162" s="13" t="inlineStr">
         <is>
-          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
+          <t>Robot báo lên group Telegram mỗi lần có người push lên `main`, báo thêm khi deploy hỏng</t>
         </is>
       </c>
       <c r="D162" s="12" t="inlineStr">
@@ -27230,12 +27230,12 @@
       </c>
       <c r="B163" s="26" t="inlineStr">
         <is>
-          <t>T35</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
+          <t>Tạo API token Cloudflare cho robot deploy, lưu vào GitHub</t>
         </is>
       </c>
       <c r="D163" s="16" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="G163" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
+          <t>`2026-10-08-trum-bao-telegram.md`</t>
         </is>
       </c>
       <c r="H163" s="5" t="inlineStr"/>
@@ -27266,12 +27266,12 @@
       </c>
       <c r="B164" s="25" t="inlineStr">
         <is>
-          <t>T34</t>
+          <t>T35</t>
         </is>
       </c>
       <c r="C164" s="13" t="inlineStr">
         <is>
-          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
+          <t>Luật phối hợp: push ngay khi nhận việc, lấy mã sau fetch, giữ chỗ QD, mỗi phiên một bản clone, ghi file dùng chung, CSS theo mục có mã việc (QD21)</t>
         </is>
       </c>
       <c r="D164" s="12" t="inlineStr">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="G164" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
+          <t>`2026-10-08-trum-luat-phoi-hop.md`</t>
         </is>
       </c>
       <c r="H164" s="13" t="inlineStr"/>
@@ -27302,12 +27302,12 @@
       </c>
       <c r="B165" s="26" t="inlineStr">
         <is>
-          <t>T29</t>
+          <t>T34</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
+          <t>Thanh lọc và chọn khoảng ngày theo iFaster cho mọi màn danh mục, danh sách, báo cáo</t>
         </is>
       </c>
       <c r="D165" s="16" t="inlineStr">
@@ -27327,7 +27327,7 @@
       </c>
       <c r="G165" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
+          <t>`2026-10-08-trum-thanh-loc-ifaster.md`</t>
         </is>
       </c>
       <c r="H165" s="5" t="inlineStr"/>
@@ -27338,12 +27338,12 @@
       </c>
       <c r="B166" s="25" t="inlineStr">
         <is>
-          <t>T28</t>
+          <t>T29</t>
         </is>
       </c>
       <c r="C166" s="13" t="inlineStr">
         <is>
-          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
+          <t>Màn chứng từ bán hàng 3.1.1 chia đôi 50/50 như 3.1.2</t>
         </is>
       </c>
       <c r="D166" s="12" t="inlineStr">
@@ -27363,7 +27363,7 @@
       </c>
       <c r="G166" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
+          <t>`2026-10-08-trum-ban-hang-chia-doi.md`</t>
         </is>
       </c>
       <c r="H166" s="13" t="inlineStr"/>
@@ -27374,12 +27374,12 @@
       </c>
       <c r="B167" s="26" t="inlineStr">
         <is>
-          <t>T26</t>
+          <t>T28</t>
         </is>
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
+          <t>Ô chọn trong form chứng từ dùng chung một kiểu, thẳng hàng. Màn đăng nhập bỏ sơ đồ kết nối</t>
         </is>
       </c>
       <c r="D167" s="16" t="inlineStr">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="G167" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
+          <t>`2026-10-08-trum-o-chon-ngay-ngan.md`</t>
         </is>
       </c>
       <c r="H167" s="5" t="inlineStr"/>
@@ -27410,12 +27410,12 @@
       </c>
       <c r="B168" s="25" t="inlineStr">
         <is>
-          <t>T24</t>
+          <t>T26</t>
         </is>
       </c>
       <c r="C168" s="13" t="inlineStr">
         <is>
-          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
+          <t>Đổi ngôn ngữ thiết kế theo iFaster (QD15), thay logo sang Accounting Powered by iPOS.vn</t>
         </is>
       </c>
       <c r="D168" s="12" t="inlineStr">
@@ -27435,7 +27435,7 @@
       </c>
       <c r="G168" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
+          <t>`2026-10-08-trum-thiet-ke-ifaster.md`</t>
         </is>
       </c>
       <c r="H168" s="13" t="inlineStr"/>
@@ -27446,12 +27446,12 @@
       </c>
       <c r="B169" s="26" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T24</t>
         </is>
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
+          <t>Bố cục danh sách chứng từ 50/50 cố định 1 trang, sửa padding form và điều hướng Trước Sau Esc</t>
         </is>
       </c>
       <c r="D169" s="16" t="inlineStr">
@@ -27471,7 +27471,7 @@
       </c>
       <c r="G169" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
+          <t>`2026-10-08-trum-bo-cuc-voucher-50-50.md`</t>
         </is>
       </c>
       <c r="H169" s="5" t="inlineStr"/>
@@ -27482,12 +27482,12 @@
       </c>
       <c r="B170" s="25" t="inlineStr">
         <is>
-          <t>T00</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C170" s="13" t="inlineStr">
         <is>
-          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
+          <t>Sửa hiệu ứng chớp khi bấm Trước, Sau ở form chứng từ</t>
         </is>
       </c>
       <c r="D170" s="12" t="inlineStr">
@@ -27502,12 +27502,12 @@
       </c>
       <c r="F170" s="12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="G170" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-khung-web.md`</t>
+          <t>`2026-10-08-trum-sua-hieu-ung-truoc-sau.md`</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr"/>
@@ -27518,12 +27518,12 @@
       </c>
       <c r="B171" s="26" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T00</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
+          <t>Bộ tài liệu làm việc nhóm, robot kiểm và deploy</t>
         </is>
       </c>
       <c r="D171" s="16" t="inlineStr">
@@ -27543,7 +27543,7 @@
       </c>
       <c r="G171" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
+          <t>`2026-10-07-trum-khung-web.md`</t>
         </is>
       </c>
       <c r="H171" s="5" t="inlineStr"/>
@@ -27554,12 +27554,12 @@
       </c>
       <c r="B172" s="25" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C172" s="13" t="inlineStr">
         <is>
-          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
+          <t>Làm lại form chứng từ và màn danh sách chứng từ theo bố cục AMIS (QD14)</t>
         </is>
       </c>
       <c r="D172" s="12" t="inlineStr">
@@ -27579,7 +27579,7 @@
       </c>
       <c r="G172" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
+          <t>`2026-10-07-trum-form-chung-tu-amis.md`</t>
         </is>
       </c>
       <c r="H172" s="13" t="inlineStr"/>
@@ -27590,12 +27590,12 @@
       </c>
       <c r="B173" s="26" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
+          <t>Chuẩn hoá BAT-DAU.md cho người mới, đồng bộ skill Clau - Anti (QD13)</t>
         </is>
       </c>
       <c r="D173" s="16" t="inlineStr">
@@ -27615,7 +27615,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
+          <t>`2026-10-07-trum-chuan-hoa-bat-dau-skills.md`</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr"/>
@@ -27626,12 +27626,12 @@
       </c>
       <c r="B174" s="25" t="inlineStr">
         <is>
-          <t>T21</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="C174" s="13" t="inlineStr">
         <is>
-          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
+          <t>Dòng chi tiết chứng từ bám DB iPOS: Đối tượng, Khoản mục, Công việc từng dòng phiếu thu chi; Số lô, Hạn dùng phiếu mua</t>
         </is>
       </c>
       <c r="D174" s="12" t="inlineStr">
@@ -27646,12 +27646,12 @@
       </c>
       <c r="F174" s="12" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="G174" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+          <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr"/>
@@ -27662,12 +27662,12 @@
       </c>
       <c r="B175" s="26" t="inlineStr">
         <is>
-          <t>T22</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
+          <t>Sửa danh sách chứng từ vỡ bố cục: lớp `sel` của hàng đang chọn đụng lớp `.sel` của ô chọn</t>
         </is>
       </c>
       <c r="D175" s="16" t="inlineStr">
@@ -27698,12 +27698,12 @@
       </c>
       <c r="B176" s="25" t="inlineStr">
         <is>
-          <t>T23</t>
+          <t>T22</t>
         </is>
       </c>
       <c r="C176" s="13" t="inlineStr">
         <is>
-          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+          <t>Danh sách chứng từ học AMIS: thẻ tổng hợp, phân trang, chọn cột, ô một dòng</t>
         </is>
       </c>
       <c r="D176" s="12" t="inlineStr">
@@ -27734,38 +27734,74 @@
       </c>
       <c r="B177" s="26" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>Danh mục học AMIS: cột Chức năng lập nhanh chứng từ; số dư ban đầu thành lưới thẻ</t>
+        </is>
+      </c>
+      <c r="D177" s="16" t="inlineStr">
+        <is>
+          <t>Trum</t>
+        </is>
+      </c>
+      <c r="E177" s="28" t="inlineStr">
+        <is>
+          <t>Xong</t>
+        </is>
+      </c>
+      <c r="F177" s="16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
+          <t>`2026-10-08-trum-hoc-amis-lan-2.md`</t>
+        </is>
+      </c>
+      <c r="H177" s="5" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="25" t="inlineStr">
+        <is>
           <t>T18</t>
         </is>
       </c>
-      <c r="C177" s="5" t="inlineStr">
+      <c r="C178" s="13" t="inlineStr">
         <is>
           <t>Danh mục và số dư bám DB iPOS: kho 1.8, đối tượng 1.5, bút toán tự động 1.15, số dư ban đầu 10.1.3</t>
         </is>
       </c>
-      <c r="D177" s="16" t="inlineStr">
+      <c r="D178" s="12" t="inlineStr">
         <is>
           <t>Trum</t>
         </is>
       </c>
-      <c r="E177" s="28" t="inlineStr">
+      <c r="E178" s="28" t="inlineStr">
         <is>
           <t>Xong</t>
         </is>
       </c>
-      <c r="F177" s="16" t="inlineStr">
+      <c r="F178" s="12" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="G177" s="5" t="inlineStr">
+      <c r="G178" s="13" t="inlineStr">
         <is>
           <t>`2026-10-07-trum-giao-dien-bam-db-ipos.md`</t>
         </is>
       </c>
-      <c r="H177" s="5" t="inlineStr"/>
+      <c r="H178" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H177"/>
+  <autoFilter ref="A1:H178"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
T176: giao diện điện thoại đợt 3, danh sách chứng từ, danh mục dạng thẻ, lọc, màn trống
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
+++ b/docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ma trận tính năng'!$A$1:$M$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chi tiết màn hình'!$A$1:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Báo cáo &amp; Mẫu in'!$A$1:$L$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tiến độ công việc'!$A$1:$H$179</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -847,7 +847,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>177 việc (T01 - T108)</t>
+          <t>178 việc (T01 - T108)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>152 việc (85.9%)</t>
+          <t>153 việc (86.0%)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -21565,7 +21565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H178"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22334,12 +22334,12 @@
       </c>
       <c r="B27" s="26" t="inlineStr">
         <is>
-          <t>T175</t>
+          <t>T176</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Điện thoại đợt 2: Trang chủ (thao tác nhanh, thẻ số liệu), Nghiệp vụ (lưới phân hệ, danh sách màn), Khác (tài khoản, danh mục, hệ thống, đơn vị, gói, đăng xuất); số đo IVT, thanh dưới nổi</t>
+          <t>Điện thoại đợt 3: danh sách chứng từ, danh mục dạng thẻ, chip trạng thái, chip loại phiếu, màn lọc, màn trống; số thẻ khớp bản máy tính</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-13-trum-dien-thoai-dot-2](nhat-ky/2026-10-13-trum-dien-thoai-dot-2.md)</t>
+          <t>[2026-10-13-trum-dien-thoai-dot-3](nhat-ky/2026-10-13-trum-dien-thoai-dot-3.md)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
@@ -22370,12 +22370,12 @@
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>T173</t>
+          <t>T175</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên (tên màn, chọn chi nhánh), thanh dưới 4 tab theo IVT Pro, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
+          <t>Điện thoại đợt 2: Trang chủ (thao tác nhanh, thẻ số liệu), Nghiệp vụ (lưới phân hệ, danh sách màn), Khác (tài khoản, danh mục, hệ thống, đơn vị, gói, đăng xuất); số đo IVT, thanh dưới nổi</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -22395,7 +22395,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-13-trum-dien-thoai-dot-1](nhat-ky/2026-10-13-trum-dien-thoai-dot-1.md)</t>
+          <t>[2026-10-13-trum-dien-thoai-dot-2](nhat-ky/2026-10-13-trum-dien-thoai-dot-2.md)</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr"/>
@@ -22406,17 +22406,17 @@
       </c>
       <c r="B29" s="26" t="inlineStr">
         <is>
-          <t>T172</t>
+          <t>T173</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
+          <t>Điện thoại đợt 1: khung `MobileShell`, thanh trên (tên màn, chọn chi nhánh), thanh dưới 4 tab theo IVT Pro, chuyển khung theo bề rộng 767px, màn chưa có bản điện thoại ra `MChiMayTinh`; `kiem_tra.py --dien-thoai`</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E29" s="28" t="inlineStr">
@@ -22431,7 +22431,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-xuat-excel](nhat-ky/2026-10-13-phuongxt-xuat-excel.md)</t>
+          <t>[2026-10-13-trum-dien-thoai-dot-1](nhat-ky/2026-10-13-trum-dien-thoai-dot-1.md)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
@@ -22442,12 +22442,12 @@
       </c>
       <c r="B30" s="25" t="inlineStr">
         <is>
-          <t>T174</t>
+          <t>T172</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Doanh nghiệp siêu nhỏ TT58 chọn 1 trong 4 nhóm ở popup khởi tạo, Thông tin đơn vị. PhuongXT bỏ chia nhóm, trả code về như cũ; chỉ giữ ô Thông tư áp dụng ở Thông tin đơn vị chuyển lên cạnh Loại hình, doanh nghiệp gói Standard khoá ở TT58, ô thuế TNDN mở cho chọn</t>
+          <t>Chạy lại `python tools/xuat_bao_cao_he_thong.py` để làm mới `docs/IACC-Cloud-Chi-Tiet-He-Thong.xlsx` sau T171 (sheet Báo cáo &amp; Mẫu in có cột Còn dùng)</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-nhom-dnsn](nhat-ky/2026-10-13-phuongxt-nhom-dnsn.md)</t>
+          <t>[2026-10-13-phuongxt-xuat-excel](nhat-ky/2026-10-13-phuongxt-xuat-excel.md)</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr"/>
@@ -22478,12 +22478,12 @@
       </c>
       <c r="B31" s="26" t="inlineStr">
         <is>
-          <t>T171</t>
+          <t>T174</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Bỏ mọi báo cáo ở mọi gói, chỉ giữ Sổ quỹ tiền mặt, Sổ ngân hàng và bộ sổ, báo cáo tài chính TT58; gói Standard (TT58) hiện bộ sổ theo trường hợp thuế của đơn vị</t>
+          <t>Doanh nghiệp siêu nhỏ TT58 chọn 1 trong 4 nhóm ở popup khởi tạo, Thông tin đơn vị. PhuongXT bỏ chia nhóm, trả code về như cũ; chỉ giữ ô Thông tư áp dụng ở Thông tin đơn vị chuyển lên cạnh Loại hình, doanh nghiệp gói Standard khoá ở TT58, ô thuế TNDN mở cho chọn</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -22503,7 +22503,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-13-phuongxt-bo-bao-cao](nhat-ky/2026-10-13-phuongxt-bo-bao-cao.md)</t>
+          <t>[2026-10-13-phuongxt-nhom-dnsn](nhat-ky/2026-10-13-phuongxt-nhom-dnsn.md)</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr"/>
@@ -22514,17 +22514,17 @@
       </c>
       <c r="B32" s="25" t="inlineStr">
         <is>
-          <t>T170</t>
+          <t>T171</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Lập kế hoạch giao diện điện thoại theo app IVT Pro: đọc APK, bộ nhận diện, khung màn, 9 đợt làm, danh sách ảnh cần chụp</t>
+          <t>Bỏ mọi báo cáo ở mọi gói, chỉ giữ Sổ quỹ tiền mặt, Sổ ngân hàng và bộ sổ, báo cáo tài chính TT58; gói Standard (TT58) hiện bộ sổ theo trường hợp thuế của đơn vị</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E32" s="28" t="inlineStr">
@@ -22534,12 +22534,12 @@
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-12-trum-ke-hoach-mobile-ivt](nhat-ky/2026-10-12-trum-ke-hoach-mobile-ivt.md)</t>
+          <t>[2026-10-13-phuongxt-bo-bao-cao](nhat-ky/2026-10-13-phuongxt-bo-bao-cao.md)</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr"/>
@@ -22550,17 +22550,17 @@
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>T168</t>
+          <t>T170</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: phiếu chi mẫu Chi phí chờ phân bổ (Tiền nhà 6 tháng, 72 triệu) có dòng tham chiếu Thẻ chi phí mở thẻ; phiếu thu, chi bỏ Mã số thuế, Ghi chú lên cột giữa, đầu phiếu 3 hàng; cột danh sách Lý do</t>
+          <t>Lập kế hoạch giao diện điện thoại theo app IVT Pro: đọc APK, bộ nhận diện, khung màn, 9 đợt làm, danh sách ảnh cần chụp</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E33" s="28" t="inlineStr">
@@ -22575,7 +22575,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb](nhat-ky/2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb.md)</t>
+          <t>[2026-10-12-trum-ke-hoach-mobile-ivt](nhat-ky/2026-10-12-trum-ke-hoach-mobile-ivt.md)</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr"/>
@@ -22586,12 +22586,12 @@
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>T165</t>
+          <t>T168</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Form thẻ chi phí: bỏ thanh tiêu đề Thông tin chung; thẻ ghi tăng không xoá, thêm dòng, sửa thì Ngày ghi tăng, Số tiền chỉ đọc; thẻ dư đầu kỳ giữ nút; Free, Standard ngừng theo tháng (bảng 12 tháng); danh sách bỏ cột Số kỳ, Trạng thái</t>
+          <t>Thu chi: phiếu chi mẫu Chi phí chờ phân bổ (Tiền nhà 6 tháng, 72 triệu) có dòng tham chiếu Thẻ chi phí mở thẻ; phiếu thu, chi bỏ Mã số thuế, Ghi chú lên cột giữa, đầu phiếu 3 hàng; cột danh sách Lý do</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -22622,17 +22622,17 @@
       </c>
       <c r="B35" s="26" t="inlineStr">
         <is>
-          <t>T167</t>
+          <t>T165</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Kho: tab Kiểm kê chia 3 tab con Kiểm kê, Xuất điều chỉnh, Nhập điều chỉnh; bỏ tab Điều chỉnh kho trên thanh tab</t>
+          <t>Form thẻ chi phí: bỏ thanh tiêu đề Thông tin chung; thẻ ghi tăng không xoá, thêm dòng, sửa thì Ngày ghi tăng, Số tiền chỉ đọc; thẻ dư đầu kỳ giữ nút; Free, Standard ngừng theo tháng (bảng 12 tháng); danh sách bỏ cột Số kỳ, Trạng thái</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E35" s="28" t="inlineStr">
@@ -22647,7 +22647,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-tab-kiem-ke.md`</t>
+          <t>[2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb](nhat-ky/2026-10-12-dinhlanphuongipacc-form-the-va-phieu-chi-cho-pb.md)</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
@@ -22658,12 +22658,12 @@
       </c>
       <c r="B36" s="25" t="inlineStr">
         <is>
-          <t>T166</t>
+          <t>T167</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Bỏ danh mục Thương hiệu cho mọi đơn vị; ô, cột Thương hiệu ở Hàng hoá, Kho, Bảng giá giữ nguyên</t>
+          <t>Kho: tab Kiểm kê chia 3 tab con Kiểm kê, Xuất điều chỉnh, Nhập điều chỉnh; bỏ tab Điều chỉnh kho trên thanh tab</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-bo-thuong-hieu.md`</t>
+          <t>`2026-10-12-phuongxt-tab-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr"/>
@@ -22694,12 +22694,12 @@
       </c>
       <c r="B37" s="26" t="inlineStr">
         <is>
-          <t>T164</t>
+          <t>T166</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng của hộ kinh doanh: Giá trị nhập kho = tiền trước thuế + tiền thuế GTGT</t>
+          <t>Bỏ danh mục Thương hiệu cho mọi đơn vị; ô, cột Thương hiệu ở Hàng hoá, Kho, Bảng giá giữ nguyên</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -22719,7 +22719,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-nhap-kho-hkd.md`</t>
+          <t>`2026-10-12-phuongxt-bo-thuong-hieu.md`</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
@@ -22730,12 +22730,12 @@
       </c>
       <c r="B38" s="25" t="inlineStr">
         <is>
-          <t>T163</t>
+          <t>T164</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: đơn vị hộ kinh doanh bỏ cột Thuế suất, Tiền thuế, hiện cột Giảm thuế GTGT; doanh nghiệp luôn hiện Thuế suất, Tiền thuế</t>
+          <t>Mua hàng của hộ kinh doanh: Giá trị nhập kho = tiền trước thuế + tiền thuế GTGT</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -22755,7 +22755,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-thue-xuat-ban-pos.md`</t>
+          <t>`2026-10-12-phuongxt-nhap-kho-hkd.md`</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr"/>
@@ -22766,12 +22766,12 @@
       </c>
       <c r="B39" s="26" t="inlineStr">
         <is>
-          <t>T162</t>
+          <t>T163</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng gói Plus, Pro tích nhận kèm hoá đơn thì dòng chi tiết có cột Nhóm HHDV mua vào; xem chi tiết phiếu mua, bán bỏ ô tích kèm hoá đơn; danh sách mua bỏ cột Nhận hoá đơn; nút Tổng hợp, Chi tiết ở danh sách bán hàng chỉ xem</t>
+          <t>Xuất bán POS: đơn vị hộ kinh doanh bỏ cột Thuế suất, Tiền thuế, hiện cột Giảm thuế GTGT; doanh nghiệp luôn hiện Thuế suất, Tiền thuế</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -22791,7 +22791,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-nhom-hhdv-mua-vao.md`</t>
+          <t>`2026-10-12-phuongxt-thue-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr"/>
@@ -22802,12 +22802,12 @@
       </c>
       <c r="B40" s="25" t="inlineStr">
         <is>
-          <t>T161</t>
+          <t>T162</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Mọi form chứng từ khi thêm mới, sửa có nút Tuỳ chỉnh giao diện như lúc xem chi tiết</t>
+          <t>Mua hàng gói Plus, Pro tích nhận kèm hoá đơn thì dòng chi tiết có cột Nhóm HHDV mua vào; xem chi tiết phiếu mua, bán bỏ ô tích kèm hoá đơn; danh sách mua bỏ cột Nhận hoá đơn; nút Tổng hợp, Chi tiết ở danh sách bán hàng chỉ xem</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -22827,7 +22827,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-tuy-chinh-khi-sua.md`</t>
+          <t>`2026-10-12-phuongxt-nhom-hhdv-mua-vao.md`</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr"/>
@@ -22838,12 +22838,12 @@
       </c>
       <c r="B41" s="26" t="inlineStr">
         <is>
-          <t>T160</t>
+          <t>T161</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Số dư ban đầu tab tiền: bỏ Thêm mới, hiện đủ mọi quỹ của đơn vị, gõ số dư rồi Lưu (lưu theo đơn vị)</t>
+          <t>Mọi form chứng từ khi thêm mới, sửa có nút Tuỳ chỉnh giao diện như lúc xem chi tiết</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -22863,7 +22863,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-12-phuongxt-tuy-chinh-khi-sua.md`</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
@@ -22874,17 +22874,17 @@
       </c>
       <c r="B42" s="25" t="inlineStr">
         <is>
-          <t>T159</t>
+          <t>T160</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí: mọi gói chỉ còn Ghi tăng (đổi tên từ Ghi tăng hàng loạt) và Ghi tăng dư đầu kỳ; ngày bắt đầu, ngừng phân bổ theo từng dòng (Standard, Plus chọn tháng); Thông tin mua của thẻ ghi tăng có link chứng từ gốc</t>
+          <t>Số dư ban đầu tab tiền: bỏ Thêm mới, hiện đủ mọi quỹ của đơn vị, gõ số dư rồi Lưu (lưu theo đơn vị)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E42" s="28" t="inlineStr">
@@ -22899,7 +22899,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong](nhat-ky/2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr"/>
@@ -22910,17 +22910,17 @@
       </c>
       <c r="B43" s="26" t="inlineStr">
         <is>
-          <t>T158</t>
+          <t>T159</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Khởi tạo từ FABi: bỏ bước Đồng bộ bán hàng, popup 3 bước bắt buộc; dùng thử 30 ngày cho mọi gói, hiện ở màn chào, giới thiệu, popup và thanh trên (còn N ngày)</t>
+          <t>Thẻ chi phí: mọi gói chỉ còn Ghi tăng (đổi tên từ Ghi tăng hàng loạt) và Ghi tăng dư đầu kỳ; ngày bắt đầu, ngừng phân bổ theo từng dòng (Standard, Plus chọn tháng); Thông tin mua của thẻ ghi tăng có link chứng từ gốc</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E43" s="28" t="inlineStr">
@@ -22935,7 +22935,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-12-phuongxt-dung-thu-30-ngay.md`</t>
+          <t>[2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong](nhat-ky/2026-10-12-dinhlanphuongipacc-ghi-tang-ngung-tung-dong.md)</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr"/>
@@ -22946,17 +22946,17 @@
       </c>
       <c r="B44" s="25" t="inlineStr">
         <is>
-          <t>T155</t>
+          <t>T158</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
+          <t>Khởi tạo từ FABi: bỏ bước Đồng bộ bán hàng, popup 3 bước bắt buộc; dùng thử 30 ngày cho mọi gói, hiện ở màn chào, giới thiệu, popup và thanh trên (còn N ngày)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E44" s="28" t="inlineStr">
@@ -22971,7 +22971,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-12-trum-dieu-chuyen-chuyen-kho](nhat-ky/2026-10-12-trum-dieu-chuyen-chuyen-kho.md)</t>
+          <t>`2026-10-12-phuongxt-dung-thu-30-ngay.md`</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr"/>
@@ -22982,12 +22982,12 @@
       </c>
       <c r="B45" s="26" t="inlineStr">
         <is>
-          <t>T157</t>
+          <t>T155</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo: bán hàng theo ngày, tổng hợp, chi tiết bán hàng; kho: xuất nhập tồn (mã hàng mở thẻ kho), tổng hợp, chi tiết nhập, xuất, hàng trả</t>
+          <t>Kho tách Xuất điều chuyển, Nhập điều chuyển giữa chi nhánh (tham chiếu nhau, Nợ 1368/Có 152, Nợ 152/Có 3368) và Chuyển kho trong chi nhánh (không hạch toán)</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -23002,12 +23002,12 @@
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>11/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-bao-cao-ban-hang-kho](nhat-ky/2026-10-11-trum-bao-cao-ban-hang-kho.md)</t>
+          <t>[2026-10-12-trum-dieu-chuyen-chuyen-kho](nhat-ky/2026-10-12-trum-dieu-chuyen-chuyen-kho.md)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr"/>
@@ -23018,12 +23018,12 @@
       </c>
       <c r="B46" s="25" t="inlineStr">
         <is>
-          <t>T154</t>
+          <t>T157</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Danh mục sửa theo iFaster: form tài khoản (cấp, loại tài khoản chọn, ô Tổng hợp), hộp quy đổi ĐVT trong hàng hoá, ô chọn nhiều kiểu iFaster toàn hệ thống, thuế ngành nghề chỉ đọc, form Quy đổi ĐVT (hàng áp dụng chọn nhiều, diễn giải tự sinh), lịch chọn ngày hết khoảng trống, nhóm hàng bỏ loại hàng và tồn kho, công việc chỉ mã tên mô tả trạng thái, form bảng giá như iFaster</t>
+          <t>Báo cáo: bán hàng theo ngày, tổng hợp, chi tiết bán hàng; kho: xuất nhập tồn (mã hàng mở thẻ kho), tổng hợp, chi tiết nhập, xuất, hàng trả</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -23043,7 +23043,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-ifaster-cong-thuc](nhat-ky/2026-10-11-trum-danh-muc-ifaster-cong-thuc.md)</t>
+          <t>[2026-10-11-trum-bao-cao-ban-hang-kho](nhat-ky/2026-10-11-trum-bao-cao-ban-hang-kho.md)</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr"/>
@@ -23054,12 +23054,12 @@
       </c>
       <c r="B47" s="26" t="inlineStr">
         <is>
-          <t>T156</t>
+          <t>T154</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Công thức sơ chế, chế biến: form chi tiết bố cục như iPOS Inventory, bỏ mức tăng, giảm tối đa</t>
+          <t>Danh mục sửa theo iFaster: form tài khoản (cấp, loại tài khoản chọn, ô Tổng hợp), hộp quy đổi ĐVT trong hàng hoá, ô chọn nhiều kiểu iFaster toàn hệ thống, thuế ngành nghề chỉ đọc, form Quy đổi ĐVT (hàng áp dụng chọn nhiều, diễn giải tự sinh), lịch chọn ngày hết khoảng trống, nhóm hàng bỏ loại hàng và tồn kho, công việc chỉ mã tên mô tả trạng thái, form bảng giá như iFaster</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -23090,17 +23090,17 @@
       </c>
       <c r="B48" s="25" t="inlineStr">
         <is>
-          <t>T150</t>
+          <t>T156</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thẻ chi phí: số thẻ link xanh mở thẻ; thẻ mở ở chế độ xem, bấm Sửa (Ctrl+E) mới sửa, Huỷ về xem như phiếu chi. Thông tin đơn vị: phương pháp thuế GTGT, TNCN, TNDN lên khối Thông tin kê khai, khoá theo loại hình, nhóm doanh thu, gói</t>
+          <t>Công thức sơ chế, chế biến: form chi tiết bố cục như iPOS Inventory, bỏ mức tăng, giảm tối đa</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E48" s="28" t="inlineStr">
@@ -23115,7 +23115,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-xem-the-thue.md`</t>
+          <t>[2026-10-11-trum-danh-muc-ifaster-cong-thuc](nhat-ky/2026-10-11-trum-danh-muc-ifaster-cong-thuc.md)</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr"/>
@@ -23126,17 +23126,17 @@
       </c>
       <c r="B49" s="26" t="inlineStr">
         <is>
-          <t>T152</t>
+          <t>T150</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
+          <t>Danh sách thẻ chi phí: số thẻ link xanh mở thẻ; thẻ mở ở chế độ xem, bấm Sửa (Ctrl+E) mới sửa, Huỷ về xem như phiếu chi. Thông tin đơn vị: phương pháp thuế GTGT, TNCN, TNDN lên khối Thông tin kê khai, khoá theo loại hình, nhóm doanh thu, gói</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E49" s="28" t="inlineStr">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
+          <t>`2026-10-11-dinhlanphuongipacc-xem-the-thue.md`</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -23162,12 +23162,12 @@
       </c>
       <c r="B50" s="25" t="inlineStr">
         <is>
-          <t>T151</t>
+          <t>T152</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
+          <t>Sản xuất ở Kho theo iPOS Inventory: 4 tab phiếu Xuất sơ chế, Nhập sơ chế, Xuất chế biến, Nhập chế biến (nhập chọn phiếu xuất tham chiếu, chip Chờ nhập, Đã nhập, Đã huỷ, Kế hoạch, Thực tế, hạch toán qua 154, chưa làm số lô); công thức sơ chế, chế biến như IVT</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -23187,7 +23187,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
+          <t>[2026-10-11-trum-san-xuat-ivt](nhat-ky/2026-10-11-trum-san-xuat-ivt.md)</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr"/>
@@ -23198,12 +23198,12 @@
       </c>
       <c r="B51" s="26" t="inlineStr">
         <is>
-          <t>T153</t>
+          <t>T151</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
+          <t>Hàng hoá theo iFaster: khối Thông tin thuế theo ngành nghề con (37 ngành nghề lấy từ iFaster, tự điền nhóm ngành, GTGT, TNCN; TT58 thay TNCN bằng TNDN; TT133, TT99 giữ thuế suất GTGT), nhóm hàng có ngành nghề ngầm định; danh mục Thương hiệu, thương hiệu trên hàng hoá và kho; kho theo dõi, nhà cung cấp; bảng và hộp thêm quy đổi đơn vị tính trong form hàng hoá</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
+          <t>[2026-10-11-trum-hang-hoa-ifaster](nhat-ky/2026-10-11-trum-hang-hoa-ifaster.md)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr"/>
@@ -23234,12 +23234,12 @@
       </c>
       <c r="B52" s="25" t="inlineStr">
         <is>
-          <t>T149</t>
+          <t>T153</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
         <is>
-          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
+          <t>Mọi danh mục vừa một trang như danh sách chứng từ: chỉ bảng cuộn, chân bảng cố định có phân trang (mặc định 50, chọn 50, 100, 200, 500, 1000 dòng), Tổng N dòng, số trang; Hệ thống tài khoản không phân trang, chỉ cố định khung và đếm</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
+          <t>[2026-10-11-trum-danh-muc-mot-trang](nhat-ky/2026-10-11-trum-danh-muc-mot-trang.md)</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr"/>
@@ -23270,12 +23270,12 @@
       </c>
       <c r="B53" s="26" t="inlineStr">
         <is>
-          <t>T148</t>
+          <t>T149</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
+          <t>Mọi ô ngày còn gõ tay dd/mm/yyyy dùng lịch `LichDon`: form danh mục, thẻ phân bổ, Ngày đầu năm ở Hệ thống và các màn khác</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -23306,12 +23306,12 @@
       </c>
       <c r="B54" s="25" t="inlineStr">
         <is>
-          <t>T147</t>
+          <t>T148</t>
         </is>
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
+          <t>Danh mục: bỏ trường Thuộc nhóm ở 5 danh mục nhóm; tài khoản thêm ô tích Tổng hợp (ô chọn cha đổi tên Thuộc tài khoản); cố định độ rộng cột khi chuyển danh mục; nút Tuỳ chọn cột cho mọi danh mục, đủ trường của form</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -23342,12 +23342,12 @@
       </c>
       <c r="B55" s="26" t="inlineStr">
         <is>
-          <t>T146</t>
+          <t>T147</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
+          <t>Danh mục lọc theo thông tư chọn ở Hệ thống (gói và thông tư chọn riêng): thông tư không ghi Nợ/Có (TT152, TT58) ẩn Hệ thống tài khoản, Bút toán tự động, cột tài khoản</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -23378,17 +23378,17 @@
       </c>
       <c r="B56" s="25" t="inlineStr">
         <is>
-          <t>T145</t>
+          <t>T146</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
+          <t>Vẽ lại sơ đồ Khởi tạo danh mục kiểu làn như Thu chi, 7 làn đánh số theo thứ tự phụ thuộc (nền tảng, chi phí, kho, hàng hoá, đối tượng, tiền, hạch toán); chuyển danh mục Tài sản cố định 1.13 sang phân hệ TSCĐ</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E56" s="28" t="inlineStr">
@@ -23403,7 +23403,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
+          <t>[2026-10-11-trum-so-do-danh-muc](nhat-ky/2026-10-11-trum-so-do-danh-muc.md)</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr"/>
@@ -23414,12 +23414,12 @@
       </c>
       <c r="B57" s="26" t="inlineStr">
         <is>
-          <t>T144</t>
+          <t>T145</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
+          <t>Hệ thống, Thông tin đơn vị gom thông tin khai lúc khởi tạo để sửa lại: tên, MST, địa chỉ, loại hình, thông tư áp dụng (doanh nghiệp), nhóm hộ kinh doanh, cách tính thuế TNCN, địa điểm kinh doanh chính, kênh bán</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -23439,7 +23439,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
+          <t>`2026-10-11-phuongxt-thong-tin-don-vi.md`</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr"/>
@@ -23450,12 +23450,12 @@
       </c>
       <c r="B58" s="25" t="inlineStr">
         <is>
-          <t>T143</t>
+          <t>T144</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
         <is>
-          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
+          <t>Form danh mục theo gói: hàng hoá (loại hàng hoá theo iPOS Inventory, đơn vị tính hiện mã và tên), nhóm hàng hoá, đối tượng, nhóm đối tượng, kho, phương thức thanh toán (đồng bộ từ FABi), quỹ tiền (chọn nhiều chi nhánh), lý do; gói Free, Standard ẩn phần tài khoản, ngầm định</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -23475,7 +23475,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
+          <t>`2026-10-11-phuongxt-form-hang-hoa.md`</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr"/>
@@ -23486,12 +23486,12 @@
       </c>
       <c r="B59" s="26" t="inlineStr">
         <is>
-          <t>T142</t>
+          <t>T143</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
+          <t>Gói Free ẩn danh mục Nhóm mục chi phí, Nhóm công việc, Nhóm kho; danh mục Kho chỉ có kho mặc định mỗi chi nhánh theo iPOS Inventory, không thêm mới</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
@@ -23511,7 +23511,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
+          <t>`2026-10-11-phuongxt-an-danh-muc-free.md`</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -23522,12 +23522,12 @@
       </c>
       <c r="B60" s="25" t="inlineStr">
         <is>
-          <t>T141</t>
+          <t>T142</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
+          <t>Bổ sung chi nhánh khi đang dùng: Danh mục chi nhánh có Thêm chi nhánh từ FABi (chỉ cửa hàng chưa dùng kế toán, lên sổ từ ngày đầu năm, mở khai số dư quỹ tiền chi nhánh mới); Bàn làm việc nhắc cửa hàng FABi mới chưa lên sổ</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
+          <t>`2026-10-11-phuongxt-them-chi-nhanh-fabi.md`</t>
         </is>
       </c>
       <c r="H60" s="13" t="inlineStr"/>
@@ -23558,17 +23558,17 @@
       </c>
       <c r="B61" s="26" t="inlineStr">
         <is>
-          <t>T136</t>
+          <t>T141</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
+          <t>Màn Số dư ban đầu theo gói, chế độ: gói Free chỉ số dư tiền (tab ở Thu chi); Standard tiền, công nợ, tồn kho; Plus, Pro thêm số dư tài khoản</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E61" s="28" t="inlineStr">
@@ -23583,7 +23583,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
+          <t>`2026-10-11-phuongxt-so-du-ban-dau.md`</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -23594,12 +23594,12 @@
       </c>
       <c r="B62" s="25" t="inlineStr">
         <is>
-          <t>T137</t>
+          <t>T136</t>
         </is>
       </c>
       <c r="C62" s="13" t="inlineStr">
         <is>
-          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
+          <t>Danh mục nhóm: nhóm đối tượng, nhóm kho, nhóm mục chi phí, nhóm công việc, nhóm hàng hoá. Hàng hoá chọn nhóm thì tự điền TK, mục chi phí, phương pháp tính giá, thuế suất theo nhóm. Kho thêm mục chi phí, công việc ngầm định, địa chỉ, SĐT, người liên hệ, ghi chú. Đối tượng và người dùng có ô bắt buộc tích "đã đồng ý chia sẻ thông tin cá nhân". Màn Người dùng có panel Thêm, Sửa như Danh mục</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -23630,17 +23630,17 @@
       </c>
       <c r="B63" s="26" t="inlineStr">
         <is>
-          <t>T135</t>
+          <t>T137</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
+          <t>Danh mục phương thức thanh toán (loại chứng từ tiền, TK Nợ, đối tượng, công việc, mục chi phí ngầm định). Ô phương thức thanh toán trên các phiếu bán hàng. Hộp đồng bộ hoá đơn POS có tích "Tự động hạch toán chứng từ theo phương thức thanh toán": Nợ TK của phương thức / Có 131, kéo chi tiết thì mỗi hoá đơn một phiếu, kéo tổng hợp thì mỗi ngày mỗi phương thức một phiếu</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E63" s="28" t="inlineStr">
@@ -23655,7 +23655,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
+          <t>[2026-10-11-trum-nhom-danh-muc-pttt](nhat-ky/2026-10-11-trum-nhom-danh-muc-pttt.md)</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr"/>
@@ -23666,17 +23666,17 @@
       </c>
       <c r="B64" s="25" t="inlineStr">
         <is>
-          <t>T134</t>
+          <t>T135</t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
+          <t>Thẻ chi phí phân bổ bản 2: một thẻ nhiều dòng (tab Chi tiết phân bổ, Đã phân bổ có cộng từng khoản), Thông tin mua, ngừng phân bổ theo dòng; danh sách thẻ kiểu danh sách chứng từ (Kỳ số liệu, Ẩn thẻ hết phân bổ, phân trang, khung chi tiết); Ghi tăng hàng loạt từ phiếu chi; mã CCDC chọn từ danh mục hàng hoá; báo cáo Bảng chi tiết phân bổ chi phí; Năm làm việc hiện tại ở Thông tin đơn vị</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E64" s="28" t="inlineStr">
@@ -23691,7 +23691,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
+          <t>`2026-10-11-dinhlanphuongipacc-the-phan-bo-ban-2.md`</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr"/>
@@ -23702,12 +23702,12 @@
       </c>
       <c r="B65" s="26" t="inlineStr">
         <is>
-          <t>T133</t>
+          <t>T134</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
+          <t>Mẫu in phiếu tự cân đối khi đổi khổ dọc, ngang, A4, A5: cột bảng chia theo tỷ lệ, chữ bảng co khi khổ hẹp, thông tin một cột ở A5 dọc, số xuống dòng thay vì đè ô</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -23722,12 +23722,12 @@
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>11/10/2026</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-tong-quan.md`</t>
+          <t>`2026-10-11-trum-mau-in-doi-kho.md`</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr"/>
@@ -23738,17 +23738,17 @@
       </c>
       <c r="B66" s="25" t="inlineStr">
         <is>
-          <t>T132</t>
+          <t>T133</t>
         </is>
       </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
+          <t>Tổng quan làm lại: 4 thẻ lời lỗ và tiền, 8 chỉ số sức khoẻ có đèn, thác nước lợi nhuận, xu hướng 4 tháng, dòng tiền, hiệu quả chi nhánh, cơ cấu chi phí; lọc kỳ, so sánh, chi nhánh; tuỳ chỉnh khối (QD46)</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E66" s="28" t="inlineStr">
@@ -23763,7 +23763,7 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
+          <t>`2026-10-10-trum-tong-quan.md`</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr"/>
@@ -23774,12 +23774,12 @@
       </c>
       <c r="B67" s="26" t="inlineStr">
         <is>
-          <t>T131</t>
+          <t>T132</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
+          <t>Mọi danh sách phiếu (cả Xuất bán POS) thêm cột Ngày tạo, Người tạo: phiếu lưu trong phiên ghi giờ lưu, người đăng nhập; phiếu mẫu đồng bộ ghi Hệ thống; phiếu mẫu nhập tay ghi một nhân viên</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -23799,7 +23799,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-ngay-nguoi-tao.md`</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
@@ -23810,12 +23810,12 @@
       </c>
       <c r="B68" s="25" t="inlineStr">
         <is>
-          <t>T130</t>
+          <t>T131</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
+          <t>Chi tiết phiếu xuất, nhập điều chỉnh bỏ cột Thuế suất, Tiền thuế (dải đáy chỉ Tổng tiền); gói Free ẩn thêm Đơn giá, Thành tiền, dải tổng tiền và cột Tổng tiền ở danh sách</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-an-cot-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr"/>
@@ -23846,12 +23846,12 @@
       </c>
       <c r="B69" s="26" t="inlineStr">
         <is>
-          <t>T129</t>
+          <t>T130</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
+          <t>Bộ lọc danh sách Kiểm kê, Điều chỉnh kho thêm ô Kho (theo kho của phiếu), hiện sẵn ngoài thanh lọc</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -23871,7 +23871,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
@@ -23882,12 +23882,12 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>T128</t>
+          <t>T129</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
+          <t>Phiếu xuất điều chỉnh, nhập điều chỉnh chỉ xem: bỏ Sửa, Ctrl+E, Sao chép, Xoá chứng từ, xoá hàng loạt. Xoá phiếu kiểm kê (ở form hoặc hàng loạt) tự xoá phiếu điều chỉnh liên quan, hộp xác nhận báo trước</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="G70" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
+          <t>`2026-10-10-phuongxt-khoa-phieu-dieu-chinh.md`</t>
         </is>
       </c>
       <c r="H70" s="13" t="inlineStr"/>
@@ -23918,12 +23918,12 @@
       </c>
       <c r="B71" s="26" t="inlineStr">
         <is>
-          <t>T127</t>
+          <t>T128</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
+          <t>Sơ đồ Kho gói Free: bấm Kiểm kê kho mở danh sách kiểm kê; Xuất điều chỉnh, Nhập điều chỉnh mở màn Điều chỉnh kho đúng tab con (`?loai=xdc`, `?loai=ndc`)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
+          <t>`2026-10-10-phuongxt-noi-so-do-kho.md`</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr"/>
@@ -23954,12 +23954,12 @@
       </c>
       <c r="B72" s="25" t="inlineStr">
         <is>
-          <t>T126</t>
+          <t>T127</t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
+          <t>Mọi danh sách phiếu có cột Tham chiếu: phiếu thu, chi sinh từ mua, bán; phiếu điều chỉnh sinh từ kiểm kê; phiếu gốc của phiếu được sinh ra; bấm số phiếu để mở</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-cot-tham-chieu.md`</t>
         </is>
       </c>
       <c r="H72" s="13" t="inlineStr"/>
@@ -23990,12 +23990,12 @@
       </c>
       <c r="B73" s="26" t="inlineStr">
         <is>
-          <t>T125</t>
+          <t>T126</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
+          <t>Kiểm kê có chênh lệch tự sinh phiếu Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa) vào màn mới Điều chỉnh kho (mọi gói, hai tab con Xuất điều chỉnh, Nhập điều chỉnh, không chip trạng thái, không Thêm mới); tham chiếu hai chiều</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
+          <t>`2026-10-10-phuongxt-dieu-chinh-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr"/>
@@ -24026,12 +24026,12 @@
       </c>
       <c r="B74" s="25" t="inlineStr">
         <is>
-          <t>T124</t>
+          <t>T125</t>
         </is>
       </c>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
+          <t>Mọi phiếu đang thêm mới: bấm Huỷ, nút đóng (X) hoặc Esc thì hỏi "Xác nhận đóng phiếu!" (Bỏ qua, Xác nhận) trước khi bỏ phiếu chưa lưu</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -24051,7 +24051,7 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
+          <t>`2026-10-10-phuongxt-canh-bao-dong-phieu-moi.md`</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr"/>
@@ -24062,12 +24062,12 @@
       </c>
       <c r="B75" s="26" t="inlineStr">
         <is>
-          <t>T123</t>
+          <t>T124</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
+          <t>Phiếu kiểm kê: bỏ Đối tượng, Người giao nhận, Địa chỉ, Mã số thuế; đầu phiếu hai dòng (Kho kiểm kê, Nhân viên thực hiện; Ghi chú); bỏ tab Hạch toán; bảng chi tiết bỏ Kho, Số lượng, Đơn giá, Thành tiền, Thuế, thay bằng Tồn hệ thống, Tồn thực tế, Chênh lệch, Loại (Xuất điều chỉnh, Nhập điều chỉnh), Ghi chú; bỏ dải tổng tiền</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-kiem-ke.md`</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr"/>
@@ -24098,17 +24098,17 @@
       </c>
       <c r="B76" s="25" t="inlineStr">
         <is>
-          <t>T122</t>
+          <t>T123</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
+          <t>Sơ đồ quy trình Kho gói Free vẽ lại dạng luồng: Mua hàng, Bán hàng tổng hợp thành Tồn hệ thống (ô kết quả, không phải màn hình), so sánh với Kiểm kê kho, tách ra Xuất điều chỉnh (thiếu), Nhập điều chỉnh (thừa)</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E76" s="28" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="G76" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-kho-free.md`</t>
         </is>
       </c>
       <c r="H76" s="13" t="inlineStr"/>
@@ -24134,17 +24134,17 @@
       </c>
       <c r="B77" s="26" t="inlineStr">
         <is>
-          <t>T121</t>
+          <t>T122</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
+          <t>Ẩn tạm 23 mã sổ, BCTC, tờ khai do agent tự dựng theo từng thông tư (QD45); giữ TT58 theo file, TT152 theo iFaster; link cũ hiện "Báo cáo chưa có mẫu"</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E77" s="28" t="inlineStr">
@@ -24159,7 +24159,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
+          <t>`2026-10-10-trum-an-tam-bao-cao.md`</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr"/>
@@ -24170,17 +24170,17 @@
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>T111</t>
+          <t>T121</t>
         </is>
       </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
+          <t>Sơ đồ quy trình Bán hàng gói Free: bỏ ô Đơn POS từ FABi trùng với nhãn làn Bán hàng từ FABi, mũi tên đồng bộ đi thẳng sang Xuất bán POS; Quy trình gói Free bỏ khung Thiết lập &amp; Thao tác</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E78" s="28" t="inlineStr">
@@ -24195,7 +24195,7 @@
       </c>
       <c r="G78" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
+          <t>`2026-10-10-phuongxt-bo-o-trung-so-do-ban-hang.md`</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr"/>
@@ -24206,12 +24206,12 @@
       </c>
       <c r="B79" s="26" t="inlineStr">
         <is>
-          <t>T112</t>
+          <t>T111</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
+          <t>Báo cáo: ô Khoảng ngày và nút Xem báo cáo nằm trong cột Bộ lọc bên trái (18 màn không có cột lọc giữ trên thanh trên); cột tỷ lệ và mọi cột không còn hẹp tới mức vỡ chữ tiêu đề</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -24242,17 +24242,17 @@
       </c>
       <c r="B80" s="25" t="inlineStr">
         <is>
-          <t>T118</t>
+          <t>T112</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
+          <t>Màn Thiết kế mẫu in làm lại ba vùng (danh sách mẫu, tờ in, thuộc tính); khung phiếu in vẽ lại, bổ sung trường theo thông tư; số bằng chữ khớp dòng Cộng, Nợ/Có đúng phiếu</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E80" s="28" t="inlineStr">
@@ -24267,7 +24267,7 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
+          <t>`2026-10-10-trum-bo-loc-ben-mau-in.md`</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr"/>
@@ -24278,12 +24278,12 @@
       </c>
       <c r="B81" s="26" t="inlineStr">
         <is>
-          <t>T117</t>
+          <t>T118</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
+          <t>Danh sách Xuất bán POS: dải đối soát đơn POS kiểu iPOS Inventory: nút Đã đồng bộ, Chưa đồng bộ; số liệu tổng số hoá đơn POS, IACC, số món, mã hoá đơn cuối, lần đồng bộ cuối; bảng hoá đơn chưa đồng bộ (mã hoá đơn, thời gian, tên món, ĐVT, số lượng, lý do lỗi); bỏ chip Tất cả, Chưa ghi sổ, Đã ghi sổ, Lệch đối soát, nút Ghi chú FABi, xoá hàng loạt; thêm lọc Hàng hoá, Theo dõi tồn kho</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -24303,7 +24303,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
+          <t>`2026-10-10-phuongxt-doi-soat-pos.md`</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr"/>
@@ -24314,12 +24314,12 @@
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>T116</t>
+          <t>T117</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
+          <t>Xuất bán POS: nút Đồng bộ POS (trước là Tải từ FABi; tên ngắn để thanh công cụ không đè chip trạng thái) mở hộp chọn khoảng thời gian, chi nhánh (mặc định chi nhánh đang chọn, tất cả chi nhánh thì phải chọn), ô tích Bỏ qua hoá đơn đã đồng bộ (tích sẵn)</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -24350,12 +24350,12 @@
       </c>
       <c r="B83" s="26" t="inlineStr">
         <is>
-          <t>T115</t>
+          <t>T116</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
+          <t>Danh sách Xuất bán POS: bộ lọc thêm Khách hàng, Kênh bán, Phương thức thanh toán (chỉ khi đồng bộ chi tiết; tổng hợp theo kênh bỏ ở bộ lọc và đầu phiếu)</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -24386,12 +24386,12 @@
       </c>
       <c r="B84" s="25" t="inlineStr">
         <is>
-          <t>T114</t>
+          <t>T115</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
+          <t>Danh sách Xuất bán POS: bỏ cột và ô lọc Nguồn (chỉ có FABi); nhãn cách đồng bộ ghi gọn Chi tiết hoặc Tổng hợp</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -24422,12 +24422,12 @@
       </c>
       <c r="B85" s="26" t="inlineStr">
         <is>
-          <t>T113</t>
+          <t>T114</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
+          <t>Danh mục hàng hoá có trường Theo dõi tồn kho (panel, cột danh sách; món chế biến không theo dõi, hàng bán lại và nguyên vật liệu có); Xuất bán POS có cột Theo dõi tồn kho ô tích chỉ xem, cột cuối cố định phải</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -24458,17 +24458,17 @@
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>T119</t>
+          <t>T113</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
         <is>
-          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
+          <t>Cấu hình cách đồng bộ bán hàng FABi (Hệ thống, Cấu hình kế toán): Chi tiết theo hoá đơn (mỗi hoá đơn FABi một chứng từ Xuất bán POS, có giờ, kênh, cách thanh toán, món của đơn) hoặc Tổng hợp theo kênh (mỗi ngày, chi nhánh, kênh một chứng từ, mặc định); tổng doanh thu, thuế không đổi</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E86" s="28" t="inlineStr">
@@ -24483,7 +24483,7 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
+          <t>`2026-10-10-phuongxt-dong-bo-fabi.md`</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr"/>
@@ -24494,12 +24494,12 @@
       </c>
       <c r="B87" s="26" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T119</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
+          <t>Thiết kế lại màn hình Gói thuê bao và bộ logo nhận diện 4 gói Free, Standard, Plus, Pro (gradient, biểu tượng vector)</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-mau-tt58.md`</t>
+          <t>`2026-10-10-trum-goi-thue-bao-logo.md`</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr"/>
@@ -24530,17 +24530,17 @@
       </c>
       <c r="B88" s="25" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T108</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
+          <t>Mẫu in phiếu và mẫu sổ, BCTC riêng TT58: Thông tin đơn vị chọn phương pháp thuế GTGT, TNDN quyết định bộ sổ (TH1–TH4); 11 sổ S1–S4d đúng cột, dòng in sẵn, công thức, có tiêu đề cột 2 tầng; 3.2.5 đổi S1/S2a/S3a theo trường hợp; B01-DNSN 14 chỉ tiêu, B02-DNSN 5 chỉ tiêu; phiếu 01-TT, 02-TT, 01-VT, 02-VT ký hiệu và khối ký TT58</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
         <is>
-          <t>dinhlanphuongipacc</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E88" s="28" t="inlineStr">
@@ -24555,7 +24555,7 @@
       </c>
       <c r="G88" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
+          <t>`2026-10-10-trum-mau-tt58.md`</t>
         </is>
       </c>
       <c r="H88" s="13" t="inlineStr"/>
@@ -24566,17 +24566,17 @@
       </c>
       <c r="B89" s="26" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T107</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
+          <t>Thẻ chi phí phân bổ 8.1.1 (Danh sách thẻ chi phí): thẻ dùng chung chi phí trả trước, CCDC, TSCĐ; thẻ dư đầu kỳ; lịch phân bổ sửa được từng dòng, ngừng phân bổ; tạo thẻ từ phiếu chi lý do Chi phí chờ phân bổ; sơ đồ Chi phí phân bổ; 4 lý do chi mới; ngày đầu năm ở Thông tin đơn vị chặn chứng từ thêm mới trước ngày này</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>dinhlanphuongipacc</t>
         </is>
       </c>
       <c r="E89" s="28" t="inlineStr">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
+          <t>`2026-10-10-dinhlanphuongipacc-the-chi-phi-phan-bo.md`</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr"/>
@@ -24602,12 +24602,12 @@
       </c>
       <c r="B90" s="25" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T106</t>
         </is>
       </c>
       <c r="C90" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
+          <t>Xuất bán POS: bảng chi tiết thêm % CK, Tiền CK, % Phí dịch vụ, Phí dịch vụ, Giảm thuế GTGT, Phí vận chuyển (hai cột sau ẩn sẵn, bật ở Tuỳ chỉnh giao diện), Doanh thu trước thuế; dòng Tổng cộng thẳng cột, bỏ cột Tổng tiền; cột #, Mã hàng, Hàng hoá, ĐVT cố định trái; dải đáy còn Phiếu giảm giá (hàng ngay trên Tổng tiền), Tổng tiền; bỏ nút Phát hành HĐĐT; đầu phiếu dạng thông tin gọn 4 cột × 2 hàng; Diễn giải đổi thành Ghi chú dưới Kênh bán</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr">
@@ -24638,12 +24638,12 @@
       </c>
       <c r="B91" s="26" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T103</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
+          <t>Xuất bán POS: thuế từng món cộng lại bằng thuế GTGT của ngày (phần lệch làm tròn dồn vào món thuế lớn nhất)</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -24674,12 +24674,12 @@
       </c>
       <c r="B92" s="25" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T105</t>
         </is>
       </c>
       <c r="C92" s="13" t="inlineStr">
         <is>
-          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
+          <t>Form mọi phiếu (form chung và Xuất bán POS): đầu phiếu đứng yên, chỉ vùng bảng chi tiết cuộn, tiêu đề cột dính; phần tổng thành dải cố định ở đáy form (QD33)</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr">
@@ -24710,12 +24710,12 @@
       </c>
       <c r="B93" s="26" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T104</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
+          <t>Xuất bán POS: số chứng từ là số hoá đơn FABi (`soBH` 12 ký tự, Thu chi tham chiếu theo); ghi chú gọn một dòng; bỏ ô Cửa hàng, Số đơn POS, tab Thanh toán, Đơn POS gốc, cột Ghi chú; Diễn giải cột trái; phần tổng thành dải cố định ở đáy form</t>
         </is>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -24746,12 +24746,12 @@
       </c>
       <c r="B94" s="25" t="inlineStr">
         <is>
-          <t>T100</t>
+          <t>T102</t>
         </is>
       </c>
       <c r="C94" s="13" t="inlineStr">
         <is>
-          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
+          <t>Chứng từ Xuất bán POS 3.1.1 vẽ lại theo form chung IACC: đầu phiếu 3 cột chỉ xem (khách hàng, cửa hàng, kênh bán, phương thức TT, thời gian xuất, số đơn POS), bảng món có giảm giá, ghi chú, khối thanh toán như iFaster; nút Phát hành HĐĐT</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr">
@@ -24771,7 +24771,7 @@
       </c>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
+          <t>`2026-10-10-phuongxt-xuat-ban-pos.md`</t>
         </is>
       </c>
       <c r="H94" s="13" t="inlineStr"/>
@@ -24782,12 +24782,12 @@
       </c>
       <c r="B95" s="26" t="inlineStr">
         <is>
-          <t>T99</t>
+          <t>T100</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
+          <t>Bỏ tiện ích 11.1 Đồng bộ bán hàng, 11.2 Xuất kho theo định lượng ở mọi gói; ô Đơn POS từ FABi trên sơ đồ Bán hàng chỉ để xem; gói Free ẩn tạm phân hệ Tiện ích và khung Tiện ích liên quan dưới sơ đồ</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -24818,12 +24818,12 @@
       </c>
       <c r="B96" s="25" t="inlineStr">
         <is>
-          <t>T98</t>
+          <t>T99</t>
         </is>
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
+          <t>Bỏ Báo cáo bán hàng 3.2.1 và Báo cáo doanh thu 3.2.3 ở mọi gói (`DA_BO` trong `plan.ts`); liên kết cũ trỏ sang Sổ doanh thu bán hàng 3.2.5</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -24854,17 +24854,17 @@
       </c>
       <c r="B97" s="26" t="inlineStr">
         <is>
-          <t>T97</t>
+          <t>T98</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
+          <t>Sơ đồ Quy trình Bán hàng gói Free kiểu hội tụ: làn Bán hàng từ FABi (Đơn POS từ FABi, mũi tên chữ đồng bộ, Xuất bán POS) về khối Báo cáo; 3.2.5, 3.2.1, 3.2.3 tự hiện khi T97 mở cho Free</t>
         </is>
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E97" s="28" t="inlineStr">
@@ -24879,7 +24879,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
+          <t>`2026-10-10-phuongxt-so-do-ban-hang-free.md`</t>
         </is>
       </c>
       <c r="H97" s="5" t="inlineStr"/>
@@ -24890,17 +24890,17 @@
       </c>
       <c r="B98" s="25" t="inlineStr">
         <is>
-          <t>T96</t>
+          <t>T97</t>
         </is>
       </c>
       <c r="C98" s="13" t="inlineStr">
         <is>
-          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
+          <t>Bộ báo cáo gói Free theo bộ hộ kinh doanh của iFaster (17 báo cáo, Báo cáo bán hàng theo T99 dùng Sổ doanh thu); thêm Tổng hợp quỹ tiền, Báo cáo dòng tiền, Mua hàng theo ngày, Sổ chi phí; báo cáo khai thông tư áp dụng, chỉ hiện khi gói có tính năng và thông tư đang chọn áp dụng (QD42)</t>
         </is>
       </c>
       <c r="D98" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E98" s="28" t="inlineStr">
@@ -24915,7 +24915,7 @@
       </c>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
+          <t>`2026-10-10-trum-bao-cao-goi-thong-tu.md`</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr"/>
@@ -24926,12 +24926,12 @@
       </c>
       <c r="B99" s="26" t="inlineStr">
         <is>
-          <t>T95</t>
+          <t>T96</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
+          <t>Danh sách thu chi 2.1.1: thêm cột Lý do thu, chi sau Diễn giải, lấy như form; chuyển quỹ để trống</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -24962,12 +24962,12 @@
       </c>
       <c r="B100" s="25" t="inlineStr">
         <is>
-          <t>T94</t>
+          <t>T95</t>
         </is>
       </c>
       <c r="C100" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
+          <t>Form mọi phiếu: nút Tuỳ chỉnh giao diện ra ngoài thanh đáy, cạnh nút In, bỏ khỏi menu Tiện ích</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -24998,12 +24998,12 @@
       </c>
       <c r="B101" s="26" t="inlineStr">
         <is>
-          <t>T93</t>
+          <t>T94</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
+          <t>Danh sách mua hàng, bán hàng: Bộ lọc thêm Kho, Hàng hoá; danh sách mua hàng gói dưới Pro thêm cột Kho; cột mới chưa có trong thứ tự cột đã lưu đứng sau cột kề trước theo mặc định</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
@@ -25023,7 +25023,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
+          <t>`2026-10-10-phuongxt-loc-kho-hang.md`</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
@@ -25034,12 +25034,12 @@
       </c>
       <c r="B102" s="25" t="inlineStr">
         <is>
-          <t>T92</t>
+          <t>T93</t>
         </is>
       </c>
       <c r="C102" s="13" t="inlineStr">
         <is>
-          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
+          <t>Danh sách mua hàng, bán hàng: cột Đã trả, Còn phải trả có số tổng ở dòng Tổng trang, Tổng cộng và khi gom nhóm</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -25070,12 +25070,12 @@
       </c>
       <c r="B103" s="26" t="inlineStr">
         <is>
-          <t>T91</t>
+          <t>T92</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
+          <t>Danh sách mua hàng, bán hàng: thêm cột Ký hiệu HĐ, Số hoá đơn, Ngày hoá đơn, Hạn thanh toán, Đã trả (Đã thu), Còn phải trả (Còn phải thu); mặc định ẩn, bật ở Tuỳ chỉnh cột, nút Mặc định ẩn lại</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -25106,12 +25106,12 @@
       </c>
       <c r="B104" s="25" t="inlineStr">
         <is>
-          <t>T90</t>
+          <t>T91</t>
         </is>
       </c>
       <c r="C104" s="13" t="inlineStr">
         <is>
-          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
+          <t>Phiếu mua, bán chưa thanh toán hoặc thanh toán một phần: tiện ích Thanh toán ngay / Thu tiền ngay, chọn hình thức, quỹ, ngày, số tiền thì sinh phiếu thu, chi; phiếu gốc hiện số đã trả và mã phiếu; trạng thái danh sách tính theo số đã trả</t>
         </is>
       </c>
       <c r="D104" s="12" t="inlineStr">
@@ -25131,7 +25131,7 @@
       </c>
       <c r="G104" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
+          <t>`2026-10-10-phuongxt-thanh-toan-sau.md`</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr"/>
@@ -25142,12 +25142,12 @@
       </c>
       <c r="B105" s="26" t="inlineStr">
         <is>
-          <t>T89</t>
+          <t>T90</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
+          <t>Đầu phiếu mua, bán: bỏ ô Nhân viên thực hiện, Người giao hàng / Người mua hàng đổi thành Người giao dịch; hàng 1 Đối tượng, Mã số thuế; hàng 2 Địa chỉ, Người giao dịch; Ghi chú kéo dài (QD33)</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -25178,17 +25178,17 @@
       </c>
       <c r="B106" s="25" t="inlineStr">
         <is>
-          <t>T88</t>
+          <t>T89</t>
         </is>
       </c>
       <c r="C106" s="13" t="inlineStr">
         <is>
-          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
+          <t>Tuỳ chỉnh giao diện phiếu mọi phiếu: thêm khối Đầu phiếu (bật tắt ô không bắt buộc, ô sau dồn lên) và Chân phiếu (dòng Tổng cộng, khối tổng tiền) (QD33)</t>
         </is>
       </c>
       <c r="D106" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E106" s="28" t="inlineStr">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="G106" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
+          <t>`2026-10-10-phuongxt-tuy-chinh-dau-chan-phieu.md`</t>
         </is>
       </c>
       <c r="H106" s="13" t="inlineStr"/>
@@ -25214,12 +25214,12 @@
       </c>
       <c r="B107" s="26" t="inlineStr">
         <is>
-          <t>T80</t>
+          <t>T88</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
+          <t>Danh mục đơn vị tính 1.3: 36 đơn vị cơ bản F&amp;B, mã viết hoa không dấu (CAI là Cái), giữ cột Mô tả; mọi ô chọn ĐVT trong panel danh mục lấy từ danh mục này</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
@@ -25239,7 +25239,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
+          <t>`2026-10-10-trum-don-vi-tinh.md`</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
@@ -25250,12 +25250,12 @@
       </c>
       <c r="B108" s="25" t="inlineStr">
         <is>
-          <t>T87</t>
+          <t>T80</t>
         </is>
       </c>
       <c r="C108" s="13" t="inlineStr">
         <is>
-          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
+          <t>Hộp tìm màn hình Ctrl K kiểu iPOS Inventory: mục Vừa mở, Gợi ý, ô biểu tượng, đường dẫn phân hệ, thanh phím tắt; gõ tên quen vẫn ra</t>
         </is>
       </c>
       <c r="D108" s="12" t="inlineStr">
@@ -25286,12 +25286,12 @@
       </c>
       <c r="B109" s="26" t="inlineStr">
         <is>
-          <t>T73</t>
+          <t>T87</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
+          <t>Panel danh mục: ô Nhóm điền sẵn nhóm của dòng đang sửa</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -25322,17 +25322,17 @@
       </c>
       <c r="B110" s="25" t="inlineStr">
         <is>
-          <t>T86</t>
+          <t>T73</t>
         </is>
       </c>
       <c r="C110" s="13" t="inlineStr">
         <is>
-          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
+          <t>Tối ưu phản hồi thao tác: panel tài khoản lần mở đầu hết khung hở 133ms (còn 33ms)</t>
         </is>
       </c>
       <c r="D110" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E110" s="28" t="inlineStr">
@@ -25347,7 +25347,7 @@
       </c>
       <c r="G110" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
+          <t>`2026-10-10-trum-ctrl-k-toi-uu.md`</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr"/>
@@ -25358,12 +25358,12 @@
       </c>
       <c r="B111" s="26" t="inlineStr">
         <is>
-          <t>T85</t>
+          <t>T86</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
+          <t>Tuỳ chỉnh giao diện phiếu: bật tắt được từng cột của bảng chi tiết (mỗi cột một mục, theo thứ tự trên bảng); Tổng tiền là cột cuối dòng phiếu mua</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -25394,12 +25394,12 @@
       </c>
       <c r="B112" s="25" t="inlineStr">
         <is>
-          <t>T84</t>
+          <t>T85</t>
         </is>
       </c>
       <c r="C112" s="13" t="inlineStr">
         <is>
-          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
+          <t>Phiếu mua, bán trả tiền ngay: lưu phiếu thì sinh phiếu thu, chi bên Thu chi 2.1.1 (mua, trả lại hàng bán thì chi; bán, trả lại hàng mua thì thu), phiếu gốc hiện mã chứng từ; còn phiếu thu, chi thì phải xoá phiếu đó trước mới xoá được phiếu gốc</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -25419,7 +25419,7 @@
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
+          <t>`2026-10-10-phuongxt-phieu-chi-tu-mua-hang.md`</t>
         </is>
       </c>
       <c r="H112" s="13" t="inlineStr"/>
@@ -25430,12 +25430,12 @@
       </c>
       <c r="B113" s="26" t="inlineStr">
         <is>
-          <t>T83</t>
+          <t>T84</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
+          <t>Phiếu mua hàng: bảng chi tiết (form và khung dưới danh sách) thêm cột Tiền trước thuế (Thành tiền trừ chiết khấu, trước cột thuế), Tổng tiền, Giá trị nhập kho (cuối dòng); khối tổng chỉ còn Tổng tiền</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -25455,7 +25455,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
+          <t>`2026-10-10-phuongxt-gia-tri-nhap-kho-dong.md`</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
@@ -25466,12 +25466,12 @@
       </c>
       <c r="B114" s="25" t="inlineStr">
         <is>
-          <t>T82</t>
+          <t>T83</t>
         </is>
       </c>
       <c r="C114" s="13" t="inlineStr">
         <is>
-          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
+          <t>Phiếu mua, hoá đơn bán hàng, phiếu trả lại có kho: gói dưới Pro chọn một kho ở đầu phiếu, bỏ cột Kho trên dòng; gói Pro giữ kho trên dòng; chi nhánh một kho thì phiếu mới điền sẵn. Thông tin hoá đơn mua, bán thành cột riêng cạnh ngày, số phiếu, bắt buộc nhập (QD33)</t>
         </is>
       </c>
       <c r="D114" s="12" t="inlineStr">
@@ -25502,12 +25502,12 @@
       </c>
       <c r="B115" s="26" t="inlineStr">
         <is>
-          <t>T27</t>
+          <t>T82</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
+          <t>Gói Free: khung chi tiết dưới mọi danh sách chứng từ (cả Bán hàng POS) bỏ tab Ghi sổ, như form</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -25538,17 +25538,17 @@
       </c>
       <c r="B116" s="25" t="inlineStr">
         <is>
-          <t>T81</t>
+          <t>T27</t>
         </is>
       </c>
       <c r="C116" s="13" t="inlineStr">
         <is>
-          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
+          <t>Danh sách chứng từ 2.1.1: khung chi tiết bên dưới lấy dòng phiếu giống form của cùng phiếu; phiếu thu, chi có cột Lý do thu, chi và Đối tượng</t>
         </is>
       </c>
       <c r="D116" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E116" s="28" t="inlineStr">
@@ -25563,7 +25563,7 @@
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
+          <t>`2026-10-10-phuongxt-chi-tiet-thu-chi-ly-do.md`</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr"/>
@@ -25574,12 +25574,12 @@
       </c>
       <c r="B117" s="26" t="inlineStr">
         <is>
-          <t>T79</t>
+          <t>T81</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
+          <t>Panel bên phải kiểu mới (mục lục trái, khối thẻ, công tắc, chân trạng thái), Tuỳ chỉnh báo cáo hai cột, Tuỳ chỉnh giao diện phiếu; mở đóng mượt (đo 331ms, mục tiêu ≤ 100ms); ô chọn đẹp, có tìm, dựng option khi mở</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -25610,12 +25610,12 @@
       </c>
       <c r="B118" s="25" t="inlineStr">
         <is>
-          <t>T70</t>
+          <t>T79</t>
         </is>
       </c>
       <c r="C118" s="13" t="inlineStr">
         <is>
-          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
+          <t>Hộp đồng bộ dữ liệu kiểu iPOS Inventory cho Tiện ích Đồng bộ bán hàng từ POS (11.1) và Tải hoá đơn đầu vào từ iPOS Invoice (11.4): khoảng ngày, chọn kho hoặc chi nhánh có tìm, món bán, đồng bộ lại</t>
         </is>
       </c>
       <c r="D118" s="12" t="inlineStr">
@@ -25646,12 +25646,12 @@
       </c>
       <c r="B119" s="26" t="inlineStr">
         <is>
-          <t>T76</t>
+          <t>T70</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
+          <t>Mọi panel bên phải rộng hơn (min(880px, 72vw)), lưới 3 cột, chia khối: panel Thêm/Sửa từng danh mục đủ trường theo bảng DM_ (truong-dm.ts), Tuỳ chỉnh báo cáo, Đối soát</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -25682,17 +25682,17 @@
       </c>
       <c r="B120" s="25" t="inlineStr">
         <is>
-          <t>T78</t>
+          <t>T76</t>
         </is>
       </c>
       <c r="C120" s="13" t="inlineStr">
         <is>
-          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
+          <t>Danh mục Hệ thống tài khoản 1.1 dạng cây theo chế độ TT133, TT99; panel Thêm/Sửa tài khoản đủ trường DM_ACCOUNT (QD41)</t>
         </is>
       </c>
       <c r="D120" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E120" s="28" t="inlineStr">
@@ -25702,12 +25702,12 @@
       </c>
       <c r="F120" s="12" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="G120" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
+          <t>`2026-10-10-trum-panel-dong-bo.md`</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr"/>
@@ -25718,12 +25718,12 @@
       </c>
       <c r="B121" s="26" t="inlineStr">
         <is>
-          <t>T77</t>
+          <t>T78</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
+          <t>Đầu mọi phiếu bỏ ô Diễn giải (Ghi chú chép sang), hai cột trái đều hàng. Form Mua hàng: Tiền mặt ngay thì chọn quỹ tiền mặt, Chuyển khoản ngay thì chọn quỹ ngân hàng. Thu, chi ngân hàng ghi nhãn Quỹ ngân hàng</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -25743,7 +25743,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-chon-quy.md`</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr"/>
@@ -25754,12 +25754,12 @@
       </c>
       <c r="B122" s="25" t="inlineStr">
         <is>
-          <t>T69</t>
+          <t>T77</t>
         </is>
       </c>
       <c r="C122" s="13" t="inlineStr">
         <is>
-          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
+          <t>Đầu phiếu thu chi, chuyển quỹ: bỏ ô Diễn giải (đã có Ghi chú), Địa chỉ lên chỗ Diễn giải, Ghi chú kéo dài qua hai cột; thu, chi ngân hàng ghi Quỹ tiền; chuyển quỹ Từ quỹ, Đến quỹ một hàng</t>
         </is>
       </c>
       <c r="D122" s="12" t="inlineStr">
@@ -25779,7 +25779,7 @@
       </c>
       <c r="G122" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
+          <t>`2026-10-09-phuongxt-dau-phieu-thu-chi-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr"/>
@@ -25790,12 +25790,12 @@
       </c>
       <c r="B123" s="26" t="inlineStr">
         <is>
-          <t>T68</t>
+          <t>T69</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
+          <t>Ô Ghi chú ở mọi phiếu (phiếu khác thu chi: để trống, độc lập với diễn giải); lưu phiếu giữ đủ các ô đầu phiếu (người giao, địa chỉ, MST, hoá đơn, thanh toán) (QD33)</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -25826,17 +25826,17 @@
       </c>
       <c r="B124" s="25" t="inlineStr">
         <is>
-          <t>T74</t>
+          <t>T68</t>
         </is>
       </c>
       <c r="C124" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
+          <t>Form Mua hàng: thông tin hoá đơn ở cột phải đầu phiếu (2 cột, dưới số phiếu); Số lô, Hạn dùng chỉ có ở gói Pro (QD33)</t>
         </is>
       </c>
       <c r="D124" s="12" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E124" s="28" t="inlineStr">
@@ -25851,7 +25851,7 @@
       </c>
       <c r="G124" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
+          <t>`2026-10-09-phuongxt-hoa-don-cot-phai-ghi-chu.md`</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr"/>
@@ -25862,12 +25862,12 @@
       </c>
       <c r="B125" s="26" t="inlineStr">
         <is>
-          <t>T72</t>
+          <t>T74</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
+          <t>Bảng danh sách theo iPOS Inventory: cột cố định đo bề rộng thật, đứng yên khi cuộn ngang, mỗi ô tự vẽ đường kẻ; kiểu tiêu đề, hàng lọc, dòng, dòng tổng như ivtstag; bấm mã phiếu mở chứng từ (bỏ đúp chuột); cột thời gian dd/MM/yyyy HH:mm</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -25898,12 +25898,12 @@
       </c>
       <c r="B126" s="25" t="inlineStr">
         <is>
-          <t>T71</t>
+          <t>T72</t>
         </is>
       </c>
       <c r="C126" s="13" t="inlineStr">
         <is>
-          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
+          <t>Màn xem báo cáo: nút Xem báo cáo (đổi kỳ, bộ lọc chỉ áp khi bấm); chia độ rộng cột, cỡ chữ theo A4 dọc, ngang cho tờ, bản in, file Excel</t>
         </is>
       </c>
       <c r="D126" s="12" t="inlineStr">
@@ -25934,12 +25934,12 @@
       </c>
       <c r="B127" s="26" t="inlineStr">
         <is>
-          <t>T75</t>
+          <t>T71</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
+          <t>Tờ báo cáo theo kiểu Ledger Studio: đầu tờ, tiêu đề chữ hoa đậm, dòng kỳ màu nhấn, bảng tiêu đề nền nhạt, dòng cộng nền, ô ký và số trang</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -25970,12 +25970,12 @@
       </c>
       <c r="B128" s="25" t="inlineStr">
         <is>
-          <t>T59</t>
+          <t>T75</t>
         </is>
       </c>
       <c r="C128" s="13" t="inlineStr">
         <is>
-          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
+          <t>Màn xem báo cáo: nút Tờ in / Bảng dữ liệu và Khổ lên thanh công cụ cạnh Tuỳ chỉnh; bộ lọc tự sinh chỉ cho cột lấy từ danh mục; tờ giấy có bóng đẹp ở Tờ in, hộp in, Thiết kế mẫu in (QD40)</t>
         </is>
       </c>
       <c r="D128" s="12" t="inlineStr">
@@ -26006,12 +26006,12 @@
       </c>
       <c r="B129" s="26" t="inlineStr">
         <is>
-          <t>T66</t>
+          <t>T59</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
+          <t>Màn Thiết kế mẫu in 11.11: thanh tab bên phải một hàng, ô tìm mẫu bên trái, xem trước vừa khung</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -26042,12 +26042,12 @@
       </c>
       <c r="B130" s="25" t="inlineStr">
         <is>
-          <t>T67</t>
+          <t>T66</t>
         </is>
       </c>
       <c r="C130" s="13" t="inlineStr">
         <is>
-          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
+          <t>Màn xem báo cáo: cột lọc bên trái luôn hiện, thu gọn được; mọi báo cáo tự có bộ lọc theo cột (chữ chọn nhiều, số từ đến), giữ Tờ in và Bảng dữ liệu</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -26078,12 +26078,12 @@
       </c>
       <c r="B131" s="26" t="inlineStr">
         <is>
-          <t>T58</t>
+          <t>T67</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
+          <t>Bảng danh sách: hàng tiêu đề và hàng lọc dính cứng một khối khi cuộn (thead dính), hết nhảy 1px và lộ chữ ở trang thu zoom</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -26114,17 +26114,17 @@
       </c>
       <c r="B132" s="25" t="inlineStr">
         <is>
-          <t>T65</t>
+          <t>T58</t>
         </is>
       </c>
       <c r="C132" s="13" t="inlineStr">
         <is>
-          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
+          <t>Màn Tất cả báo cáo dạng danh sách gọn theo nhóm: một dòng mỗi báo cáo, hai cột, biểu tượng theo loại, Ghim và Mở gần đây; ẩn thanh tab chỉ có một tab</t>
         </is>
       </c>
       <c r="D132" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E132" s="28" t="inlineStr">
@@ -26139,7 +26139,7 @@
       </c>
       <c r="G132" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
+          <t>`2026-10-09-trum-bao-cao-dot-2.md`</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr"/>
@@ -26150,12 +26150,12 @@
       </c>
       <c r="B133" s="26" t="inlineStr">
         <is>
-          <t>T64</t>
+          <t>T65</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
+          <t>Form chứng từ mọi phân hệ: ô lấy từ danh mục (đối tượng, nhân viên, lý do, quỹ, tài khoản ngân hàng, hàng hoá, kho, khoản mục, công việc) xổ danh sách có ô tìm, chưa có thì thêm mới ngay tại form (QD39)</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -26186,12 +26186,12 @@
       </c>
       <c r="B134" s="25" t="inlineStr">
         <is>
-          <t>T63</t>
+          <t>T64</t>
         </is>
       </c>
       <c r="C134" s="13" t="inlineStr">
         <is>
-          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
+          <t>Mua hàng: nguồn chứng từ chỉ Thủ công hoặc Excel, bỏ Tải từ iPOS Inventory ở nút Thêm mới và ô trên sơ đồ (QD39)</t>
         </is>
       </c>
       <c r="D134" s="12" t="inlineStr">
@@ -26222,12 +26222,12 @@
       </c>
       <c r="B135" s="26" t="inlineStr">
         <is>
-          <t>T62</t>
+          <t>T63</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
+          <t>Mua hàng: báo cáo Tổng hợp mua hàng, Chi tiết mua hàng (dùng lại 4.2.2, 4.2.1), thêm Tổng hợp nhập 4.2.4, Chi tiết nhập 4.2.5, mở cho mọi gói, theo chi nhánh; sơ đồ Mua hàng kiểu hội tụ; Sổ ngân hàng gói Free ghi Thu, Chi, Tồn (QD38)</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -26258,12 +26258,12 @@
       </c>
       <c r="B136" s="25" t="inlineStr">
         <is>
-          <t>T61</t>
+          <t>T62</t>
         </is>
       </c>
       <c r="C136" s="13" t="inlineStr">
         <is>
-          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
+          <t>Form Mua hàng: tích Nhận kèm hoá đơn thì thông tin hoá đơn ở đầu phiếu, bỏ tab Hoá đơn; gói Free bỏ tab Ghi sổ ở mọi phiếu; lịch sử thêm mới, sửa, xoá cho mọi phiếu (QD33)</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
@@ -26294,17 +26294,17 @@
       </c>
       <c r="B137" s="26" t="inlineStr">
         <is>
-          <t>T57</t>
+          <t>T61</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
+          <t>Đầu form mọi phiếu như Thu chi: tiêu đề chỉ tên phiếu, trạng thái Thêm mới / Đang chỉnh sửa / Chi tiết phiếu ở giữa, bỏ chip Chưa lưu, Số, tên màn, ô Loại phiếu, Tổng tiền góc phải (QD33)</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E137" s="28" t="inlineStr">
@@ -26319,7 +26319,7 @@
       </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-mua-hang-form-danh-muc.md`</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
@@ -26330,12 +26330,12 @@
       </c>
       <c r="B138" s="25" t="inlineStr">
         <is>
-          <t>T56</t>
+          <t>T57</t>
         </is>
       </c>
       <c r="C138" s="13" t="inlineStr">
         <is>
-          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
+          <t>Màn xem báo cáo: bỏ tiêu đề lặp, khung kéo tới đáy, nút Tuỳ chỉnh, Xuất, In có chữ, chế độ Tờ in hoặc Bảng dữ liệu, bỏ "0 dòng" sai (QD37)</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
@@ -26355,7 +26355,7 @@
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
+          <t>`2026-10-09-trum-man-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr"/>
@@ -26366,17 +26366,17 @@
       </c>
       <c r="B139" s="26" t="inlineStr">
         <is>
-          <t>T25</t>
+          <t>T56</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
+          <t>Hộp in chứng từ 2 cột (chọn mẫu trái, xem trước phải); dính tiêu đề, hàng lọc bảng danh sách chứng từ khi cuộn; nút In Tờ khai GTGT chạy được. Bỏ phần thanh trên báo cáo của bản Anti vì trùng T55</t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E139" s="28" t="inlineStr">
@@ -26391,7 +26391,7 @@
       </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-trum-hop-in-hai-cot.md`</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
@@ -26402,12 +26402,12 @@
       </c>
       <c r="B140" s="25" t="inlineStr">
         <is>
-          <t>T55</t>
+          <t>T25</t>
         </is>
       </c>
       <c r="C140" s="13" t="inlineStr">
         <is>
-          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
+          <t>Thu chi gói Free theo sheet Roadmap: form phiếu thu, chi, chuyển quỹ; danh sách 2.1.1; sơ đồ Quy trình; sổ quỹ, sổ ngân hàng, sổ công nợ theo chi nhánh; sổ gói Free không dùng tài khoản. Điểm mô tả gói tách thành T60</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
@@ -26427,7 +26427,7 @@
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr"/>
@@ -26438,12 +26438,12 @@
       </c>
       <c r="B141" s="26" t="inlineStr">
         <is>
-          <t>T54</t>
+          <t>T55</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
+          <t>Màn xem báo cáo gọn: ô chọn báo cáo kiêm tiêu đề, thanh công cụ cùng hàng, ẩn thanh tab khi xem một báo cáo, bỏ khoảng trống đáy; xem một tờ liền, bỏ ngắt trang, Liên tục/Từng trang, nút In dưới; in vẫn chia trang (QD36)</t>
         </is>
       </c>
       <c r="D141" s="16" t="inlineStr">
@@ -26474,12 +26474,12 @@
       </c>
       <c r="B142" s="25" t="inlineStr">
         <is>
-          <t>T53</t>
+          <t>T54</t>
         </is>
       </c>
       <c r="C142" s="13" t="inlineStr">
         <is>
-          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
+          <t>Thu chi: gói Free ẩn Sổ chi tiết tiền, Sổ công nợ; Sổ quỹ, Sổ ngân hàng lọc Quỹ tiền (số tồn tính lại); Sổ công nợ lọc Đối tượng; Sổ ngân hàng cột Quỹ tiền, xem tất cả quỹ mặc định khổ ngang (QD36)</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
@@ -26510,12 +26510,12 @@
       </c>
       <c r="B143" s="26" t="inlineStr">
         <is>
-          <t>T52</t>
+          <t>T53</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
+          <t>Thanh bên trái: đường kẻ giữa Danh mục và Hệ thống (QD35)</t>
         </is>
       </c>
       <c r="D143" s="16" t="inlineStr">
@@ -26535,7 +26535,7 @@
       </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
+          <t>`2026-10-09-phuongxt-so-thu-chi-bao-cao-gon.md`</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr"/>
@@ -26546,12 +26546,12 @@
       </c>
       <c r="B144" s="25" t="inlineStr">
         <is>
-          <t>T51</t>
+          <t>T52</t>
         </is>
       </c>
       <c r="C144" s="13" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
+          <t>Gói Free gọn theo hộ kinh doanh: Bán hàng chỉ Xuất bán POS, Kho chỉ Kiểm kê và Xuất nhập tồn, mở Mua hàng và Sổ công nợ NCC, ẩn Tổng hợp, bỏ Đính kèm. Đổi tên Thu chi, Kê khai thuế, Chi phí phân bổ; sắp lại thanh bên trái; tab Bán hàng lập tay từ Plus (QD35)</t>
         </is>
       </c>
       <c r="D144" s="12" t="inlineStr">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="G144" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
+          <t>`2026-10-09-phuongxt-goi-free-phan-he.md`</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr"/>
@@ -26582,17 +26582,17 @@
       </c>
       <c r="B145" s="26" t="inlineStr">
         <is>
-          <t>T50</t>
+          <t>T51</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
+          <t>Form phiếu thu chi: ô Quỹ (tiền mặt theo chi nhánh, ngân hàng), Ghi chú cạnh Địa chỉ, lưu xong ở lại xem phiếu; nhật ký thêm mới, sửa, xoá; tab Lịch sử có từ gói Free (QD33)</t>
         </is>
       </c>
       <c r="D145" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E145" s="28" t="inlineStr">
@@ -26607,7 +26607,7 @@
       </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
+          <t>`2026-10-09-phuongxt-quy-nhat-ky-phieu.md`</t>
         </is>
       </c>
       <c r="H145" s="5" t="inlineStr"/>
@@ -26618,12 +26618,12 @@
       </c>
       <c r="B146" s="25" t="inlineStr">
         <is>
-          <t>T47</t>
+          <t>T50</t>
         </is>
       </c>
       <c r="C146" s="13" t="inlineStr">
         <is>
-          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
+          <t>Tối ưu bộ khung 1 trang nhìn và bigdata cho Danh sách chứng từ và Báo cáo theo LedgerStudio (QD34)</t>
         </is>
       </c>
       <c r="D146" s="12" t="inlineStr">
@@ -26643,7 +26643,7 @@
       </c>
       <c r="G146" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
+          <t>`2026-10-09-trum-toi-uu-khung-bang-ledgerstudio.md`</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr"/>
@@ -26654,17 +26654,17 @@
       </c>
       <c r="B147" s="26" t="inlineStr">
         <is>
-          <t>T49</t>
+          <t>T47</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
+          <t>Phân hệ Báo cáo, màn xem như bản in A4, mẫu theo thông tư, chế độ kế toán tách khỏi gói, mẫu in chứng từ, tiện ích Thiết kế mẫu in, xuất 5 định dạng, bộ lọc và tuỳ chỉnh báo cáo, 10 sổ bổ sung (QD31)</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E147" s="28" t="inlineStr">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
+          <t>`2026-10-09-trum-phan-he-bao-cao.md`</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
@@ -26690,12 +26690,12 @@
       </c>
       <c r="B148" s="25" t="inlineStr">
         <is>
-          <t>T48</t>
+          <t>T49</t>
         </is>
       </c>
       <c r="C148" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
+          <t>Form phiếu thu chi (5 loại): đầu form gọn, trạng thái ở giữa; Đối tượng từ danh mục; Lý do trên Diễn giải, Ghi chú; Người giao dịch; Ngày chứng từ có lịch; gói Free có Tháng hạch toán lãi lỗ; cột Lý do ở dòng; Tổng tiền ở dải đáy; bỏ tab Hạch toán. Mọi phiếu: Sao chép, Tuỳ chỉnh giao diện phiếu, phiếu lưu và sửa hiện ở danh sách (QD33)</t>
         </is>
       </c>
       <c r="D148" s="12" t="inlineStr">
@@ -26715,7 +26715,7 @@
       </c>
       <c r="G148" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
+          <t>`2026-10-09-phuongxt-form-phieu-thu-chi.md`</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr"/>
@@ -26726,17 +26726,17 @@
       </c>
       <c r="B149" s="26" t="inlineStr">
         <is>
-          <t>T46</t>
+          <t>T48</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
+          <t>Danh sách chứng từ mọi phân hệ: gói Free bỏ chip trạng thái; Tổng trang, Tổng cộng mọi trang trên hàng phân trang thẳng cột; Tổng tiền là cột cuối, bỏ cột Chức năng; khung chi tiết mặc định đóng; xoá hỏi lại, kỳ đã khoá sổ không xoá (QD32)</t>
         </is>
       </c>
       <c r="D149" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E149" s="28" t="inlineStr">
@@ -26751,7 +26751,7 @@
       </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
+          <t>`2026-10-09-phuongxt-so-chi-nhanh-danh-sach.md`</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
@@ -26762,12 +26762,12 @@
       </c>
       <c r="B150" s="25" t="inlineStr">
         <is>
-          <t>T43</t>
+          <t>T46</t>
         </is>
       </c>
       <c r="C150" s="13" t="inlineStr">
         <is>
-          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
+          <t>Cải tiến chân quy trình (lưới 3 khối), nút cột tài khoản sáng rõ, chiều cao dòng bảng 36px, mở date picker trực tiếp ô lọc ngày, tuỳ chọn hiển thị &amp; đóng băng cột theo mẫu mới (QD30)</t>
         </is>
       </c>
       <c r="D150" s="12" t="inlineStr">
@@ -26787,7 +26787,7 @@
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
+          <t>`2026-10-09-trum-redesign-quy-trinh-tk-dong-bang.md`</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr"/>
@@ -26798,12 +26798,12 @@
       </c>
       <c r="B151" s="26" t="inlineStr">
         <is>
-          <t>T45</t>
+          <t>T43</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
+          <t>Đợt chỉnh 13 điểm: thanh công cụ một hàng, nút Excel và Hàng loạt dạng biểu tượng, chip đếm mới, dòng tổng, bỏ cột Trạng thái và dòng tiêu đề, màu sidebar và cam logo, bỏ giới hạn rộng, gói Free/Standard/Plus/Pro (mã F/S/PL/PR), 80 phiếu mua hàng, dòng tổng bảng chi tiết (QD27)</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
+          <t>`2026-10-09-trum-dot-chinh-13-diem.md`</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
@@ -26834,12 +26834,12 @@
       </c>
       <c r="B152" s="25" t="inlineStr">
         <is>
-          <t>T44</t>
+          <t>T45</t>
         </is>
       </c>
       <c r="C152" s="13" t="inlineStr">
         <is>
-          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
+          <t>Bảng flyout tooltip khi rê chuột vào phân hệ ở sidebar: hiện 2 cột Nghiệp vụ và Tiện ích để truy cập nhanh (QD29)</t>
         </is>
       </c>
       <c r="D152" s="12" t="inlineStr">
@@ -26859,7 +26859,7 @@
       </c>
       <c r="G152" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
+          <t>`2026-10-09-trum-sidebar-flyout.md`</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr"/>
@@ -26870,12 +26870,12 @@
       </c>
       <c r="B153" s="26" t="inlineStr">
         <is>
-          <t>T42</t>
+          <t>T44</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
+          <t>Giao diện gọn 85% cho màn 14 inch, tìm kiếm Ctrl K lên thanh trên cạnh Chi nhánh, bỏ Thêm nhanh, badge Pro giống Inventory, gõ trực tiếp hàng lọc và xoá khe hở tiêu đề (QD28)</t>
         </is>
       </c>
       <c r="D153" s="16" t="inlineStr">
@@ -26890,12 +26890,12 @@
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="G153" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
+          <t>`2026-10-09-trum-giao-dien-14inch-loc-cot.md`</t>
         </is>
       </c>
       <c r="H153" s="5" t="inlineStr"/>
@@ -26906,12 +26906,12 @@
       </c>
       <c r="B154" s="25" t="inlineStr">
         <is>
-          <t>T41</t>
+          <t>T42</t>
         </is>
       </c>
       <c r="C154" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
+          <t>Giao diện gọn cho màn nhỏ (thu nhỏ dưới 1700px), bỏ đường dẫn trên tiêu đề, nút Thêm mới kèm menu gom công cụ, chip trạng thái mới, dòng tổng dính đáy, phân trang mới, lọc cột theo kiểu cột (QD26)</t>
         </is>
       </c>
       <c r="D154" s="12" t="inlineStr">
@@ -26931,7 +26931,7 @@
       </c>
       <c r="G154" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
+          <t>`2026-10-08-trum-giao-dien-gon.md`</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr"/>
@@ -26942,12 +26942,12 @@
       </c>
       <c r="B155" s="26" t="inlineStr">
         <is>
-          <t>T40</t>
+          <t>T41</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
+          <t>Danh sách chứng từ và màn Bán hàng 3.1.1 theo iFaster: chip trạng thái, ô lọc nhãn trên viền, Bộ lọc nâng cao, nút Lọc, Tuỳ chỉnh cột, kẻ dọc và kéo giãn cột, Thao tác hàng loạt (QD25)</t>
         </is>
       </c>
       <c r="D155" s="16" t="inlineStr">
@@ -26967,7 +26967,7 @@
       </c>
       <c r="G155" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
+          <t>`2026-10-08-trum-danh-sach-ifaster.md`</t>
         </is>
       </c>
       <c r="H155" s="5" t="inlineStr"/>
@@ -26978,17 +26978,17 @@
       </c>
       <c r="B156" s="25" t="inlineStr">
         <is>
-          <t>T39</t>
+          <t>T40</t>
         </is>
       </c>
       <c r="C156" s="13" t="inlineStr">
         <is>
-          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
+          <t>Biểu tượng riêng cho 17 màn danh mục, hiện ở menu Khác, ô tìm Ctrl K, hàng Danh mục dưới sơ đồ và sơ đồ Khởi tạo danh mục (QD23)</t>
         </is>
       </c>
       <c r="D156" s="12" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E156" s="28" t="inlineStr">
@@ -27003,7 +27003,7 @@
       </c>
       <c r="G156" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-danh-muc.md`</t>
         </is>
       </c>
       <c r="H156" s="13" t="inlineStr"/>
@@ -27014,17 +27014,17 @@
       </c>
       <c r="B157" s="26" t="inlineStr">
         <is>
-          <t>T38</t>
+          <t>T39</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
+          <t>Danh sách chứng từ mọi phân hệ: bỏ chia đôi 50/50, kỳ lên đầu trang, nút Excel và Tuỳ chỉnh giao diện, bỏ thanh lọc dưới; STT và lọc từng cột có phễu theo kiểu dữ liệu. Gói đang dùng dưới logo, bỏ dòng mã, giai đoạn, nhãn gói dưới tiêu đề mọi màn (QD24)</t>
         </is>
       </c>
       <c r="D157" s="16" t="inlineStr">
         <is>
-          <t>Trum</t>
+          <t>PhuongXT</t>
         </is>
       </c>
       <c r="E157" s="28" t="inlineStr">
@@ -27039,7 +27039,7 @@
       </c>
       <c r="G157" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
+          <t>`2026-10-08-phuongxt-danh-sach-chung-tu.md`</t>
         </is>
       </c>
       <c r="H157" s="5" t="inlineStr"/>
@@ -27050,12 +27050,12 @@
       </c>
       <c r="B158" s="25" t="inlineStr">
         <is>
-          <t>T37</t>
+          <t>T38</t>
         </is>
       </c>
       <c r="C158" s="13" t="inlineStr">
         <is>
-          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
+          <t>Sơ đồ Quy trình hội tụ (phân hệ Tiền) làm lại giao diện: làn gọn có màu, nút nghiệp vụ nằm ngang, đường nối vẽ bằng một lớp SVG, khối Sổ sách nổi bật</t>
         </is>
       </c>
       <c r="D158" s="12" t="inlineStr">
@@ -27075,7 +27075,7 @@
       </c>
       <c r="G158" s="13" t="inlineStr">
         <is>
-          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
+          <t>`2026-10-08-trum-so-do-hoi-tu.md`</t>
         </is>
       </c>
       <c r="H158" s="13" t="inlineStr"/>
@@ -27086,17 +27086,17 @@
       </c>
       <c r="B159" s="26" t="inlineStr">
         <is>
-          <t>T36</t>
+          <t>T37</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
+          <t>Biểu tượng theo iFaster: phân hệ dùng bộ khối đặc của iFaster, đồ vật dùng Solar bản đặc, thao tác giữ nét mảnh (QD23)</t>
         </is>
       </c>
       <c r="D159" s="16" t="inlineStr">
         <is>
-          <t>PhuongXT</t>
+          <t>Trum</t>
         </is>
       </c>
       <c r="E159" s="28" t="inlineStr">
@@ -27111,7 +27111,7 @@
       </c>
       <c r="G159" s="5" t="inlineStr">
         <is>
-          <t>`2026-10-08-phuongxt-thanh-tren-free.md`</t>
+          <t>`2026-10-08-trum-bieu-tuong-ifaster.md`</t>
         </is>
       </c>
       <c r="H159" s="5" t="inlineStr"/>
@@ -27122,12 +27122,12 @@
       </c>
       <c r="B160" s="25" t="inlineStr">
         <is>
-          <t>T32</t>
+          <t>T36</t>
         </is>
       </c>
       <c r="C160" s="13" t="inlineStr">
         <is>
-          <t>Thanh trên chọn chi nhánh làm việc, bỏ ô kỳ và trạng thái đồng bộ FABi; ô tìm kiếm chuyển sang sidebar; danh mục chi nhánh; chứng từ mới lập theo chi nhánh chọn ngoài (QD17)</t>
+          <t>Thanh trên: đủ tên công ty kèm nhãn Công ty, nhãn Chi nhánh, nút Trải nghiệm gói nổi bật, bỏ chọn vai trò (vai trò theo tài khoản đăng nhập). Gói Free ẩn hẳn tính năng ngoài gói. Quy trình tiền gộp khung Báo cáo vào khối sổ sách (QD22)</t>
         </is>
       </c>
